<commit_message>
Add detailed migration steps with hour estimates to Excel
- New sheet: "Migration Steps Detail" with 30+ individual steps
- Each step includes: Phase, Activity, Owner, Manual Hours, EC/AEMCoder Hours
- Hour breakdown for all 45 blocks by category
- Resources sheet now shows hours by phase per role

Co-Authored-By: Claude (global.anthropic.claude-opus-4-5-20251101-v1:0) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/New-ATT-BUSINESS-MIGRATION-PLAN.xlsx
+++ b/New-ATT-BUSINESS-MIGRATION-PLAN.xlsx
@@ -4,10 +4,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Executive Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Templates" sheetId="2" r:id="rId2"/>
-    <sheet name="Migration Phases" sheetId="3" r:id="rId3"/>
-    <sheet name="Block Requirements" sheetId="4" r:id="rId4"/>
-    <sheet name="Block Dev Comparison" sheetId="5" r:id="rId5"/>
+    <sheet name="Migration Steps Detail" sheetId="2" r:id="rId2"/>
+    <sheet name="Templates" sheetId="3" r:id="rId3"/>
+    <sheet name="Phase Summary" sheetId="4" r:id="rId4"/>
+    <sheet name="Block Requirements" sheetId="5" r:id="rId5"/>
     <sheet name="Resources" sheetId="6" r:id="rId6"/>
     <sheet name="Cost Summary" sheetId="7" r:id="rId7"/>
     <sheet name="Risk Assessment" sheetId="8" r:id="rId8"/>
@@ -758,6 +758,1968 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G86"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="45.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>AT&amp;T Business Migration - Detailed Steps &amp; Hour Estimates</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Step #</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Phase</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Activity</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="F3" t="str">
+        <v>EC/AEMCoder Hrs</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Deliverables</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>PHASE 0: PRE-MIGRATION (Weeks 1-2)</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>0a</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Pre-Migration</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Site audit &amp; inventory</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Content Strategist</v>
+      </c>
+      <c r="E6">
+        <v>40</v>
+      </c>
+      <c r="F6">
+        <v>40</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Complete page inventory, asset list</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>0b</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Pre-Migration</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Performance baseline</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Tech Lead</v>
+      </c>
+      <c r="E7">
+        <v>24</v>
+      </c>
+      <c r="F7">
+        <v>24</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Current Core Web Vitals report</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>0c</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Pre-Migration</v>
+      </c>
+      <c r="C8" t="str">
+        <v>SEO audit</v>
+      </c>
+      <c r="D8" t="str">
+        <v>SEO Specialist</v>
+      </c>
+      <c r="E8">
+        <v>32</v>
+      </c>
+      <c r="F8">
+        <v>32</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Rankings, meta data, structured data</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>0d</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Pre-Migration</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Stakeholder alignment &amp; kickoff</v>
+      </c>
+      <c r="D9" t="str">
+        <v>PM</v>
+      </c>
+      <c r="E9">
+        <v>24</v>
+      </c>
+      <c r="F9">
+        <v>24</v>
+      </c>
+      <c r="G9" t="str">
+        <v>RACI matrix, kickoff deck, timeline</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>0e</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Pre-Migration</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Technical discovery</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Tech Lead</v>
+      </c>
+      <c r="E10">
+        <v>40</v>
+      </c>
+      <c r="F10">
+        <v>40</v>
+      </c>
+      <c r="G10" t="str">
+        <v>API inventory, integration mapping</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v>Phase 0 Subtotal</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11">
+        <v>160</v>
+      </c>
+      <c r="F11">
+        <v>160</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>PHASE 1: FOUNDATION (Weeks 3-6)</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>1</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Foundation</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Run EC/AEMcoder for initial migration</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E14">
+        <v>80</v>
+      </c>
+      <c r="F14">
+        <v>40</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Initial blocks, markdown, page structure</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Foundation</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Update blocks, functionality, CSS</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E15">
+        <v>160</v>
+      </c>
+      <c r="F15">
+        <v>80</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Production-ready block code</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2a</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Foundation</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Extract design system tokens</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E16">
+        <v>80</v>
+      </c>
+      <c r="F16">
+        <v>60</v>
+      </c>
+      <c r="G16" t="str">
+        <v>styles.css, CSS custom properties</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2b</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Foundation</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Typography &amp; font setup</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E17">
+        <v>24</v>
+      </c>
+      <c r="F17">
+        <v>24</v>
+      </c>
+      <c r="G17" t="str">
+        <v>fonts.css, AT&amp;T brand fonts</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2c</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Foundation</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Core navigation blocks</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E18">
+        <v>80</v>
+      </c>
+      <c r="F18">
+        <v>80</v>
+      </c>
+      <c r="G18" t="str">
+        <v>header/, footer/, mega-menu</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v>Phase 1 Subtotal</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19">
+        <v>424</v>
+      </c>
+      <c r="F19">
+        <v>284</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>PHASE 2: CONTENT MODELING (Weeks 7-8)</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>3</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Content Modeling</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Create component-model.json</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Tech Lead</v>
+      </c>
+      <c r="E22">
+        <v>60</v>
+      </c>
+      <c r="F22">
+        <v>54</v>
+      </c>
+      <c r="G22" t="str">
+        <v>JCR package structure for AEM importer</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>3a</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Content Modeling</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Create component-definitions.json</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Tech Lead</v>
+      </c>
+      <c r="E23">
+        <v>60</v>
+      </c>
+      <c r="F23">
+        <v>54</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Universal Editor field definitions</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>3b</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Content Modeling</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Define content fragment models</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Content Strategist</v>
+      </c>
+      <c r="E24">
+        <v>40</v>
+      </c>
+      <c r="F24">
+        <v>36</v>
+      </c>
+      <c r="G24" t="str">
+        <v>CF models for products, stories</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>3c</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Content Modeling</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Update transformations</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E25">
+        <v>40</v>
+      </c>
+      <c r="F25">
+        <v>36</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Import script transformations</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v/>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v>Phase 2 Subtotal</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26">
+        <v>200</v>
+      </c>
+      <c r="F26">
+        <v>180</v>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v/>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>PHASE 3: BLOCK DEVELOPMENT (Weeks 9-14)</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>4a</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Block Development</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Hero blocks (6 variants)</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E29">
+        <v>120</v>
+      </c>
+      <c r="F29">
+        <v>72</v>
+      </c>
+      <c r="G29" t="str">
+        <v>hero-video, hero-carousel, hero-split, etc.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>4b</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Block Development</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Card blocks (10 variants)</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E30">
+        <v>200</v>
+      </c>
+      <c r="F30">
+        <v>100</v>
+      </c>
+      <c r="G30" t="str">
+        <v>cards-product, cards-feature, cards-pricing, etc.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>4c</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Block Development</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Interactive blocks</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E31">
+        <v>280</v>
+      </c>
+      <c r="F31">
+        <v>168</v>
+      </c>
+      <c r="G31" t="str">
+        <v>tabs, accordion, carousel, modal, search</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>4d</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Block Development</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Form blocks</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E32">
+        <v>120</v>
+      </c>
+      <c r="F32">
+        <v>72</v>
+      </c>
+      <c r="G32" t="str">
+        <v>lead-form, contact-form, newsletter</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>4e</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Block Development</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Content blocks</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E33">
+        <v>160</v>
+      </c>
+      <c r="F33">
+        <v>80</v>
+      </c>
+      <c r="G33" t="str">
+        <v>columns, quote, table, embed, download</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>4f</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Block Development</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Product-specific blocks</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E34">
+        <v>200</v>
+      </c>
+      <c r="F34">
+        <v>108</v>
+      </c>
+      <c r="G34" t="str">
+        <v>pricing-table, comparison, spec-sheet</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v>Phase 3 Subtotal</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35">
+        <v>1080</v>
+      </c>
+      <c r="F35">
+        <v>600</v>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v/>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>PHASE 4: PAGE REVIEW &amp; ASSET MIGRATION (Weeks 15-16)</v>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>4</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Assets</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Review each page, re-author assets</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Content Team</v>
+      </c>
+      <c r="E38">
+        <v>200</v>
+      </c>
+      <c r="F38">
+        <v>200</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Validated content in AEM DAM</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>4a</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Assets</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Create URL redirect mapping</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Content Strategist</v>
+      </c>
+      <c r="E39">
+        <v>40</v>
+      </c>
+      <c r="F39">
+        <v>40</v>
+      </c>
+      <c r="G39" t="str">
+        <v>301 redirect spreadsheet</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>4b</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Assets</v>
+      </c>
+      <c r="C40" t="str">
+        <v>DAM asset migration</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Content Team</v>
+      </c>
+      <c r="E40">
+        <v>80</v>
+      </c>
+      <c r="F40">
+        <v>80</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Assets with metadata in AEM</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>4c</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Assets</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Image optimization</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E41">
+        <v>40</v>
+      </c>
+      <c r="F41">
+        <v>40</v>
+      </c>
+      <c r="G41" t="str">
+        <v>WebP conversion, lazy loading</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v/>
+      </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
+      <c r="C42" t="str">
+        <v>Phase 4 Subtotal</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42">
+        <v>360</v>
+      </c>
+      <c r="F42">
+        <v>360</v>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v/>
+      </c>
+      <c r="B43" t="str">
+        <v/>
+      </c>
+      <c r="C43" t="str">
+        <v/>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>PHASE 5: EDGE WORKERS &amp; APIs (Weeks 17-18)</v>
+      </c>
+      <c r="B44" t="str">
+        <v/>
+      </c>
+      <c r="C44" t="str">
+        <v/>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>5</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Edge Workers</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Move servlets/APIs to Edge workers</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E45">
+        <v>160</v>
+      </c>
+      <c r="F45">
+        <v>160</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Edge worker functions</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>5a</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Edge Workers</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Pricing API integration</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E46">
+        <v>60</v>
+      </c>
+      <c r="F46">
+        <v>60</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Dynamic pricing endpoints</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>5b</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Edge Workers</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Lead form submission handling</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E47">
+        <v>40</v>
+      </c>
+      <c r="F47">
+        <v>40</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Form backend integration</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>5c</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Edge Workers</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Search functionality</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E48">
+        <v>80</v>
+      </c>
+      <c r="F48">
+        <v>80</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Site search implementation</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v/>
+      </c>
+      <c r="B49" t="str">
+        <v/>
+      </c>
+      <c r="C49" t="str">
+        <v>Phase 5 Subtotal</v>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+      <c r="E49">
+        <v>340</v>
+      </c>
+      <c r="F49">
+        <v>340</v>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v/>
+      </c>
+      <c r="B50" t="str">
+        <v/>
+      </c>
+      <c r="C50" t="str">
+        <v/>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>PHASE 6: AEM MIGRATION (Weeks 19-20)</v>
+      </c>
+      <c r="B51" t="str">
+        <v/>
+      </c>
+      <c r="C51" t="str">
+        <v/>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>6</v>
+      </c>
+      <c r="B52" t="str">
+        <v>AEM Migration</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Migrate custom functionality to AEMaaCS</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E52">
+        <v>120</v>
+      </c>
+      <c r="F52">
+        <v>120</v>
+      </c>
+      <c r="G52" t="str">
+        <v>Reports, scheduled jobs</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>7</v>
+      </c>
+      <c r="B53" t="str">
+        <v>AEM Migration</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Migrate meta-schema, taxonomy, workflows</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Tech Lead</v>
+      </c>
+      <c r="E53">
+        <v>80</v>
+      </c>
+      <c r="F53">
+        <v>80</v>
+      </c>
+      <c r="G53" t="str">
+        <v>AEM configurations</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>7a</v>
+      </c>
+      <c r="B54" t="str">
+        <v>AEM Migration</v>
+      </c>
+      <c r="C54" t="str">
+        <v>User/group migration</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="E54">
+        <v>40</v>
+      </c>
+      <c r="F54">
+        <v>40</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Permissions in AEMaaCS</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>7b</v>
+      </c>
+      <c r="B55" t="str">
+        <v>AEM Migration</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Workflow configuration</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Tech Lead</v>
+      </c>
+      <c r="E55">
+        <v>40</v>
+      </c>
+      <c r="F55">
+        <v>40</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Approval workflows</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v/>
+      </c>
+      <c r="B56" t="str">
+        <v/>
+      </c>
+      <c r="C56" t="str">
+        <v>Phase 6 Subtotal</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56">
+        <v>280</v>
+      </c>
+      <c r="F56">
+        <v>280</v>
+      </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v/>
+      </c>
+      <c r="B57" t="str">
+        <v/>
+      </c>
+      <c r="C57" t="str">
+        <v/>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>PHASE 7: INTEGRATIONS (Weeks 21-22)</v>
+      </c>
+      <c r="B58" t="str">
+        <v/>
+      </c>
+      <c r="C58" t="str">
+        <v/>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>8a</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Integrations</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Analytics/tracking setup</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E59">
+        <v>60</v>
+      </c>
+      <c r="F59">
+        <v>60</v>
+      </c>
+      <c r="G59" t="str">
+        <v>Adobe Launch configuration</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>8b</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Integrations</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Third-party scripts</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E60">
+        <v>40</v>
+      </c>
+      <c r="F60">
+        <v>40</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Chat, pixels, consent banner</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>8c</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Integrations</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Search indexing configuration</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E61">
+        <v>40</v>
+      </c>
+      <c r="F61">
+        <v>40</v>
+      </c>
+      <c r="G61" t="str">
+        <v>Sitemap, robots.txt</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>8d</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Integrations</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Social meta tags</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Dev Team</v>
+      </c>
+      <c r="E62">
+        <v>20</v>
+      </c>
+      <c r="F62">
+        <v>20</v>
+      </c>
+      <c r="G62" t="str">
+        <v>OG tags, Twitter cards</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v/>
+      </c>
+      <c r="B63" t="str">
+        <v/>
+      </c>
+      <c r="C63" t="str">
+        <v>Phase 7 Subtotal</v>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+      <c r="E63">
+        <v>160</v>
+      </c>
+      <c r="F63">
+        <v>160</v>
+      </c>
+      <c r="G63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v/>
+      </c>
+      <c r="B64" t="str">
+        <v/>
+      </c>
+      <c r="C64" t="str">
+        <v/>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+      <c r="G64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>PHASE 8: VALIDATION &amp; TESTING (Weeks 23-24)</v>
+      </c>
+      <c r="B65" t="str">
+        <v/>
+      </c>
+      <c r="C65" t="str">
+        <v/>
+      </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
+      <c r="F65" t="str">
+        <v/>
+      </c>
+      <c r="G65" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>8</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Validation</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Validate all functionalities</v>
+      </c>
+      <c r="D66" t="str">
+        <v>QA Team</v>
+      </c>
+      <c r="E66">
+        <v>160</v>
+      </c>
+      <c r="F66">
+        <v>150</v>
+      </c>
+      <c r="G66" t="str">
+        <v>Functional test reports</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>9</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Validation</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Accessibility audit (WCAG 2.1 AA)</v>
+      </c>
+      <c r="D67" t="str">
+        <v>QA Team</v>
+      </c>
+      <c r="E67">
+        <v>80</v>
+      </c>
+      <c r="F67">
+        <v>75</v>
+      </c>
+      <c r="G67" t="str">
+        <v>Accessibility report, fixes</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>10</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Validation</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Performance/load testing</v>
+      </c>
+      <c r="D68" t="str">
+        <v>QA Team</v>
+      </c>
+      <c r="E68">
+        <v>60</v>
+      </c>
+      <c r="F68">
+        <v>55</v>
+      </c>
+      <c r="G68" t="str">
+        <v>Performance test results</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>11</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Validation</v>
+      </c>
+      <c r="C69" t="str">
+        <v>SEO validation</v>
+      </c>
+      <c r="D69" t="str">
+        <v>SEO Specialist</v>
+      </c>
+      <c r="E69">
+        <v>40</v>
+      </c>
+      <c r="F69">
+        <v>40</v>
+      </c>
+      <c r="G69" t="str">
+        <v>Redirect testing, sitemap validation</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>12</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Validation</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Security review</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Security Team</v>
+      </c>
+      <c r="E70">
+        <v>40</v>
+      </c>
+      <c r="F70">
+        <v>40</v>
+      </c>
+      <c r="G70" t="str">
+        <v>Security headers, CSP audit</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v/>
+      </c>
+      <c r="B71" t="str">
+        <v/>
+      </c>
+      <c r="C71" t="str">
+        <v>Phase 8 Subtotal</v>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+      <c r="E71">
+        <v>380</v>
+      </c>
+      <c r="F71">
+        <v>360</v>
+      </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v/>
+      </c>
+      <c r="B72" t="str">
+        <v/>
+      </c>
+      <c r="C72" t="str">
+        <v/>
+      </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
+      <c r="F72" t="str">
+        <v/>
+      </c>
+      <c r="G72" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>PHASE 9: LAUNCH (Week 24+)</v>
+      </c>
+      <c r="B73" t="str">
+        <v/>
+      </c>
+      <c r="C73" t="str">
+        <v/>
+      </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+      <c r="G73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>13</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Launch</v>
+      </c>
+      <c r="C74" t="str">
+        <v>UAT &amp; stakeholder sign-off</v>
+      </c>
+      <c r="D74" t="str">
+        <v>PM</v>
+      </c>
+      <c r="E74">
+        <v>80</v>
+      </c>
+      <c r="F74">
+        <v>76</v>
+      </c>
+      <c r="G74" t="str">
+        <v>Sign-off documentation</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>14</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Launch</v>
+      </c>
+      <c r="C75" t="str">
+        <v>DNS cutover &amp; rollback plan</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Tech Lead</v>
+      </c>
+      <c r="E75">
+        <v>40</v>
+      </c>
+      <c r="F75">
+        <v>40</v>
+      </c>
+      <c r="G75" t="str">
+        <v>Production deployment</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>15</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Launch</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Author training on Universal Editor</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Training Lead</v>
+      </c>
+      <c r="E76">
+        <v>60</v>
+      </c>
+      <c r="F76">
+        <v>60</v>
+      </c>
+      <c r="G76" t="str">
+        <v>Training materials, sessions</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>16</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Launch</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Hypercare &amp; monitoring setup</v>
+      </c>
+      <c r="D77" t="str">
+        <v>DevOps</v>
+      </c>
+      <c r="E77">
+        <v>80</v>
+      </c>
+      <c r="F77">
+        <v>80</v>
+      </c>
+      <c r="G77" t="str">
+        <v>Monitoring dashboards, alerts</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v/>
+      </c>
+      <c r="B78" t="str">
+        <v/>
+      </c>
+      <c r="C78" t="str">
+        <v>Phase 9 Subtotal</v>
+      </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
+      <c r="E78">
+        <v>260</v>
+      </c>
+      <c r="F78">
+        <v>256</v>
+      </c>
+      <c r="G78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v/>
+      </c>
+      <c r="B79" t="str">
+        <v/>
+      </c>
+      <c r="C79" t="str">
+        <v/>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
+      <c r="F79" t="str">
+        <v/>
+      </c>
+      <c r="G79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v/>
+      </c>
+      <c r="B80" t="str">
+        <v/>
+      </c>
+      <c r="C80" t="str">
+        <v/>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+      <c r="G80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>SUMMARY</v>
+      </c>
+      <c r="B81" t="str">
+        <v/>
+      </c>
+      <c r="C81" t="str">
+        <v/>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
+      <c r="F81" t="str">
+        <v/>
+      </c>
+      <c r="G81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v/>
+      </c>
+      <c r="B82" t="str">
+        <v/>
+      </c>
+      <c r="C82" t="str">
+        <v>Base Hours Total</v>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+      <c r="E82">
+        <v>3644</v>
+      </c>
+      <c r="F82">
+        <v>2980</v>
+      </c>
+      <c r="G82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v/>
+      </c>
+      <c r="B83" t="str">
+        <v/>
+      </c>
+      <c r="C83" t="str">
+        <v>Contingency (~32% / ~38%)</v>
+      </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
+      <c r="E83">
+        <v>1156</v>
+      </c>
+      <c r="F83">
+        <v>1140</v>
+      </c>
+      <c r="G83" t="str">
+        <v>Risk buffer for unknowns</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v/>
+      </c>
+      <c r="B84" t="str">
+        <v/>
+      </c>
+      <c r="C84" t="str">
+        <v>GRAND TOTAL</v>
+      </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
+      <c r="E84">
+        <v>4800</v>
+      </c>
+      <c r="F84">
+        <v>4120</v>
+      </c>
+      <c r="G84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v/>
+      </c>
+      <c r="B85" t="str">
+        <v/>
+      </c>
+      <c r="C85" t="str">
+        <v>Hours Saved</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+      <c r="F85">
+        <v>680</v>
+      </c>
+      <c r="G85" t="str">
+        <v>~14% reduction</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v/>
+      </c>
+      <c r="B86" t="str">
+        <v/>
+      </c>
+      <c r="C86" t="str">
+        <v>Weeks Saved</v>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
+      <c r="F86" t="str">
+        <v>3-4 weeks</v>
+      </c>
+      <c r="G86" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G86"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D13"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
@@ -937,7 +2899,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
   <cols>
@@ -1206,13 +3168,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:E78"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1238,6 +3202,12 @@
         <v>Complexity</v>
       </c>
       <c r="C4" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D4" t="str">
+        <v>EC Hrs</v>
+      </c>
+      <c r="E4" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1248,7 +3218,13 @@
       <c r="B5" t="str">
         <v>Very High</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C5">
+        <v>30</v>
+      </c>
+      <c r="D5">
+        <v>30</v>
+      </c>
+      <c r="E5" t="str">
         <v>Mega menu, search, account login, Personal/Business toggle</v>
       </c>
     </row>
@@ -1259,7 +3235,13 @@
       <c r="B6" t="str">
         <v>High</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C6">
+        <v>20</v>
+      </c>
+      <c r="D6">
+        <v>20</v>
+      </c>
+      <c r="E6" t="str">
         <v>Multi-column, social links, legal links</v>
       </c>
     </row>
@@ -1270,7 +3252,13 @@
       <c r="B7" t="str">
         <v>Low</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C7">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>10</v>
+      </c>
+      <c r="E7" t="str">
         <v>Standard hierarchy</v>
       </c>
     </row>
@@ -1281,12 +3269,30 @@
       <c r="B8" t="str">
         <v>High</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C8">
+        <v>20</v>
+      </c>
+      <c r="D8">
+        <v>20</v>
+      </c>
+      <c r="E8" t="str">
         <v>Mobile menu with nested items</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
         <v/>
       </c>
     </row>
@@ -1303,6 +3309,12 @@
         <v>Complexity</v>
       </c>
       <c r="C11" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D11" t="str">
+        <v>EC Hrs</v>
+      </c>
+      <c r="E11" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1313,7 +3325,13 @@
       <c r="B12" t="str">
         <v>High</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C12">
+        <v>24</v>
+      </c>
+      <c r="D12">
+        <v>14</v>
+      </c>
+      <c r="E12" t="str">
         <v>Background video with overlay text, CTAs</v>
       </c>
     </row>
@@ -1324,7 +3342,13 @@
       <c r="B13" t="str">
         <v>High</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C13">
+        <v>24</v>
+      </c>
+      <c r="D13">
+        <v>14</v>
+      </c>
+      <c r="E13" t="str">
         <v>Multiple slides with auto-rotation</v>
       </c>
     </row>
@@ -1335,7 +3359,13 @@
       <c r="B14" t="str">
         <v>High</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C14">
+        <v>24</v>
+      </c>
+      <c r="D14">
+        <v>14</v>
+      </c>
+      <c r="E14" t="str">
         <v>Tabbed content (Mobile, Internet, Voice, etc.)</v>
       </c>
     </row>
@@ -1346,7 +3376,13 @@
       <c r="B15" t="str">
         <v>Medium</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C15">
+        <v>16</v>
+      </c>
+      <c r="D15">
+        <v>10</v>
+      </c>
+      <c r="E15" t="str">
         <v>Two-column layout</v>
       </c>
     </row>
@@ -1357,7 +3393,13 @@
       <c r="B16" t="str">
         <v>Low</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C16">
+        <v>16</v>
+      </c>
+      <c r="D16">
+        <v>10</v>
+      </c>
+      <c r="E16" t="str">
         <v>Text-only section header</v>
       </c>
     </row>
@@ -1368,12 +3410,30 @@
       <c r="B17" t="str">
         <v>Medium</v>
       </c>
-      <c r="C17" t="str">
+      <c r="C17">
+        <v>16</v>
+      </c>
+      <c r="D17">
+        <v>10</v>
+      </c>
+      <c r="E17" t="str">
         <v>Promotional banner with pricing</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v/>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
         <v/>
       </c>
     </row>
@@ -1390,6 +3450,12 @@
         <v>Complexity</v>
       </c>
       <c r="C20" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D20" t="str">
+        <v>EC Hrs</v>
+      </c>
+      <c r="E20" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1400,7 +3466,13 @@
       <c r="B21" t="str">
         <v>Medium</v>
       </c>
-      <c r="C21" t="str">
+      <c r="C21">
+        <v>20</v>
+      </c>
+      <c r="D21">
+        <v>10</v>
+      </c>
+      <c r="E21" t="str">
         <v>Product tiles with pricing</v>
       </c>
     </row>
@@ -1411,7 +3483,13 @@
       <c r="B22" t="str">
         <v>Medium</v>
       </c>
-      <c r="C22" t="str">
+      <c r="C22">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>10</v>
+      </c>
+      <c r="E22" t="str">
         <v>Icon/image with text</v>
       </c>
     </row>
@@ -1422,7 +3500,13 @@
       <c r="B23" t="str">
         <v>High</v>
       </c>
-      <c r="C23" t="str">
+      <c r="C23">
+        <v>24</v>
+      </c>
+      <c r="D23">
+        <v>12</v>
+      </c>
+      <c r="E23" t="str">
         <v>Pricing comparison cards</v>
       </c>
     </row>
@@ -1433,7 +3517,13 @@
       <c r="B24" t="str">
         <v>Medium</v>
       </c>
-      <c r="C24" t="str">
+      <c r="C24">
+        <v>20</v>
+      </c>
+      <c r="D24">
+        <v>10</v>
+      </c>
+      <c r="E24" t="str">
         <v>Industry solution cards</v>
       </c>
     </row>
@@ -1444,7 +3534,13 @@
       <c r="B25" t="str">
         <v>Medium</v>
       </c>
-      <c r="C25" t="str">
+      <c r="C25">
+        <v>20</v>
+      </c>
+      <c r="D25">
+        <v>10</v>
+      </c>
+      <c r="E25" t="str">
         <v>Customer story previews</v>
       </c>
     </row>
@@ -1455,7 +3551,13 @@
       <c r="B26" t="str">
         <v>Medium</v>
       </c>
-      <c r="C26" t="str">
+      <c r="C26">
+        <v>20</v>
+      </c>
+      <c r="D26">
+        <v>10</v>
+      </c>
+      <c r="E26" t="str">
         <v>Large numbers with descriptions</v>
       </c>
     </row>
@@ -1466,7 +3568,13 @@
       <c r="B27" t="str">
         <v>Low</v>
       </c>
-      <c r="C27" t="str">
+      <c r="C27">
+        <v>16</v>
+      </c>
+      <c r="D27">
+        <v>8</v>
+      </c>
+      <c r="E27" t="str">
         <v>Simple call-to-action cards</v>
       </c>
     </row>
@@ -1477,7 +3585,13 @@
       <c r="B28" t="str">
         <v>Medium</v>
       </c>
-      <c r="C28" t="str">
+      <c r="C28">
+        <v>20</v>
+      </c>
+      <c r="D28">
+        <v>10</v>
+      </c>
+      <c r="E28" t="str">
         <v>Icon-based feature cards</v>
       </c>
     </row>
@@ -1488,7 +3602,13 @@
       <c r="B29" t="str">
         <v>Medium</v>
       </c>
-      <c r="C29" t="str">
+      <c r="C29">
+        <v>20</v>
+      </c>
+      <c r="D29">
+        <v>10</v>
+      </c>
+      <c r="E29" t="str">
         <v>Customer quotes</v>
       </c>
     </row>
@@ -1499,12 +3619,30 @@
       <c r="B30" t="str">
         <v>Low</v>
       </c>
-      <c r="C30" t="str">
+      <c r="C30">
+        <v>20</v>
+      </c>
+      <c r="D30">
+        <v>10</v>
+      </c>
+      <c r="E30" t="str">
         <v>Quick link lists</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
+        <v/>
+      </c>
+      <c r="B31" t="str">
+        <v/>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
         <v/>
       </c>
     </row>
@@ -1521,6 +3659,12 @@
         <v>Complexity</v>
       </c>
       <c r="C33" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D33" t="str">
+        <v>EC Hrs</v>
+      </c>
+      <c r="E33" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1531,7 +3675,13 @@
       <c r="B34" t="str">
         <v>Medium</v>
       </c>
-      <c r="C34" t="str">
+      <c r="C34">
+        <v>24</v>
+      </c>
+      <c r="D34">
+        <v>14</v>
+      </c>
+      <c r="E34" t="str">
         <v>FAQ, product details</v>
       </c>
     </row>
@@ -1542,7 +3692,13 @@
       <c r="B35" t="str">
         <v>Medium</v>
       </c>
-      <c r="C35" t="str">
+      <c r="C35">
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <v>14</v>
+      </c>
+      <c r="E35" t="str">
         <v>Content organization</v>
       </c>
     </row>
@@ -1553,7 +3709,13 @@
       <c r="B36" t="str">
         <v>High</v>
       </c>
-      <c r="C36" t="str">
+      <c r="C36">
+        <v>32</v>
+      </c>
+      <c r="D36">
+        <v>19</v>
+      </c>
+      <c r="E36" t="str">
         <v>Image/content slider</v>
       </c>
     </row>
@@ -1564,7 +3726,13 @@
       <c r="B37" t="str">
         <v>Medium</v>
       </c>
-      <c r="C37" t="str">
+      <c r="C37">
+        <v>24</v>
+      </c>
+      <c r="D37">
+        <v>14</v>
+      </c>
+      <c r="E37" t="str">
         <v>Popup dialogs, offer details</v>
       </c>
     </row>
@@ -1575,7 +3743,13 @@
       <c r="B38" t="str">
         <v>Medium</v>
       </c>
-      <c r="C38" t="str">
+      <c r="C38">
+        <v>24</v>
+      </c>
+      <c r="D38">
+        <v>14</v>
+      </c>
+      <c r="E38" t="str">
         <v>Inline video player</v>
       </c>
     </row>
@@ -1586,7 +3760,13 @@
       <c r="B39" t="str">
         <v>High</v>
       </c>
-      <c r="C39" t="str">
+      <c r="C39">
+        <v>32</v>
+      </c>
+      <c r="D39">
+        <v>19</v>
+      </c>
+      <c r="E39" t="str">
         <v>Lightbox video player</v>
       </c>
     </row>
@@ -1597,7 +3777,13 @@
       <c r="B40" t="str">
         <v>High</v>
       </c>
-      <c r="C40" t="str">
+      <c r="C40">
+        <v>32</v>
+      </c>
+      <c r="D40">
+        <v>19</v>
+      </c>
+      <c r="E40" t="str">
         <v>Site search with filtering</v>
       </c>
     </row>
@@ -1608,7 +3794,13 @@
       <c r="B41" t="str">
         <v>High</v>
       </c>
-      <c r="C41" t="str">
+      <c r="C41">
+        <v>32</v>
+      </c>
+      <c r="D41">
+        <v>19</v>
+      </c>
+      <c r="E41" t="str">
         <v>Product filtering</v>
       </c>
     </row>
@@ -1619,7 +3811,13 @@
       <c r="B42" t="str">
         <v>Very High</v>
       </c>
-      <c r="C42" t="str">
+      <c r="C42">
+        <v>32</v>
+      </c>
+      <c r="D42">
+        <v>19</v>
+      </c>
+      <c r="E42" t="str">
         <v>Dynamic pricing tool</v>
       </c>
     </row>
@@ -1630,12 +3828,30 @@
       <c r="B43" t="str">
         <v>High</v>
       </c>
-      <c r="C43" t="str">
+      <c r="C43">
+        <v>24</v>
+      </c>
+      <c r="D43">
+        <v>17</v>
+      </c>
+      <c r="E43" t="str">
         <v>Product comparison</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
+        <v/>
+      </c>
+      <c r="B44" t="str">
+        <v/>
+      </c>
+      <c r="C44" t="str">
+        <v/>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
         <v/>
       </c>
     </row>
@@ -1652,6 +3868,12 @@
         <v>Complexity</v>
       </c>
       <c r="C46" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D46" t="str">
+        <v>EC Hrs</v>
+      </c>
+      <c r="E46" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1662,7 +3884,13 @@
       <c r="B47" t="str">
         <v>Low</v>
       </c>
-      <c r="C47" t="str">
+      <c r="C47">
+        <v>16</v>
+      </c>
+      <c r="D47">
+        <v>8</v>
+      </c>
+      <c r="E47" t="str">
         <v>Multi-column layouts</v>
       </c>
     </row>
@@ -1673,7 +3901,13 @@
       <c r="B48" t="str">
         <v>Low</v>
       </c>
-      <c r="C48" t="str">
+      <c r="C48">
+        <v>16</v>
+      </c>
+      <c r="D48">
+        <v>8</v>
+      </c>
+      <c r="E48" t="str">
         <v>Testimonials, pull quotes</v>
       </c>
     </row>
@@ -1684,7 +3918,13 @@
       <c r="B49" t="str">
         <v>Medium</v>
       </c>
-      <c r="C49" t="str">
+      <c r="C49">
+        <v>24</v>
+      </c>
+      <c r="D49">
+        <v>12</v>
+      </c>
+      <c r="E49" t="str">
         <v>Data tables</v>
       </c>
     </row>
@@ -1695,7 +3935,13 @@
       <c r="B50" t="str">
         <v>Medium</v>
       </c>
-      <c r="C50" t="str">
+      <c r="C50">
+        <v>24</v>
+      </c>
+      <c r="D50">
+        <v>12</v>
+      </c>
+      <c r="E50" t="str">
         <v>External content (YouTube, maps)</v>
       </c>
     </row>
@@ -1706,7 +3952,13 @@
       <c r="B51" t="str">
         <v>Low</v>
       </c>
-      <c r="C51" t="str">
+      <c r="C51">
+        <v>16</v>
+      </c>
+      <c r="D51">
+        <v>8</v>
+      </c>
+      <c r="E51" t="str">
         <v>PDF/document links</v>
       </c>
     </row>
@@ -1717,7 +3969,13 @@
       <c r="B52" t="str">
         <v>Medium</v>
       </c>
-      <c r="C52" t="str">
+      <c r="C52">
+        <v>24</v>
+      </c>
+      <c r="D52">
+        <v>12</v>
+      </c>
+      <c r="E52" t="str">
         <v>Full-width call-to-action</v>
       </c>
     </row>
@@ -1728,7 +3986,13 @@
       <c r="B53" t="str">
         <v>Low</v>
       </c>
-      <c r="C53" t="str">
+      <c r="C53">
+        <v>16</v>
+      </c>
+      <c r="D53">
+        <v>8</v>
+      </c>
+      <c r="E53" t="str">
         <v>Section separators</v>
       </c>
     </row>
@@ -1739,12 +4003,30 @@
       <c r="B54" t="str">
         <v>Medium</v>
       </c>
-      <c r="C54" t="str">
+      <c r="C54">
+        <v>24</v>
+      </c>
+      <c r="D54">
+        <v>12</v>
+      </c>
+      <c r="E54" t="str">
         <v>Feature lists with icons</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
+        <v/>
+      </c>
+      <c r="B55" t="str">
+        <v/>
+      </c>
+      <c r="C55" t="str">
+        <v/>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
         <v/>
       </c>
     </row>
@@ -1761,6 +4043,12 @@
         <v>Complexity</v>
       </c>
       <c r="C57" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D57" t="str">
+        <v>EC Hrs</v>
+      </c>
+      <c r="E57" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1771,7 +4059,13 @@
       <c r="B58" t="str">
         <v>High</v>
       </c>
-      <c r="C58" t="str">
+      <c r="C58">
+        <v>36</v>
+      </c>
+      <c r="D58">
+        <v>22</v>
+      </c>
+      <c r="E58" t="str">
         <v>Sales contact form (RAI form)</v>
       </c>
     </row>
@@ -1782,7 +4076,13 @@
       <c r="B59" t="str">
         <v>Medium</v>
       </c>
-      <c r="C59" t="str">
+      <c r="C59">
+        <v>28</v>
+      </c>
+      <c r="D59">
+        <v>17</v>
+      </c>
+      <c r="E59" t="str">
         <v>General inquiry</v>
       </c>
     </row>
@@ -1793,7 +4093,13 @@
       <c r="B60" t="str">
         <v>Medium</v>
       </c>
-      <c r="C60" t="str">
+      <c r="C60">
+        <v>28</v>
+      </c>
+      <c r="D60">
+        <v>17</v>
+      </c>
+      <c r="E60" t="str">
         <v>Email signup</v>
       </c>
     </row>
@@ -1804,12 +4110,30 @@
       <c r="B61" t="str">
         <v>Medium</v>
       </c>
-      <c r="C61" t="str">
+      <c r="C61">
+        <v>28</v>
+      </c>
+      <c r="D61">
+        <v>16</v>
+      </c>
+      <c r="E61" t="str">
         <v>Search box</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
+        <v/>
+      </c>
+      <c r="B62" t="str">
+        <v/>
+      </c>
+      <c r="C62" t="str">
+        <v/>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+      <c r="E62" t="str">
         <v/>
       </c>
     </row>
@@ -1826,6 +4150,12 @@
         <v>Complexity</v>
       </c>
       <c r="C64" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D64" t="str">
+        <v>EC Hrs</v>
+      </c>
+      <c r="E64" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1836,7 +4166,13 @@
       <c r="B65" t="str">
         <v>Medium</v>
       </c>
-      <c r="C65" t="str">
+      <c r="C65">
+        <v>24</v>
+      </c>
+      <c r="D65">
+        <v>13</v>
+      </c>
+      <c r="E65" t="str">
         <v>AT&amp;T Guarantee messaging</v>
       </c>
     </row>
@@ -1847,7 +4183,13 @@
       <c r="B66" t="str">
         <v>High</v>
       </c>
-      <c r="C66" t="str">
+      <c r="C66">
+        <v>32</v>
+      </c>
+      <c r="D66">
+        <v>17</v>
+      </c>
+      <c r="E66" t="str">
         <v>Dynamic promotional offers</v>
       </c>
     </row>
@@ -1858,196 +4200,230 @@
       <c r="B67" t="str">
         <v>Low</v>
       </c>
-      <c r="C67" t="str">
+      <c r="C67">
+        <v>16</v>
+      </c>
+      <c r="D67">
+        <v>8</v>
+      </c>
+      <c r="E67" t="str">
         <v>Award/certification badges</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v/>
+      </c>
+      <c r="B68" t="str">
+        <v/>
+      </c>
+      <c r="C68" t="str">
+        <v/>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>BLOCK TOTALS</v>
+      </c>
+      <c r="B69" t="str">
+        <v/>
+      </c>
+      <c r="C69" t="str">
+        <v/>
+      </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Category</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Count</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D70" t="str">
+        <v>EC Hrs</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Reduction</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Navigation</v>
+      </c>
+      <c r="B71">
+        <v>4</v>
+      </c>
+      <c r="C71">
+        <v>80</v>
+      </c>
+      <c r="D71">
+        <v>80</v>
+      </c>
+      <c r="E71" t="str">
+        <v>0%</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Hero</v>
+      </c>
+      <c r="B72">
+        <v>6</v>
+      </c>
+      <c r="C72">
+        <v>120</v>
+      </c>
+      <c r="D72">
+        <v>72</v>
+      </c>
+      <c r="E72" t="str">
+        <v>40%</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Cards</v>
+      </c>
+      <c r="B73">
+        <v>10</v>
+      </c>
+      <c r="C73">
+        <v>200</v>
+      </c>
+      <c r="D73">
+        <v>100</v>
+      </c>
+      <c r="E73" t="str">
+        <v>50%</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Interactive</v>
+      </c>
+      <c r="B74">
+        <v>10</v>
+      </c>
+      <c r="C74">
+        <v>280</v>
+      </c>
+      <c r="D74">
+        <v>168</v>
+      </c>
+      <c r="E74" t="str">
+        <v>40%</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>Content</v>
+      </c>
+      <c r="B75">
+        <v>8</v>
+      </c>
+      <c r="C75">
+        <v>160</v>
+      </c>
+      <c r="D75">
+        <v>80</v>
+      </c>
+      <c r="E75" t="str">
+        <v>50%</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Forms</v>
+      </c>
+      <c r="B76">
+        <v>4</v>
+      </c>
+      <c r="C76">
+        <v>120</v>
+      </c>
+      <c r="D76">
+        <v>72</v>
+      </c>
+      <c r="E76" t="str">
+        <v>40%</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>AT&amp;T-Specific</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77">
+        <v>72</v>
+      </c>
+      <c r="D77">
+        <v>38</v>
+      </c>
+      <c r="E77" t="str">
+        <v>47%</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B78">
+        <v>45</v>
+      </c>
+      <c r="C78">
+        <v>1032</v>
+      </c>
+      <c r="D78">
+        <v>610</v>
+      </c>
+      <c r="E78" t="str">
+        <v>~41%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C67"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Block Development Comparison - Phase 3</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Block Category</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Block Count</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Manual (hrs)</v>
-      </c>
-      <c r="D3" t="str">
-        <v>EC/AEMCoder (hrs)</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Reduction %</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Hero Blocks</v>
-      </c>
-      <c r="B4" t="str">
-        <v>6</v>
-      </c>
-      <c r="C4" t="str">
-        <v>120</v>
-      </c>
-      <c r="D4" t="str">
-        <v>72</v>
-      </c>
-      <c r="E4" t="str">
-        <v>40%</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Card Blocks</v>
-      </c>
-      <c r="B5" t="str">
-        <v>10</v>
-      </c>
-      <c r="C5" t="str">
-        <v>200</v>
-      </c>
-      <c r="D5" t="str">
-        <v>100</v>
-      </c>
-      <c r="E5" t="str">
-        <v>50%</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Interactive Blocks</v>
-      </c>
-      <c r="B6" t="str">
-        <v>10</v>
-      </c>
-      <c r="C6" t="str">
-        <v>280</v>
-      </c>
-      <c r="D6" t="str">
-        <v>168</v>
-      </c>
-      <c r="E6" t="str">
-        <v>40%</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Form Blocks</v>
-      </c>
-      <c r="B7" t="str">
-        <v>4</v>
-      </c>
-      <c r="C7" t="str">
-        <v>120</v>
-      </c>
-      <c r="D7" t="str">
-        <v>72</v>
-      </c>
-      <c r="E7" t="str">
-        <v>40%</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Content Blocks</v>
-      </c>
-      <c r="B8" t="str">
-        <v>8</v>
-      </c>
-      <c r="C8" t="str">
-        <v>160</v>
-      </c>
-      <c r="D8" t="str">
-        <v>80</v>
-      </c>
-      <c r="E8" t="str">
-        <v>50%</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Product-specific</v>
-      </c>
-      <c r="B9" t="str">
-        <v>6</v>
-      </c>
-      <c r="C9" t="str">
-        <v>200</v>
-      </c>
-      <c r="D9" t="str">
-        <v>108</v>
-      </c>
-      <c r="E9" t="str">
-        <v>46%</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="B10" t="str">
-        <v>45</v>
-      </c>
-      <c r="C10" t="str">
-        <v>1,080</v>
-      </c>
-      <c r="D10" t="str">
-        <v>600</v>
-      </c>
-      <c r="E10" t="str">
-        <v>~44%</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E78"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:K17"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="8.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Team Structure</v>
+        <v>Team Structure &amp; Hours by Phase</v>
       </c>
     </row>
     <row r="2">
@@ -2066,13 +4442,28 @@
         <v>Rate/Hr</v>
       </c>
       <c r="D3" t="str">
-        <v>Hours</v>
+        <v>Ph 0</v>
       </c>
       <c r="E3" t="str">
+        <v>Ph 1</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Ph 2</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Ph 3</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Ph 4-6</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Ph 7-9</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Total Hrs</v>
+      </c>
+      <c r="K3" t="str">
         <v>Total Cost</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Responsibilities</v>
       </c>
     </row>
     <row r="4">
@@ -2085,14 +4476,29 @@
       <c r="C4" t="str">
         <v>$150</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D4">
+        <v>24</v>
+      </c>
+      <c r="E4">
+        <v>40</v>
+      </c>
+      <c r="F4">
+        <v>20</v>
+      </c>
+      <c r="G4">
+        <v>60</v>
+      </c>
+      <c r="H4">
+        <v>60</v>
+      </c>
+      <c r="I4">
+        <v>80</v>
+      </c>
+      <c r="J4">
         <v>284</v>
       </c>
-      <c r="E4" t="str">
+      <c r="K4" t="str">
         <v>$42,600</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Timeline, coordination, stakeholder management</v>
       </c>
     </row>
     <row r="5">
@@ -2105,14 +4511,29 @@
       <c r="C5" t="str">
         <v>$200</v>
       </c>
-      <c r="D5" t="str">
+      <c r="D5">
+        <v>64</v>
+      </c>
+      <c r="E5">
+        <v>80</v>
+      </c>
+      <c r="F5">
+        <v>100</v>
+      </c>
+      <c r="G5">
+        <v>120</v>
+      </c>
+      <c r="H5">
+        <v>120</v>
+      </c>
+      <c r="I5">
+        <v>80</v>
+      </c>
+      <c r="J5">
         <v>564</v>
       </c>
-      <c r="E5" t="str">
+      <c r="K5" t="str">
         <v>$112,800</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Architecture, code review, technical decisions</v>
       </c>
     </row>
     <row r="6">
@@ -2125,14 +4546,29 @@
       <c r="C6" t="str">
         <v>$185</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>120</v>
+      </c>
+      <c r="F6">
+        <v>40</v>
+      </c>
+      <c r="G6">
+        <v>320</v>
+      </c>
+      <c r="H6">
+        <v>200</v>
+      </c>
+      <c r="I6">
+        <v>80</v>
+      </c>
+      <c r="J6">
         <v>760</v>
       </c>
-      <c r="E6" t="str">
+      <c r="K6" t="str">
         <v>$140,600</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Core blocks, complex components, edge workers</v>
       </c>
     </row>
     <row r="7">
@@ -2145,14 +4581,29 @@
       <c r="C7" t="str">
         <v>$185</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>100</v>
+      </c>
+      <c r="F7">
+        <v>40</v>
+      </c>
+      <c r="G7">
+        <v>280</v>
+      </c>
+      <c r="H7">
+        <v>200</v>
+      </c>
+      <c r="I7">
+        <v>80</v>
+      </c>
+      <c r="J7">
         <v>700</v>
       </c>
-      <c r="E7" t="str">
+      <c r="K7" t="str">
         <v>$129,500</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Complex components</v>
       </c>
     </row>
     <row r="8">
@@ -2165,14 +4616,29 @@
       <c r="C8" t="str">
         <v>$165</v>
       </c>
-      <c r="D8" t="str">
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>80</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>200</v>
+      </c>
+      <c r="H8">
+        <v>160</v>
+      </c>
+      <c r="I8">
+        <v>80</v>
+      </c>
+      <c r="J8">
         <v>520</v>
       </c>
-      <c r="E8" t="str">
+      <c r="K8" t="str">
         <v>$85,800</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Standard blocks</v>
       </c>
     </row>
     <row r="9">
@@ -2185,14 +4651,29 @@
       <c r="C9" t="str">
         <v>$165</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>40</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>160</v>
+      </c>
+      <c r="H9">
+        <v>120</v>
+      </c>
+      <c r="I9">
+        <v>60</v>
+      </c>
+      <c r="J9">
         <v>380</v>
       </c>
-      <c r="E9" t="str">
+      <c r="K9" t="str">
         <v>$62,700</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Templates, CSS</v>
       </c>
     </row>
     <row r="10">
@@ -2205,14 +4686,29 @@
       <c r="C10" t="str">
         <v>$140</v>
       </c>
-      <c r="D10" t="str">
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>24</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>80</v>
+      </c>
+      <c r="H10">
+        <v>80</v>
+      </c>
+      <c r="I10">
+        <v>60</v>
+      </c>
+      <c r="J10">
         <v>244</v>
       </c>
-      <c r="E10" t="str">
+      <c r="K10" t="str">
         <v>$34,160</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Support, simple blocks, testing</v>
       </c>
     </row>
     <row r="11">
@@ -2225,14 +4721,29 @@
       <c r="C11" t="str">
         <v>$135</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D11">
+        <v>40</v>
+      </c>
+      <c r="E11">
+        <v>20</v>
+      </c>
+      <c r="F11">
+        <v>80</v>
+      </c>
+      <c r="G11">
+        <v>40</v>
+      </c>
+      <c r="H11">
+        <v>80</v>
+      </c>
+      <c r="I11">
+        <v>40</v>
+      </c>
+      <c r="J11">
         <v>300</v>
       </c>
-      <c r="E11" t="str">
+      <c r="K11" t="str">
         <v>$40,500</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Content mapping, IA, CF models</v>
       </c>
     </row>
     <row r="12">
@@ -2245,14 +4756,29 @@
       <c r="C12" t="str">
         <v>$95</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>240</v>
+      </c>
+      <c r="I12">
+        <v>60</v>
+      </c>
+      <c r="J12">
         <v>300</v>
       </c>
-      <c r="E12" t="str">
+      <c r="K12" t="str">
         <v>$28,500</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Content migration, DAM management</v>
       </c>
     </row>
     <row r="13">
@@ -2265,14 +4791,29 @@
       <c r="C13" t="str">
         <v>$95</v>
       </c>
-      <c r="D13" t="str">
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>160</v>
+      </c>
+      <c r="I13">
+        <v>40</v>
+      </c>
+      <c r="J13">
         <v>200</v>
       </c>
-      <c r="E13" t="str">
+      <c r="K13" t="str">
         <v>$19,000</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Secondary support</v>
       </c>
     </row>
     <row r="14">
@@ -2285,14 +4826,29 @@
       <c r="C14" t="str">
         <v>$130</v>
       </c>
-      <c r="D14" t="str">
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>80</v>
+      </c>
+      <c r="I14">
+        <v>280</v>
+      </c>
+      <c r="J14">
         <v>360</v>
       </c>
-      <c r="E14" t="str">
+      <c r="K14" t="str">
         <v>$46,800</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Testing, validation, accessibility</v>
       </c>
     </row>
     <row r="15">
@@ -2305,14 +4861,29 @@
       <c r="C15" t="str">
         <v>$140</v>
       </c>
-      <c r="D15" t="str">
+      <c r="D15">
+        <v>32</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>40</v>
+      </c>
+      <c r="J15">
         <v>72</v>
       </c>
-      <c r="E15" t="str">
+      <c r="K15" t="str">
         <v>$10,080</v>
-      </c>
-      <c r="F15" t="str">
-        <v>SEO audit, redirect validation</v>
       </c>
     </row>
     <row r="16">
@@ -2325,14 +4896,29 @@
       <c r="C16" t="str">
         <v>$160</v>
       </c>
-      <c r="D16" t="str">
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>60</v>
+      </c>
+      <c r="I16">
+        <v>60</v>
+      </c>
+      <c r="J16">
         <v>120</v>
       </c>
-      <c r="E16" t="str">
+      <c r="K16" t="str">
         <v>$19,200</v>
-      </c>
-      <c r="F16" t="str">
-        <v>AEM admin, monitoring setup</v>
       </c>
     </row>
     <row r="17">
@@ -2345,19 +4931,34 @@
       <c r="C17" t="str">
         <v/>
       </c>
-      <c r="D17" t="str">
-        <v>4,804</v>
-      </c>
-      <c r="E17" t="str">
+      <c r="D17">
+        <v>160</v>
+      </c>
+      <c r="E17">
+        <v>504</v>
+      </c>
+      <c r="F17">
+        <v>280</v>
+      </c>
+      <c r="G17">
+        <v>1260</v>
+      </c>
+      <c r="H17">
+        <v>1560</v>
+      </c>
+      <c r="I17">
+        <v>1040</v>
+      </c>
+      <c r="J17">
+        <v>4804</v>
+      </c>
+      <c r="K17" t="str">
         <v>$772,240</v>
-      </c>
-      <c r="F17" t="str">
-        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2405,7 +5006,7 @@
       <c r="A5" t="str">
         <v>Phase 0: Pre-Migration</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B5">
         <v>160</v>
       </c>
       <c r="C5" t="str">
@@ -2419,7 +5020,7 @@
       <c r="A6" t="str">
         <v>Phase 1: Foundation</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B6">
         <v>504</v>
       </c>
       <c r="C6" t="str">
@@ -2433,7 +5034,7 @@
       <c r="A7" t="str">
         <v>Phase 2: Content Modeling</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B7">
         <v>280</v>
       </c>
       <c r="C7" t="str">
@@ -2447,8 +5048,8 @@
       <c r="A8" t="str">
         <v>Phase 3: Block Development</v>
       </c>
-      <c r="B8" t="str">
-        <v>1,260</v>
+      <c r="B8">
+        <v>1260</v>
       </c>
       <c r="C8" t="str">
         <v>$218,000</v>
@@ -2461,8 +5062,8 @@
       <c r="A9" t="str">
         <v>Phase 4-6: Migration</v>
       </c>
-      <c r="B9" t="str">
-        <v>1,560</v>
+      <c r="B9">
+        <v>1560</v>
       </c>
       <c r="C9" t="str">
         <v>$248,000</v>
@@ -2475,8 +5076,8 @@
       <c r="A10" t="str">
         <v>Phase 7-9: Validation/Launch</v>
       </c>
-      <c r="B10" t="str">
-        <v>1,040</v>
+      <c r="B10">
+        <v>1040</v>
       </c>
       <c r="C10" t="str">
         <v>$146,240</v>
@@ -2489,8 +5090,8 @@
       <c r="A11" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B11" t="str">
-        <v>4,804</v>
+      <c r="B11">
+        <v>4804</v>
       </c>
       <c r="C11" t="str">
         <v>$772,240</v>

</xml_diff>

<commit_message>
Update Excel with detailed "Why Still Needed" refinement explanations
Block Requirements sheet now includes specific reasons for each block:
- Navigation: Mega-menu JS, touch gestures, focus management
- Hero: Video autoplay, swipe gestures, ARIA roles
- Cards: Hover states, price formatting, animations
- Interactive: State management, API integration, validation
- Forms: CRM integration, GDPR consent, error handling

New "EC Refinement Details" sheet explains 5 categories:
1. Brand Compliance (colors, fonts, spacing)
2. Accessibility (ARIA, keyboard nav, focus)
3. Responsive Behavior (breakpoints, touch, images)
4. Complex Interactions (state, animations, APIs)
5. Testing & QA (cross-browser, devices, edge cases)

Co-Authored-By: Claude (global.anthropic.claude-opus-4-5-20251101-v1:0) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/New-ATT-BUSINESS-MIGRATION-PLAN.xlsx
+++ b/New-ATT-BUSINESS-MIGRATION-PLAN.xlsx
@@ -8,11 +8,12 @@
     <sheet name="Templates" sheetId="3" r:id="rId3"/>
     <sheet name="Phase Summary" sheetId="4" r:id="rId4"/>
     <sheet name="Block Requirements" sheetId="5" r:id="rId5"/>
-    <sheet name="Resources" sheetId="6" r:id="rId6"/>
-    <sheet name="Cost Summary" sheetId="7" r:id="rId7"/>
-    <sheet name="Risk Assessment" sheetId="8" r:id="rId8"/>
-    <sheet name="Manual vs EC-AEMCoder" sheetId="9" r:id="rId9"/>
-    <sheet name="Success Criteria" sheetId="10" r:id="rId10"/>
+    <sheet name="EC Refinement Details" sheetId="6" r:id="rId6"/>
+    <sheet name="Resources" sheetId="7" r:id="rId7"/>
+    <sheet name="Cost Summary" sheetId="8" r:id="rId8"/>
+    <sheet name="Risk Assessment" sheetId="9" r:id="rId9"/>
+    <sheet name="Manual vs EC-AEMCoder" sheetId="10" r:id="rId10"/>
+    <sheet name="Success Criteria" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -598,6 +599,315 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D29"/>
+  <cols>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>EC/AEMCoder vs Manual Approach Comparison</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>WHAT EC/AEMCODER AUTOMATES</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Capability</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Automated</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Manual Effort Remaining</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Block structure generation</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Review and refinement</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Initial HTML → Markdown conversion</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Content validation</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Block CSS scaffolding</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Brand refinement, responsive tuning</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Content mapping to blocks</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Edge case handling</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Basic JavaScript decoration</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Complex interactions, state management</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Image extraction &amp; references</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C10" t="str">
+        <v>DAM migration, optimization</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>WHAT REQUIRES MANUAL WORK</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Task</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Why Manual</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Effort Level</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>CSS brand refinement</v>
+      </c>
+      <c r="B14" t="str">
+        <v>AT&amp;T brand compliance, pixel-perfect styling</v>
+      </c>
+      <c r="C14" t="str">
+        <v>High</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Complex JavaScript interactions</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Pricing calculators, dynamic filtering, animations</v>
+      </c>
+      <c r="C15" t="str">
+        <v>High</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Accessibility compliance</v>
+      </c>
+      <c r="B16" t="str">
+        <v>WCAG 2.1 AA testing, ARIA attributes, keyboard nav</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>component-model.json</v>
+      </c>
+      <c r="B17" t="str">
+        <v>JCR package structure for AEM importer</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>component-definitions.json</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Universal Editor field definitions</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Edge workers</v>
+      </c>
+      <c r="B19" t="str">
+        <v>API proxies, form handling, personalization</v>
+      </c>
+      <c r="C19" t="str">
+        <v>High</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Integration testing</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Third-party scripts, analytics, CRM</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Content validation</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Business accuracy, legal review</v>
+      </c>
+      <c r="C21" t="str">
+        <v>High</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Performance optimization</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Core Web Vitals tuning, lazy loading</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>OVERALL COMPARISON</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Metric</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="C25" t="str">
+        <v>EC/AEMCoder</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Savings</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Duration</v>
+      </c>
+      <c r="B26" t="str">
+        <v>24 weeks</v>
+      </c>
+      <c r="C26" t="str">
+        <v>20-21 weeks</v>
+      </c>
+      <c r="D26" t="str">
+        <v>3-4 weeks</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Total Hours</v>
+      </c>
+      <c r="B27" t="str">
+        <v>4,800</v>
+      </c>
+      <c r="C27" t="str">
+        <v>4,120</v>
+      </c>
+      <c r="D27" t="str">
+        <v>680 hours</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Total Cost</v>
+      </c>
+      <c r="B28" t="str">
+        <v>$920,000</v>
+      </c>
+      <c r="C28" t="str">
+        <v>$790,000</v>
+      </c>
+      <c r="D28" t="str">
+        <v>$130,000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Percentage Reduction</v>
+      </c>
+      <c r="B29" t="str">
+        <v>-</v>
+      </c>
+      <c r="C29" t="str">
+        <v>-</v>
+      </c>
+      <c r="D29" t="str">
+        <v>14%</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D29"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B20"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
@@ -3170,13 +3480,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E80"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="55.83203125" customWidth="1"/>
+    <col min="5" max="5" width="70.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3191,80 +3501,56 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>NAVIGATION BLOCKS (4)</v>
+        <v>NOTE: EC/AEMCoder Hours = Refinement work after automated block generation</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Block Name</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Complexity</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Manual Hrs</v>
-      </c>
-      <c r="D4" t="str">
-        <v>EC Hrs</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Notes</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>header</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Very High</v>
-      </c>
-      <c r="C5">
-        <v>30</v>
-      </c>
-      <c r="D5">
-        <v>30</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Mega menu, search, account login, Personal/Business toggle</v>
+        <v>NAVIGATION BLOCKS (4) - Manual development required (complex interactions)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>footer</v>
+        <v>Block Name</v>
       </c>
       <c r="B6" t="str">
-        <v>High</v>
-      </c>
-      <c r="C6">
-        <v>20</v>
-      </c>
-      <c r="D6">
-        <v>20</v>
+        <v>Complexity</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D6" t="str">
+        <v>EC Hrs</v>
       </c>
       <c r="E6" t="str">
-        <v>Multi-column, social links, legal links</v>
+        <v>Why Refinement Still Needed</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>breadcrumb</v>
+        <v>header</v>
       </c>
       <c r="B7" t="str">
-        <v>Low</v>
+        <v>Very High</v>
       </c>
       <c r="C7">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D7">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E7" t="str">
-        <v>Standard hierarchy</v>
+        <v>Mega-menu requires custom JS for dropdowns, hover states, mobile toggle</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>mobile-nav</v>
+        <v>footer</v>
       </c>
       <c r="B8" t="str">
         <v>High</v>
@@ -3276,85 +3562,85 @@
         <v>20</v>
       </c>
       <c r="E8" t="str">
-        <v>Mobile menu with nested items</v>
+        <v>Multi-region links, dynamic year, legal compliance requirements</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v/>
+        <v>breadcrumb</v>
       </c>
       <c r="B9" t="str">
-        <v/>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v/>
+        <v>Low</v>
+      </c>
+      <c r="C9">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>Schema.org structured data, dynamic path generation</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>HERO BLOCKS (6)</v>
+        <v>mobile-nav</v>
+      </c>
+      <c r="B10" t="str">
+        <v>High</v>
+      </c>
+      <c r="C10">
+        <v>20</v>
+      </c>
+      <c r="D10">
+        <v>20</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Touch gestures, nested accordion behavior, focus management</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Block Name</v>
+        <v/>
       </c>
       <c r="B11" t="str">
-        <v>Complexity</v>
+        <v/>
       </c>
       <c r="C11" t="str">
-        <v>Manual Hrs</v>
+        <v/>
       </c>
       <c r="D11" t="str">
-        <v>EC Hrs</v>
+        <v/>
       </c>
       <c r="E11" t="str">
-        <v>Notes</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>hero-video</v>
-      </c>
-      <c r="B12" t="str">
-        <v>High</v>
-      </c>
-      <c r="C12">
-        <v>24</v>
-      </c>
-      <c r="D12">
-        <v>14</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Background video with overlay text, CTAs</v>
+        <v>HERO BLOCKS (6) - EC generates structure, refinement for brand/interactions</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>hero-carousel</v>
+        <v>Block Name</v>
       </c>
       <c r="B13" t="str">
-        <v>High</v>
-      </c>
-      <c r="C13">
-        <v>24</v>
-      </c>
-      <c r="D13">
-        <v>14</v>
+        <v>Complexity</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D13" t="str">
+        <v>EC Hrs</v>
       </c>
       <c r="E13" t="str">
-        <v>Multiple slides with auto-rotation</v>
+        <v>Why Refinement Still Needed</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>hero-tabs</v>
+        <v>hero-video</v>
       </c>
       <c r="B14" t="str">
         <v>High</v>
@@ -3366,46 +3652,46 @@
         <v>14</v>
       </c>
       <c r="E14" t="str">
-        <v>Tabbed content (Mobile, Internet, Voice, etc.)</v>
+        <v>Video autoplay policies, fallback images, mobile optimization</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>hero-split</v>
+        <v>hero-carousel</v>
       </c>
       <c r="B15" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
       <c r="C15">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D15">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E15" t="str">
-        <v>Two-column layout</v>
+        <v>Swipe gestures, auto-rotation pause on hover, dot navigation</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>hero-minimal</v>
+        <v>hero-tabs</v>
       </c>
       <c r="B16" t="str">
-        <v>Low</v>
+        <v>High</v>
       </c>
       <c r="C16">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E16" t="str">
-        <v>Text-only section header</v>
+        <v>Tab panel ARIA roles, keyboard navigation, content lazy-load</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>hero-promo</v>
+        <v>hero-split</v>
       </c>
       <c r="B17" t="str">
         <v>Medium</v>
@@ -3417,102 +3703,102 @@
         <v>10</v>
       </c>
       <c r="E17" t="str">
-        <v>Promotional banner with pricing</v>
+        <v>Responsive breakpoint tuning, image aspect ratio handling</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v/>
+        <v>hero-minimal</v>
       </c>
       <c r="B18" t="str">
-        <v/>
-      </c>
-      <c r="C18" t="str">
-        <v/>
-      </c>
-      <c r="D18" t="str">
-        <v/>
+        <v>Low</v>
+      </c>
+      <c r="C18">
+        <v>16</v>
+      </c>
+      <c r="D18">
+        <v>10</v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>Typography fine-tuning, spacing adjustments per brand</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>CARD BLOCKS (10)</v>
+        <v>hero-promo</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C19">
+        <v>16</v>
+      </c>
+      <c r="D19">
+        <v>10</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Dynamic pricing display, countdown timer integration</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Block Name</v>
+        <v/>
       </c>
       <c r="B20" t="str">
-        <v>Complexity</v>
+        <v/>
       </c>
       <c r="C20" t="str">
-        <v>Manual Hrs</v>
+        <v/>
       </c>
       <c r="D20" t="str">
-        <v>EC Hrs</v>
+        <v/>
       </c>
       <c r="E20" t="str">
-        <v>Notes</v>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>cards-product</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="C21">
-        <v>20</v>
-      </c>
-      <c r="D21">
-        <v>10</v>
-      </c>
-      <c r="E21" t="str">
-        <v>Product tiles with pricing</v>
+        <v>CARD BLOCKS (10) - EC generates well, minor brand refinement</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>cards-feature</v>
+        <v>Block Name</v>
       </c>
       <c r="B22" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="C22">
-        <v>20</v>
-      </c>
-      <c r="D22">
-        <v>10</v>
+        <v>Complexity</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D22" t="str">
+        <v>EC Hrs</v>
       </c>
       <c r="E22" t="str">
-        <v>Icon/image with text</v>
+        <v>Why Refinement Still Needed</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>cards-pricing</v>
+        <v>cards-product</v>
       </c>
       <c r="B23" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="C23">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D23">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E23" t="str">
-        <v>Pricing comparison cards</v>
+        <v>Hover states, price formatting, "Add to cart" integration</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>cards-industry</v>
+        <v>cards-feature</v>
       </c>
       <c r="B24" t="str">
         <v>Medium</v>
@@ -3524,29 +3810,29 @@
         <v>10</v>
       </c>
       <c r="E24" t="str">
-        <v>Industry solution cards</v>
+        <v>Icon alignment, responsive grid behavior</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>cards-story</v>
+        <v>cards-pricing</v>
       </c>
       <c r="B25" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
       <c r="C25">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D25">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E25" t="str">
-        <v>Customer story previews</v>
+        <v>Price comparison logic, "Most Popular" badge, toggle monthly/annual</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>cards-stat</v>
+        <v>cards-industry</v>
       </c>
       <c r="B26" t="str">
         <v>Medium</v>
@@ -3558,29 +3844,29 @@
         <v>10</v>
       </c>
       <c r="E26" t="str">
-        <v>Large numbers with descriptions</v>
+        <v>Industry icon mapping, hover animations</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>cards-cta</v>
+        <v>cards-story</v>
       </c>
       <c r="B27" t="str">
-        <v>Low</v>
+        <v>Medium</v>
       </c>
       <c r="C27">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D27">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E27" t="str">
-        <v>Simple call-to-action cards</v>
+        <v>Thumbnail cropping, read time calculation, category tags</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>cards-icon</v>
+        <v>cards-stat</v>
       </c>
       <c r="B28" t="str">
         <v>Medium</v>
@@ -3592,32 +3878,32 @@
         <v>10</v>
       </c>
       <c r="E28" t="str">
-        <v>Icon-based feature cards</v>
+        <v>Number animation on scroll, suffix/prefix handling</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>cards-testimonial</v>
+        <v>cards-cta</v>
       </c>
       <c r="B29" t="str">
-        <v>Medium</v>
+        <v>Low</v>
       </c>
       <c r="C29">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D29">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E29" t="str">
-        <v>Customer quotes</v>
+        <v>Button variant styling, tracking attributes</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>cards-link</v>
+        <v>cards-icon</v>
       </c>
       <c r="B30" t="str">
-        <v>Low</v>
+        <v>Medium</v>
       </c>
       <c r="C30">
         <v>20</v>
@@ -3626,102 +3912,102 @@
         <v>10</v>
       </c>
       <c r="E30" t="str">
-        <v>Quick link lists</v>
+        <v>SVG icon color inheritance, spacing consistency</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v/>
+        <v>cards-testimonial</v>
       </c>
       <c r="B31" t="str">
-        <v/>
-      </c>
-      <c r="C31" t="str">
-        <v/>
-      </c>
-      <c r="D31" t="str">
-        <v/>
+        <v>Medium</v>
+      </c>
+      <c r="C31">
+        <v>20</v>
+      </c>
+      <c r="D31">
+        <v>10</v>
       </c>
       <c r="E31" t="str">
-        <v/>
+        <v>Quote styling, avatar fallbacks, company logo placement</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>INTERACTIVE BLOCKS (10)</v>
+        <v>cards-link</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Low</v>
+      </c>
+      <c r="C32">
+        <v>20</v>
+      </c>
+      <c r="D32">
+        <v>10</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Arrow icon animation, visited state styling</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Block Name</v>
+        <v/>
       </c>
       <c r="B33" t="str">
-        <v>Complexity</v>
+        <v/>
       </c>
       <c r="C33" t="str">
-        <v>Manual Hrs</v>
+        <v/>
       </c>
       <c r="D33" t="str">
-        <v>EC Hrs</v>
+        <v/>
       </c>
       <c r="E33" t="str">
-        <v>Notes</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>accordion</v>
-      </c>
-      <c r="B34" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="C34">
-        <v>24</v>
-      </c>
-      <c r="D34">
-        <v>14</v>
-      </c>
-      <c r="E34" t="str">
-        <v>FAQ, product details</v>
+        <v>INTERACTIVE BLOCKS (10) - Require significant JS refinement</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>tabs</v>
+        <v>Block Name</v>
       </c>
       <c r="B35" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="C35">
-        <v>24</v>
-      </c>
-      <c r="D35">
-        <v>14</v>
+        <v>Complexity</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D35" t="str">
+        <v>EC Hrs</v>
       </c>
       <c r="E35" t="str">
-        <v>Content organization</v>
+        <v>Why Refinement Still Needed</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>carousel</v>
+        <v>accordion</v>
       </c>
       <c r="B36" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="C36">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D36">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E36" t="str">
-        <v>Image/content slider</v>
+        <v>ARIA expanded states, smooth height animation, multi-open option</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>modal</v>
+        <v>tabs</v>
       </c>
       <c r="B37" t="str">
         <v>Medium</v>
@@ -3733,63 +4019,63 @@
         <v>14</v>
       </c>
       <c r="E37" t="str">
-        <v>Popup dialogs, offer details</v>
+        <v>Keyboard arrow navigation, ARIA tablist roles, lazy content load</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>video</v>
+        <v>carousel</v>
       </c>
       <c r="B38" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
       <c r="C38">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D38">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E38" t="str">
-        <v>Inline video player</v>
+        <v>Touch/swipe support, infinite loop, responsive slides per view</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>video-modal</v>
+        <v>modal</v>
       </c>
       <c r="B39" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="C39">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D39">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E39" t="str">
-        <v>Lightbox video player</v>
+        <v>Focus trap, escape key close, scroll lock on body</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>search</v>
+        <v>video</v>
       </c>
       <c r="B40" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="C40">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D40">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E40" t="str">
-        <v>Site search with filtering</v>
+        <v>YouTube/Vimeo API integration, custom controls, tracking events</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>filter</v>
+        <v>video-modal</v>
       </c>
       <c r="B41" t="str">
         <v>High</v>
@@ -3801,15 +4087,15 @@
         <v>19</v>
       </c>
       <c r="E41" t="str">
-        <v>Product filtering</v>
+        <v>Lightbox overlay, video pause on close, responsive sizing</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>pricing-calculator</v>
+        <v>search</v>
       </c>
       <c r="B42" t="str">
-        <v>Very High</v>
+        <v>High</v>
       </c>
       <c r="C42">
         <v>32</v>
@@ -3818,153 +4104,153 @@
         <v>19</v>
       </c>
       <c r="E42" t="str">
-        <v>Dynamic pricing tool</v>
+        <v>Autocomplete, debounced API calls, result highlighting</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>comparison-table</v>
+        <v>filter</v>
       </c>
       <c r="B43" t="str">
         <v>High</v>
       </c>
       <c r="C43">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D43">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E43" t="str">
-        <v>Product comparison</v>
+        <v>Multi-select logic, URL state sync, clear all functionality</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v/>
+        <v>pricing-calculator</v>
       </c>
       <c r="B44" t="str">
-        <v/>
-      </c>
-      <c r="C44" t="str">
-        <v/>
-      </c>
-      <c r="D44" t="str">
-        <v/>
+        <v>Very High</v>
+      </c>
+      <c r="C44">
+        <v>32</v>
+      </c>
+      <c r="D44">
+        <v>19</v>
       </c>
       <c r="E44" t="str">
-        <v/>
+        <v>Complex business logic, real-time API calls, validation</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>CONTENT BLOCKS (8)</v>
+        <v>comparison-table</v>
+      </c>
+      <c r="B45" t="str">
+        <v>High</v>
+      </c>
+      <c r="C45">
+        <v>24</v>
+      </c>
+      <c r="D45">
+        <v>17</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Sticky headers, horizontal scroll on mobile, highlight differences</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Block Name</v>
+        <v/>
       </c>
       <c r="B46" t="str">
-        <v>Complexity</v>
+        <v/>
       </c>
       <c r="C46" t="str">
-        <v>Manual Hrs</v>
+        <v/>
       </c>
       <c r="D46" t="str">
-        <v>EC Hrs</v>
+        <v/>
       </c>
       <c r="E46" t="str">
-        <v>Notes</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>columns</v>
-      </c>
-      <c r="B47" t="str">
-        <v>Low</v>
-      </c>
-      <c r="C47">
-        <v>16</v>
-      </c>
-      <c r="D47">
-        <v>8</v>
-      </c>
-      <c r="E47" t="str">
-        <v>Multi-column layouts</v>
+        <v>CONTENT BLOCKS (8) - EC generates well, minimal refinement</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>quote</v>
+        <v>Block Name</v>
       </c>
       <c r="B48" t="str">
-        <v>Low</v>
-      </c>
-      <c r="C48">
-        <v>16</v>
-      </c>
-      <c r="D48">
-        <v>8</v>
+        <v>Complexity</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D48" t="str">
+        <v>EC Hrs</v>
       </c>
       <c r="E48" t="str">
-        <v>Testimonials, pull quotes</v>
+        <v>Why Refinement Still Needed</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>table</v>
+        <v>columns</v>
       </c>
       <c r="B49" t="str">
-        <v>Medium</v>
+        <v>Low</v>
       </c>
       <c r="C49">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D49">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E49" t="str">
-        <v>Data tables</v>
+        <v>Responsive stacking order, gap consistency</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>embed</v>
+        <v>quote</v>
       </c>
       <c r="B50" t="str">
-        <v>Medium</v>
+        <v>Low</v>
       </c>
       <c r="C50">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D50">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E50" t="str">
-        <v>External content (YouTube, maps)</v>
+        <v>Quotation mark styling, attribution formatting</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>download</v>
+        <v>table</v>
       </c>
       <c r="B51" t="str">
-        <v>Low</v>
+        <v>Medium</v>
       </c>
       <c r="C51">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D51">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E51" t="str">
-        <v>PDF/document links</v>
+        <v>Responsive horizontal scroll, sortable headers option</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>cta-banner</v>
+        <v>embed</v>
       </c>
       <c r="B52" t="str">
         <v>Medium</v>
@@ -3976,12 +4262,12 @@
         <v>12</v>
       </c>
       <c r="E52" t="str">
-        <v>Full-width call-to-action</v>
+        <v>Aspect ratio preservation, lazy loading, consent wrapper</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>divider</v>
+        <v>download</v>
       </c>
       <c r="B53" t="str">
         <v>Low</v>
@@ -3993,12 +4279,12 @@
         <v>8</v>
       </c>
       <c r="E53" t="str">
-        <v>Section separators</v>
+        <v>File type icons, size display, download tracking</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>icon-list</v>
+        <v>cta-banner</v>
       </c>
       <c r="B54" t="str">
         <v>Medium</v>
@@ -4010,102 +4296,102 @@
         <v>12</v>
       </c>
       <c r="E54" t="str">
-        <v>Feature lists with icons</v>
+        <v>Background image positioning, button placement variants</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v/>
+        <v>divider</v>
       </c>
       <c r="B55" t="str">
-        <v/>
-      </c>
-      <c r="C55" t="str">
-        <v/>
-      </c>
-      <c r="D55" t="str">
-        <v/>
+        <v>Low</v>
+      </c>
+      <c r="C55">
+        <v>16</v>
+      </c>
+      <c r="D55">
+        <v>8</v>
       </c>
       <c r="E55" t="str">
-        <v/>
+        <v>Spacing tokens, optional icon/text in divider</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>FORM BLOCKS (4)</v>
+        <v>icon-list</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C56">
+        <v>24</v>
+      </c>
+      <c r="D56">
+        <v>12</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Icon color theming, vertical/horizontal layout options</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Block Name</v>
+        <v/>
       </c>
       <c r="B57" t="str">
-        <v>Complexity</v>
+        <v/>
       </c>
       <c r="C57" t="str">
-        <v>Manual Hrs</v>
+        <v/>
       </c>
       <c r="D57" t="str">
-        <v>EC Hrs</v>
+        <v/>
       </c>
       <c r="E57" t="str">
-        <v>Notes</v>
+        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>lead-form</v>
-      </c>
-      <c r="B58" t="str">
-        <v>High</v>
-      </c>
-      <c r="C58">
-        <v>36</v>
-      </c>
-      <c r="D58">
-        <v>22</v>
-      </c>
-      <c r="E58" t="str">
-        <v>Sales contact form (RAI form)</v>
+        <v>FORM BLOCKS (4) - Require validation and backend integration</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>contact-form</v>
+        <v>Block Name</v>
       </c>
       <c r="B59" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="C59">
-        <v>28</v>
-      </c>
-      <c r="D59">
-        <v>17</v>
+        <v>Complexity</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D59" t="str">
+        <v>EC Hrs</v>
       </c>
       <c r="E59" t="str">
-        <v>General inquiry</v>
+        <v>Why Refinement Still Needed</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>newsletter</v>
+        <v>lead-form</v>
       </c>
       <c r="B60" t="str">
-        <v>Medium</v>
+        <v>High</v>
       </c>
       <c r="C60">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D60">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E60" t="str">
-        <v>Email signup</v>
+        <v>Field validation, CRM integration, GDPR consent, error states</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>search-input</v>
+        <v>contact-form</v>
       </c>
       <c r="B61" t="str">
         <v>Medium</v>
@@ -4114,216 +4400,216 @@
         <v>28</v>
       </c>
       <c r="D61">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E61" t="str">
-        <v>Search box</v>
+        <v>reCAPTCHA integration, email formatting, success/error messages</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v/>
+        <v>newsletter</v>
       </c>
       <c r="B62" t="str">
-        <v/>
-      </c>
-      <c r="C62" t="str">
-        <v/>
-      </c>
-      <c r="D62" t="str">
-        <v/>
+        <v>Medium</v>
+      </c>
+      <c r="C62">
+        <v>28</v>
+      </c>
+      <c r="D62">
+        <v>17</v>
       </c>
       <c r="E62" t="str">
-        <v/>
+        <v>Email validation, double opt-in flow, Mailchimp/Marketo integration</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>AT&amp;T-SPECIFIC BLOCKS (3)</v>
+        <v>search-input</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C63">
+        <v>28</v>
+      </c>
+      <c r="D63">
+        <v>16</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Autocomplete dropdown, clear button, voice search option</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Block Name</v>
+        <v/>
       </c>
       <c r="B64" t="str">
-        <v>Complexity</v>
+        <v/>
       </c>
       <c r="C64" t="str">
-        <v>Manual Hrs</v>
+        <v/>
       </c>
       <c r="D64" t="str">
-        <v>EC Hrs</v>
+        <v/>
       </c>
       <c r="E64" t="str">
-        <v>Notes</v>
+        <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>guarantee-banner</v>
-      </c>
-      <c r="B65" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="C65">
-        <v>24</v>
-      </c>
-      <c r="D65">
-        <v>13</v>
-      </c>
-      <c r="E65" t="str">
-        <v>AT&amp;T Guarantee messaging</v>
+        <v>AT&amp;T-SPECIFIC BLOCKS (3) - Brand-specific customization</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>offer-card</v>
+        <v>Block Name</v>
       </c>
       <c r="B66" t="str">
-        <v>High</v>
-      </c>
-      <c r="C66">
-        <v>32</v>
-      </c>
-      <c r="D66">
-        <v>17</v>
+        <v>Complexity</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D66" t="str">
+        <v>EC Hrs</v>
       </c>
       <c r="E66" t="str">
-        <v>Dynamic promotional offers</v>
+        <v>Why Refinement Still Needed</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>jd-power-badge</v>
+        <v>guarantee-banner</v>
       </c>
       <c r="B67" t="str">
-        <v>Low</v>
+        <v>Medium</v>
       </c>
       <c r="C67">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D67">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E67" t="str">
-        <v>Award/certification badges</v>
+        <v>Legal text formatting, icon animation, link to terms</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v/>
+        <v>offer-card</v>
       </c>
       <c r="B68" t="str">
-        <v/>
-      </c>
-      <c r="C68" t="str">
-        <v/>
-      </c>
-      <c r="D68" t="str">
-        <v/>
+        <v>High</v>
+      </c>
+      <c r="C68">
+        <v>32</v>
+      </c>
+      <c r="D68">
+        <v>17</v>
       </c>
       <c r="E68" t="str">
-        <v/>
+        <v>Dynamic offer API, expiration countdown, personalization rules</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>BLOCK TOTALS</v>
+        <v>jd-power-badge</v>
       </c>
       <c r="B69" t="str">
-        <v/>
-      </c>
-      <c r="C69" t="str">
-        <v/>
-      </c>
-      <c r="D69" t="str">
-        <v/>
+        <v>Low</v>
+      </c>
+      <c r="C69">
+        <v>16</v>
+      </c>
+      <c r="D69">
+        <v>8</v>
       </c>
       <c r="E69" t="str">
-        <v/>
+        <v>Badge image optimization, award year update, tooltip</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Category</v>
+        <v/>
       </c>
       <c r="B70" t="str">
-        <v>Count</v>
+        <v/>
       </c>
       <c r="C70" t="str">
-        <v>Manual Hrs</v>
+        <v/>
       </c>
       <c r="D70" t="str">
-        <v>EC Hrs</v>
+        <v/>
       </c>
       <c r="E70" t="str">
-        <v>Reduction</v>
+        <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Navigation</v>
-      </c>
-      <c r="B71">
-        <v>4</v>
-      </c>
-      <c r="C71">
-        <v>80</v>
-      </c>
-      <c r="D71">
-        <v>80</v>
+        <v>BLOCK TOTALS</v>
+      </c>
+      <c r="B71" t="str">
+        <v/>
+      </c>
+      <c r="C71" t="str">
+        <v/>
+      </c>
+      <c r="D71" t="str">
+        <v/>
       </c>
       <c r="E71" t="str">
-        <v>0%</v>
+        <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Hero</v>
-      </c>
-      <c r="B72">
-        <v>6</v>
-      </c>
-      <c r="C72">
-        <v>120</v>
-      </c>
-      <c r="D72">
-        <v>72</v>
+        <v>Category</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Count</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Manual Hrs</v>
+      </c>
+      <c r="D72" t="str">
+        <v>EC Hrs</v>
       </c>
       <c r="E72" t="str">
-        <v>40%</v>
+        <v>Reduction</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Cards</v>
+        <v>Navigation</v>
       </c>
       <c r="B73">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C73">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="D73">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="E73" t="str">
-        <v>50%</v>
+        <v>0% (manual required)</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Interactive</v>
+        <v>Hero</v>
       </c>
       <c r="B74">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C74">
-        <v>280</v>
+        <v>120</v>
       </c>
       <c r="D74">
-        <v>168</v>
+        <v>72</v>
       </c>
       <c r="E74" t="str">
         <v>40%</v>
@@ -4331,16 +4617,16 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Content</v>
+        <v>Cards</v>
       </c>
       <c r="B75">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C75">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="D75">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="E75" t="str">
         <v>50%</v>
@@ -4348,16 +4634,16 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Forms</v>
+        <v>Interactive</v>
       </c>
       <c r="B76">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C76">
-        <v>120</v>
+        <v>280</v>
       </c>
       <c r="D76">
-        <v>72</v>
+        <v>168</v>
       </c>
       <c r="E76" t="str">
         <v>40%</v>
@@ -4365,46 +4651,766 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>AT&amp;T-Specific</v>
+        <v>Content</v>
       </c>
       <c r="B77">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C77">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="D77">
-        <v>38</v>
+        <v>80</v>
       </c>
       <c r="E77" t="str">
-        <v>47%</v>
+        <v>50%</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
+        <v>Forms</v>
+      </c>
+      <c r="B78">
+        <v>4</v>
+      </c>
+      <c r="C78">
+        <v>120</v>
+      </c>
+      <c r="D78">
+        <v>72</v>
+      </c>
+      <c r="E78" t="str">
+        <v>40%</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>AT&amp;T-Specific</v>
+      </c>
+      <c r="B79">
+        <v>3</v>
+      </c>
+      <c r="C79">
+        <v>72</v>
+      </c>
+      <c r="D79">
+        <v>38</v>
+      </c>
+      <c r="E79" t="str">
+        <v>47%</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B78">
+      <c r="B80">
         <v>45</v>
       </c>
-      <c r="C78">
+      <c r="C80">
         <v>1032</v>
       </c>
-      <c r="D78">
+      <c r="D80">
         <v>610</v>
       </c>
-      <c r="E78" t="str">
+      <c r="E80" t="str">
         <v>~41%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E80"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D51"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="55.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>EC/AEMCoder Block Refinement - Why Hours Are Still Needed</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>EC/AEMCoder generates initial block structure, CSS scaffolding, and content mapping.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>The hours below represent REFINEMENT work required after automated generation.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>REFINEMENT CATEGORY</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Description</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Typical Effort</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Blocks Affected</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>1. BRAND COMPLIANCE</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>AT&amp;T color tokens</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Map generated colors to AT&amp;T brand palette (#009FDB, #0568AE)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2-4 hrs/block</v>
+      </c>
+      <c r="D9" t="str">
+        <v>All blocks</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Typography tuning</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Apply AT&amp;T Aleck Sans/Slab fonts, adjust line heights</v>
+      </c>
+      <c r="C10" t="str">
+        <v>1-2 hrs/block</v>
+      </c>
+      <c r="D10" t="str">
+        <v>All blocks</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Spacing consistency</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Align padding/margins to AT&amp;T design system grid</v>
+      </c>
+      <c r="C11" t="str">
+        <v>1-2 hrs/block</v>
+      </c>
+      <c r="D11" t="str">
+        <v>All blocks</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2. ACCESSIBILITY (WCAG 2.1 AA)</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>ARIA attributes</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Add aria-label, aria-expanded, aria-controls, roles</v>
+      </c>
+      <c r="C14" t="str">
+        <v>2-4 hrs/block</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Interactive, Forms</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Keyboard navigation</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Tab order, Enter/Space activation, arrow key support</v>
+      </c>
+      <c r="C15" t="str">
+        <v>2-4 hrs/block</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Interactive, Nav</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Focus management</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Visible focus rings, focus trap in modals</v>
+      </c>
+      <c r="C16" t="str">
+        <v>1-2 hrs/block</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Modal, Forms</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Screen reader testing</v>
+      </c>
+      <c r="B17" t="str">
+        <v>VoiceOver/NVDA testing and fixes</v>
+      </c>
+      <c r="C17" t="str">
+        <v>2-3 hrs/block</v>
+      </c>
+      <c r="D17" t="str">
+        <v>All blocks</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v/>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>3. RESPONSIVE BEHAVIOR</v>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Mobile breakpoints</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Adjust layouts for 320px-768px viewports</v>
+      </c>
+      <c r="C20" t="str">
+        <v>2-4 hrs/block</v>
+      </c>
+      <c r="D20" t="str">
+        <v>All blocks</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Touch interactions</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Swipe gestures, tap targets (44px min)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>2-3 hrs/block</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Carousel, Nav</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Image optimization</v>
+      </c>
+      <c r="B22" t="str">
+        <v>srcset, lazy loading, aspect ratio handling</v>
+      </c>
+      <c r="C22" t="str">
+        <v>1-2 hrs/block</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Hero, Cards</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v/>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v/>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>4. COMPLEX INTERACTIONS (Not automated)</v>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>State management</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Open/close states, active tabs, selected filters</v>
+      </c>
+      <c r="C25" t="str">
+        <v>4-8 hrs/block</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Interactive</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Animation/transitions</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Smooth height changes, fade effects, slide animations</v>
+      </c>
+      <c r="C26" t="str">
+        <v>2-4 hrs/block</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Accordion, Modal</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>API integration</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Fetch data, handle loading/error states</v>
+      </c>
+      <c r="C27" t="str">
+        <v>4-8 hrs/block</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Search, Pricing</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Form validation</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Field validation, error messages, submit handling</v>
+      </c>
+      <c r="C28" t="str">
+        <v>4-6 hrs/block</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Forms</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v/>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>5. TESTING &amp; QA</v>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Cross-browser testing</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Chrome, Safari, Firefox, Edge verification</v>
+      </c>
+      <c r="C31" t="str">
+        <v>1-2 hrs/block</v>
+      </c>
+      <c r="D31" t="str">
+        <v>All blocks</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Device testing</v>
+      </c>
+      <c r="B32" t="str">
+        <v>iOS Safari, Android Chrome, tablet layouts</v>
+      </c>
+      <c r="C32" t="str">
+        <v>1-2 hrs/block</v>
+      </c>
+      <c r="D32" t="str">
+        <v>All blocks</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Edge case handling</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Empty states, long text, missing images</v>
+      </c>
+      <c r="C33" t="str">
+        <v>1-2 hrs/block</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Cards, Content</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v/>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>SUMMARY: WHY 600 HOURS FOR EC/AEMCODER BLOCKS</v>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v/>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>What EC/AEMCoder Handles (saves ~480 hours):</v>
+      </c>
+      <c r="B38" t="str">
+        <v/>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>- Initial HTML structure generation</v>
+      </c>
+      <c r="B39" t="str">
+        <v/>
+      </c>
+      <c r="C39" t="str">
+        <v/>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>- Basic CSS scaffolding from source site</v>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>- Content-to-block mapping</v>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v/>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>- Image reference extraction</v>
+      </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
+      <c r="C42" t="str">
+        <v/>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>- Markdown structure creation</v>
+      </c>
+      <c r="B43" t="str">
+        <v/>
+      </c>
+      <c r="C43" t="str">
+        <v/>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v/>
+      </c>
+      <c r="B44" t="str">
+        <v/>
+      </c>
+      <c r="C44" t="str">
+        <v/>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>What Still Requires Manual Work (600 hours):</v>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45" t="str">
+        <v/>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>- AT&amp;T brand compliance (colors, fonts, spacing)</v>
+      </c>
+      <c r="B46" t="str">
+        <v/>
+      </c>
+      <c r="C46" t="str">
+        <v/>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>- WCAG 2.1 AA accessibility compliance</v>
+      </c>
+      <c r="B47" t="str">
+        <v/>
+      </c>
+      <c r="C47" t="str">
+        <v/>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>- Complex JavaScript interactions</v>
+      </c>
+      <c r="B48" t="str">
+        <v/>
+      </c>
+      <c r="C48" t="str">
+        <v/>
+      </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>- Form validation and backend integration</v>
+      </c>
+      <c r="B49" t="str">
+        <v/>
+      </c>
+      <c r="C49" t="str">
+        <v/>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>- Responsive fine-tuning for all breakpoints</v>
+      </c>
+      <c r="B50" t="str">
+        <v/>
+      </c>
+      <c r="C50" t="str">
+        <v/>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>- Cross-browser and device testing</v>
+      </c>
+      <c r="B51" t="str">
+        <v/>
+      </c>
+      <c r="C51" t="str">
+        <v/>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D51"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K17"/>
   <cols>
@@ -4963,7 +5969,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D36"/>
   <cols>
@@ -5403,7 +6409,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D20"/>
   <cols>
@@ -5662,313 +6668,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D29"/>
-  <cols>
-    <col min="1" max="1" width="35.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>EC/AEMCoder vs Manual Approach Comparison</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>WHAT EC/AEMCODER AUTOMATES</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Capability</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Automated</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Manual Effort Remaining</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Block structure generation</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Review and refinement</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Initial HTML → Markdown conversion</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Content validation</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Block CSS scaffolding</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Brand refinement, responsive tuning</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Content mapping to blocks</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Edge case handling</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Basic JavaScript decoration</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Partial</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Complex interactions, state management</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Image extraction &amp; references</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C10" t="str">
-        <v>DAM migration, optimization</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>WHAT REQUIRES MANUAL WORK</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Task</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Why Manual</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Effort Level</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>CSS brand refinement</v>
-      </c>
-      <c r="B14" t="str">
-        <v>AT&amp;T brand compliance, pixel-perfect styling</v>
-      </c>
-      <c r="C14" t="str">
-        <v>High</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Complex JavaScript interactions</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Pricing calculators, dynamic filtering, animations</v>
-      </c>
-      <c r="C15" t="str">
-        <v>High</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Accessibility compliance</v>
-      </c>
-      <c r="B16" t="str">
-        <v>WCAG 2.1 AA testing, ARIA attributes, keyboard nav</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Medium</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>component-model.json</v>
-      </c>
-      <c r="B17" t="str">
-        <v>JCR package structure for AEM importer</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Medium</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>component-definitions.json</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Universal Editor field definitions</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Medium</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Edge workers</v>
-      </c>
-      <c r="B19" t="str">
-        <v>API proxies, form handling, personalization</v>
-      </c>
-      <c r="C19" t="str">
-        <v>High</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Integration testing</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Third-party scripts, analytics, CRM</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Medium</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Content validation</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Business accuracy, legal review</v>
-      </c>
-      <c r="C21" t="str">
-        <v>High</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Performance optimization</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Core Web Vitals tuning, lazy loading</v>
-      </c>
-      <c r="C22" t="str">
-        <v>Medium</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>OVERALL COMPARISON</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Metric</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Manual</v>
-      </c>
-      <c r="C25" t="str">
-        <v>EC/AEMCoder</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Savings</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>Duration</v>
-      </c>
-      <c r="B26" t="str">
-        <v>24 weeks</v>
-      </c>
-      <c r="C26" t="str">
-        <v>20-21 weeks</v>
-      </c>
-      <c r="D26" t="str">
-        <v>3-4 weeks</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>Total Hours</v>
-      </c>
-      <c r="B27" t="str">
-        <v>4,800</v>
-      </c>
-      <c r="C27" t="str">
-        <v>4,120</v>
-      </c>
-      <c r="D27" t="str">
-        <v>680 hours</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Total Cost</v>
-      </c>
-      <c r="B28" t="str">
-        <v>$920,000</v>
-      </c>
-      <c r="C28" t="str">
-        <v>$790,000</v>
-      </c>
-      <c r="D28" t="str">
-        <v>$130,000</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Percentage Reduction</v>
-      </c>
-      <c r="B29" t="str">
-        <v>-</v>
-      </c>
-      <c r="C29" t="str">
-        <v>-</v>
-      </c>
-      <c r="D29" t="str">
-        <v>14%</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D29"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Update migration plan for 749 pages (was 200+)
Major estimate revisions:
- Duration: 28-30 weeks (Manual) / 24-26 weeks (EC/AEMCoder)
- Hours: 7,200 (Manual) / 6,400 (EC/AEMCoder)
- Cost: $1,380,000 (Manual) / $1,225,000 (EC/AEMCoder)
- Savings: ~$155,000 (11%)

Key changes:
- Phase 4 (Page Review & Assets): 360 → 1,350 hours
- Added 3rd Content Author to handle volume
- Team size: 12-14 FTEs (was 10-12)
- Validation hours increased for 749 page coverage
- Risk assessment updated for content volume challenges

Co-Authored-By: Claude (global.anthropic.claude-opus-4-5-20251101-v1:0) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/New-ATT-BUSINESS-MIGRATION-PLAN.xlsx
+++ b/New-ATT-BUSINESS-MIGRATION-PLAN.xlsx
@@ -453,7 +453,7 @@
         <v>Document Version</v>
       </c>
       <c r="B6" t="str">
-        <v>1.0</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="7">
@@ -482,13 +482,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Total Estimated Pages</v>
+        <v>Total Pages to Migrate</v>
       </c>
       <c r="B10" t="str">
-        <v>200+</v>
+        <v>749</v>
       </c>
       <c r="C10" t="str">
-        <v>200+</v>
+        <v>749</v>
       </c>
     </row>
     <row r="11">
@@ -540,10 +540,10 @@
         <v>Estimated Duration</v>
       </c>
       <c r="B15" t="str">
-        <v>24 weeks</v>
+        <v>28-30 weeks</v>
       </c>
       <c r="C15" t="str">
-        <v>20-21 weeks</v>
+        <v>24-26 weeks</v>
       </c>
     </row>
     <row r="16">
@@ -551,10 +551,10 @@
         <v>Total Project Hours</v>
       </c>
       <c r="B16" t="str">
-        <v>4,800 hours</v>
+        <v>7,200 hours</v>
       </c>
       <c r="C16" t="str">
-        <v>4,120 hours</v>
+        <v>6,400 hours</v>
       </c>
     </row>
     <row r="17">
@@ -562,10 +562,10 @@
         <v>Team Size</v>
       </c>
       <c r="B17" t="str">
-        <v>10-12 FTEs</v>
+        <v>12-14 FTEs</v>
       </c>
       <c r="C17" t="str">
-        <v>9-11 FTEs</v>
+        <v>11-13 FTEs</v>
       </c>
     </row>
     <row r="18">
@@ -573,10 +573,10 @@
         <v>Estimated Cost</v>
       </c>
       <c r="B18" t="str">
-        <v>$920,000</v>
+        <v>$1,380,000</v>
       </c>
       <c r="C18" t="str">
-        <v>$790,000</v>
+        <v>$1,225,000</v>
       </c>
     </row>
     <row r="19">
@@ -587,7 +587,7 @@
         <v>-</v>
       </c>
       <c r="C19" t="str">
-        <v>~$130,000 (14%)</v>
+        <v>~$155,000 (11%)</v>
       </c>
     </row>
   </sheetData>
@@ -599,7 +599,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -609,7 +609,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>EC/AEMCoder vs Manual Approach Comparison</v>
+        <v>EC/AEMCoder vs Manual Approach Comparison (749 Pages)</v>
       </c>
     </row>
     <row r="2">
@@ -799,13 +799,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Content validation</v>
+        <v>Content validation (749 pages)</v>
       </c>
       <c r="B21" t="str">
         <v>Business accuracy, legal review</v>
       </c>
       <c r="C21" t="str">
-        <v>High</v>
+        <v>Very High</v>
       </c>
     </row>
     <row r="22">
@@ -826,7 +826,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>OVERALL COMPARISON</v>
+        <v>OVERALL COMPARISON (749 PAGES)</v>
       </c>
     </row>
     <row r="25">
@@ -848,13 +848,13 @@
         <v>Duration</v>
       </c>
       <c r="B26" t="str">
-        <v>24 weeks</v>
+        <v>28-30 weeks</v>
       </c>
       <c r="C26" t="str">
-        <v>20-21 weeks</v>
+        <v>24-26 weeks</v>
       </c>
       <c r="D26" t="str">
-        <v>3-4 weeks</v>
+        <v>4-6 weeks</v>
       </c>
     </row>
     <row r="27">
@@ -862,13 +862,13 @@
         <v>Total Hours</v>
       </c>
       <c r="B27" t="str">
-        <v>4,800</v>
+        <v>7,200</v>
       </c>
       <c r="C27" t="str">
-        <v>4,120</v>
+        <v>6,400</v>
       </c>
       <c r="D27" t="str">
-        <v>680 hours</v>
+        <v>800 hours</v>
       </c>
     </row>
     <row r="28">
@@ -876,13 +876,13 @@
         <v>Total Cost</v>
       </c>
       <c r="B28" t="str">
-        <v>$920,000</v>
+        <v>$1,380,000</v>
       </c>
       <c r="C28" t="str">
-        <v>$790,000</v>
+        <v>$1,225,000</v>
       </c>
       <c r="D28" t="str">
-        <v>$130,000</v>
+        <v>$155,000</v>
       </c>
     </row>
     <row r="29">
@@ -896,27 +896,41 @@
         <v>-</v>
       </c>
       <c r="D29" t="str">
-        <v>14%</v>
+        <v>~11%</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Team Size</v>
+      </c>
+      <c r="B30" t="str">
+        <v>12-14 FTEs</v>
+      </c>
+      <c r="C30" t="str">
+        <v>11-13 FTEs</v>
+      </c>
+      <c r="D30" t="str">
+        <v>1-2 FTEs</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Success Criteria</v>
+        <v>Success Criteria (749 Pages)</v>
       </c>
     </row>
     <row r="2">
@@ -982,7 +996,7 @@
         <v>Mobile responsiveness</v>
       </c>
       <c r="B10" t="str">
-        <v>100% pages</v>
+        <v>100% of 749 pages</v>
       </c>
     </row>
     <row r="11">
@@ -1056,12 +1070,20 @@
         <v>SEO rankings</v>
       </c>
       <c r="B20" t="str">
-        <v>No degradation</v>
+        <v>No degradation across 749 pages</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Redirect success rate</v>
+      </c>
+      <c r="B21" t="str">
+        <v>&gt; 99.5% (749 URLs)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1072,7 +1094,7 @@
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="3" max="3" width="55.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" customWidth="1"/>
@@ -1081,7 +1103,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>AT&amp;T Business Migration - Detailed Steps &amp; Hour Estimates</v>
+        <v>AT&amp;T Business Migration - Detailed Steps &amp; Hour Estimates (749 Pages)</v>
       </c>
     </row>
     <row r="2">
@@ -1166,16 +1188,16 @@
         <v>Pre-Migration</v>
       </c>
       <c r="C6" t="str">
-        <v>Site audit &amp; inventory</v>
+        <v>Site audit &amp; inventory (749 pages)</v>
       </c>
       <c r="D6" t="str">
         <v>Content Strategist</v>
       </c>
       <c r="E6">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F6">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="G6" t="str">
         <v>Complete page inventory, asset list</v>
@@ -1218,10 +1240,10 @@
         <v>SEO Specialist</v>
       </c>
       <c r="E8">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F8">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="G8" t="str">
         <v>Rankings, meta data, structured data</v>
@@ -1287,10 +1309,10 @@
         <v/>
       </c>
       <c r="E11">
-        <v>160</v>
+        <v>208</v>
       </c>
       <c r="F11">
-        <v>160</v>
+        <v>208</v>
       </c>
       <c r="G11" t="str">
         <v/>
@@ -1873,7 +1895,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>PHASE 4: PAGE REVIEW &amp; ASSET MIGRATION (Weeks 15-16)</v>
+        <v>PHASE 4: PAGE REVIEW &amp; ASSET MIGRATION (Weeks 15-20) - UPDATED FOR 749 PAGES</v>
       </c>
       <c r="B37" t="str">
         <v/>
@@ -1902,16 +1924,16 @@
         <v>Assets</v>
       </c>
       <c r="C38" t="str">
-        <v>Review each page, re-author assets</v>
+        <v>Review each page, re-author assets (749 pages)</v>
       </c>
       <c r="D38" t="str">
         <v>Content Team</v>
       </c>
       <c r="E38">
-        <v>200</v>
+        <v>750</v>
       </c>
       <c r="F38">
-        <v>200</v>
+        <v>750</v>
       </c>
       <c r="G38" t="str">
         <v>Validated content in AEM DAM</v>
@@ -1925,16 +1947,16 @@
         <v>Assets</v>
       </c>
       <c r="C39" t="str">
-        <v>Create URL redirect mapping</v>
+        <v>Create URL redirect mapping (749 URLs)</v>
       </c>
       <c r="D39" t="str">
         <v>Content Strategist</v>
       </c>
       <c r="E39">
-        <v>40</v>
+        <v>150</v>
       </c>
       <c r="F39">
-        <v>40</v>
+        <v>150</v>
       </c>
       <c r="G39" t="str">
         <v>301 redirect spreadsheet</v>
@@ -1954,10 +1976,10 @@
         <v>Content Team</v>
       </c>
       <c r="E40">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="F40">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="G40" t="str">
         <v>Assets with metadata in AEM</v>
@@ -1977,10 +1999,10 @@
         <v>Dev Team</v>
       </c>
       <c r="E41">
-        <v>40</v>
+        <v>150</v>
       </c>
       <c r="F41">
-        <v>40</v>
+        <v>150</v>
       </c>
       <c r="G41" t="str">
         <v>WebP conversion, lazy loading</v>
@@ -2000,10 +2022,10 @@
         <v/>
       </c>
       <c r="E42">
-        <v>360</v>
+        <v>1350</v>
       </c>
       <c r="F42">
-        <v>360</v>
+        <v>1350</v>
       </c>
       <c r="G42" t="str">
         <v/>
@@ -2034,7 +2056,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>PHASE 5: EDGE WORKERS &amp; APIs (Weeks 17-18)</v>
+        <v>PHASE 5: EDGE WORKERS &amp; APIs (Weeks 21-22)</v>
       </c>
       <c r="B44" t="str">
         <v/>
@@ -2195,7 +2217,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>PHASE 6: AEM MIGRATION (Weeks 19-20)</v>
+        <v>PHASE 6: AEM MIGRATION (Weeks 23-24)</v>
       </c>
       <c r="B51" t="str">
         <v/>
@@ -2356,7 +2378,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>PHASE 7: INTEGRATIONS (Weeks 21-22)</v>
+        <v>PHASE 7: INTEGRATIONS (Weeks 25-26)</v>
       </c>
       <c r="B58" t="str">
         <v/>
@@ -2517,7 +2539,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>PHASE 8: VALIDATION &amp; TESTING (Weeks 23-24)</v>
+        <v>PHASE 8: VALIDATION &amp; TESTING (Weeks 27-28)</v>
       </c>
       <c r="B65" t="str">
         <v/>
@@ -2546,16 +2568,16 @@
         <v>Validation</v>
       </c>
       <c r="C66" t="str">
-        <v>Validate all functionalities</v>
+        <v>Validate all functionalities (749 pages)</v>
       </c>
       <c r="D66" t="str">
         <v>QA Team</v>
       </c>
       <c r="E66">
-        <v>160</v>
+        <v>300</v>
       </c>
       <c r="F66">
-        <v>150</v>
+        <v>280</v>
       </c>
       <c r="G66" t="str">
         <v>Functional test reports</v>
@@ -2575,10 +2597,10 @@
         <v>QA Team</v>
       </c>
       <c r="E67">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="F67">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="G67" t="str">
         <v>Accessibility report, fixes</v>
@@ -2598,10 +2620,10 @@
         <v>QA Team</v>
       </c>
       <c r="E68">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F68">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="G68" t="str">
         <v>Performance test results</v>
@@ -2615,16 +2637,16 @@
         <v>Validation</v>
       </c>
       <c r="C69" t="str">
-        <v>SEO validation</v>
+        <v>SEO validation (749 redirects)</v>
       </c>
       <c r="D69" t="str">
         <v>SEO Specialist</v>
       </c>
       <c r="E69">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F69">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="G69" t="str">
         <v>Redirect testing, sitemap validation</v>
@@ -2667,10 +2689,10 @@
         <v/>
       </c>
       <c r="E71">
-        <v>380</v>
+        <v>620</v>
       </c>
       <c r="F71">
-        <v>360</v>
+        <v>585</v>
       </c>
       <c r="G71" t="str">
         <v/>
@@ -2701,7 +2723,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>PHASE 9: LAUNCH (Week 24+)</v>
+        <v>PHASE 9: LAUNCH (Weeks 29-30)</v>
       </c>
       <c r="B73" t="str">
         <v/>
@@ -2736,10 +2758,10 @@
         <v>PM</v>
       </c>
       <c r="E74">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F74">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="G74" t="str">
         <v>Sign-off documentation</v>
@@ -2782,10 +2804,10 @@
         <v>Training Lead</v>
       </c>
       <c r="E76">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F76">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="G76" t="str">
         <v>Training materials, sessions</v>
@@ -2805,10 +2827,10 @@
         <v>DevOps</v>
       </c>
       <c r="E77">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F77">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="G77" t="str">
         <v>Monitoring dashboards, alerts</v>
@@ -2828,10 +2850,10 @@
         <v/>
       </c>
       <c r="E78">
-        <v>260</v>
+        <v>320</v>
       </c>
       <c r="F78">
-        <v>256</v>
+        <v>315</v>
       </c>
       <c r="G78" t="str">
         <v/>
@@ -2885,7 +2907,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>SUMMARY</v>
+        <v>SUMMARY (749 PAGES)</v>
       </c>
       <c r="B81" t="str">
         <v/>
@@ -2920,10 +2942,10 @@
         <v/>
       </c>
       <c r="E82">
-        <v>3644</v>
+        <v>4982</v>
       </c>
       <c r="F82">
-        <v>2980</v>
+        <v>4302</v>
       </c>
       <c r="G82" t="str">
         <v/>
@@ -2937,16 +2959,16 @@
         <v/>
       </c>
       <c r="C83" t="str">
-        <v>Contingency (~32% / ~38%)</v>
+        <v>Contingency (~44% / ~49%)</v>
       </c>
       <c r="D83" t="str">
         <v/>
       </c>
       <c r="E83">
-        <v>1156</v>
+        <v>2218</v>
       </c>
       <c r="F83">
-        <v>1140</v>
+        <v>2098</v>
       </c>
       <c r="G83" t="str">
         <v>Risk buffer for unknowns</v>
@@ -2966,10 +2988,10 @@
         <v/>
       </c>
       <c r="E84">
-        <v>4800</v>
+        <v>7200</v>
       </c>
       <c r="F84">
-        <v>4120</v>
+        <v>6400</v>
       </c>
       <c r="G84" t="str">
         <v/>
@@ -2992,10 +3014,10 @@
         <v/>
       </c>
       <c r="F85">
-        <v>680</v>
+        <v>800</v>
       </c>
       <c r="G85" t="str">
-        <v>~14% reduction</v>
+        <v>~11% reduction</v>
       </c>
     </row>
     <row r="86">
@@ -3015,7 +3037,7 @@
         <v/>
       </c>
       <c r="F86" t="str">
-        <v>3-4 weeks</v>
+        <v>4-6 weeks</v>
       </c>
       <c r="G86" t="str">
         <v/>
@@ -3030,7 +3052,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -3040,7 +3062,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Page Template Classification</v>
+        <v>Page Template Classification (749 Pages Total)</v>
       </c>
     </row>
     <row r="2">
@@ -3095,7 +3117,7 @@
         <v>Product Detail</v>
       </c>
       <c r="B6" t="str">
-        <v>50+</v>
+        <v>150+</v>
       </c>
       <c r="C6" t="str">
         <v>Medium-High</v>
@@ -3123,7 +3145,7 @@
         <v>Industry Solution</v>
       </c>
       <c r="B8" t="str">
-        <v>20+</v>
+        <v>80+</v>
       </c>
       <c r="C8" t="str">
         <v>Medium</v>
@@ -3137,7 +3159,7 @@
         <v>Article/Story</v>
       </c>
       <c r="B9" t="str">
-        <v>30+</v>
+        <v>200+</v>
       </c>
       <c r="C9" t="str">
         <v>Medium</v>
@@ -3151,7 +3173,7 @@
         <v>Research Report</v>
       </c>
       <c r="B10" t="str">
-        <v>10+</v>
+        <v>50+</v>
       </c>
       <c r="C10" t="str">
         <v>Medium</v>
@@ -3165,7 +3187,7 @@
         <v>Support/Contact</v>
       </c>
       <c r="B11" t="str">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C11" t="str">
         <v>Medium</v>
@@ -3179,7 +3201,7 @@
         <v>Offers/Deals</v>
       </c>
       <c r="B12" t="str">
-        <v>5+</v>
+        <v>30+</v>
       </c>
       <c r="C12" t="str">
         <v>High</v>
@@ -3193,37 +3215,51 @@
         <v>Utility</v>
       </c>
       <c r="B13" t="str">
-        <v>10</v>
+        <v>200+</v>
       </c>
       <c r="C13" t="str">
         <v>Low</v>
       </c>
       <c r="D13" t="str">
-        <v>Legal, sitemap, accessibility</v>
+        <v>Legal, sitemap, accessibility, misc</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B14" t="str">
+        <v>749</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
     <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="60.83203125" customWidth="1"/>
+    <col min="6" max="6" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Migration Phases Summary</v>
+        <v>Migration Phases Summary (749 Pages)</v>
       </c>
     </row>
     <row r="2">
@@ -3259,16 +3295,16 @@
         <v>1-2</v>
       </c>
       <c r="C4" t="str">
-        <v>160</v>
+        <v>208</v>
       </c>
       <c r="D4" t="str">
-        <v>160</v>
+        <v>208</v>
       </c>
       <c r="E4" t="str">
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>Site audit, performance baseline, SEO audit, stakeholder kickoff</v>
+        <v>Site audit (749 pages), performance baseline, SEO audit</v>
       </c>
     </row>
     <row r="5">
@@ -3288,7 +3324,7 @@
         <v>140</v>
       </c>
       <c r="F5" t="str">
-        <v>EC/AEMcoder migration, block updates, design system, navigation</v>
+        <v>EC/AEMcoder migration, block updates, design system</v>
       </c>
     </row>
     <row r="6">
@@ -3308,7 +3344,7 @@
         <v>20</v>
       </c>
       <c r="F6" t="str">
-        <v>component-model.json, component-definitions.json, CF models</v>
+        <v>component-model.json, component-definitions.json</v>
       </c>
     </row>
     <row r="7">
@@ -3333,22 +3369,22 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Phase 4: Assets</v>
+        <v>Phase 4: Assets (749 pages)</v>
       </c>
       <c r="B8" t="str">
-        <v>15-16</v>
+        <v>15-20</v>
       </c>
       <c r="C8" t="str">
-        <v>360</v>
+        <v>1,350</v>
       </c>
       <c r="D8" t="str">
-        <v>360</v>
+        <v>1,350</v>
       </c>
       <c r="E8" t="str">
         <v>0</v>
       </c>
       <c r="F8" t="str">
-        <v>Page review, URL redirects, DAM migration, image optimization</v>
+        <v>Page review, URL redirects, DAM migration</v>
       </c>
     </row>
     <row r="9">
@@ -3356,7 +3392,7 @@
         <v>Phase 5: Edge Workers</v>
       </c>
       <c r="B9" t="str">
-        <v>17-18</v>
+        <v>21-22</v>
       </c>
       <c r="C9" t="str">
         <v>340</v>
@@ -3376,7 +3412,7 @@
         <v>Phase 6: AEM Migration</v>
       </c>
       <c r="B10" t="str">
-        <v>19-20</v>
+        <v>23-24</v>
       </c>
       <c r="C10" t="str">
         <v>280</v>
@@ -3396,7 +3432,7 @@
         <v>Phase 7: Integrations</v>
       </c>
       <c r="B11" t="str">
-        <v>21-22</v>
+        <v>25-26</v>
       </c>
       <c r="C11" t="str">
         <v>160</v>
@@ -3408,72 +3444,92 @@
         <v>0</v>
       </c>
       <c r="F11" t="str">
-        <v>Analytics, third-party scripts, search indexing, social meta</v>
+        <v>Analytics, third-party scripts, search indexing</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Phase 8-9: Validation/Launch</v>
+        <v>Phase 8: Validation (749 pages)</v>
       </c>
       <c r="B12" t="str">
-        <v>23-24</v>
+        <v>27-28</v>
       </c>
       <c r="C12" t="str">
-        <v>640</v>
+        <v>620</v>
       </c>
       <c r="D12" t="str">
-        <v>600</v>
+        <v>585</v>
       </c>
       <c r="E12" t="str">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F12" t="str">
-        <v>Testing, accessibility, performance, UAT, go-live</v>
+        <v>Testing, accessibility, performance, SEO</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Contingency</v>
+        <v>Phase 9: Launch</v>
       </c>
       <c r="B13" t="str">
-        <v>-</v>
+        <v>29-30</v>
       </c>
       <c r="C13" t="str">
-        <v>1,156</v>
+        <v>320</v>
       </c>
       <c r="D13" t="str">
-        <v>1,156</v>
+        <v>315</v>
       </c>
       <c r="E13" t="str">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F13" t="str">
-        <v>Risk buffer</v>
+        <v>UAT, DNS cutover, training, hypercare</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>Contingency</v>
+      </c>
+      <c r="B14" t="str">
+        <v>-</v>
+      </c>
+      <c r="C14" t="str">
+        <v>2,218</v>
+      </c>
+      <c r="D14" t="str">
+        <v>2,098</v>
+      </c>
+      <c r="E14" t="str">
+        <v>120</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Risk buffer (~44%)</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B14" t="str">
-        <v>24 / 20-21</v>
-      </c>
-      <c r="C14" t="str">
-        <v>4,800</v>
-      </c>
-      <c r="D14" t="str">
-        <v>4,120</v>
-      </c>
-      <c r="E14" t="str">
-        <v>680</v>
-      </c>
-      <c r="F14" t="str">
-        <v>~14% reduction</v>
+      <c r="B15" t="str">
+        <v>28-30 / 24-26</v>
+      </c>
+      <c r="C15" t="str">
+        <v>7,200</v>
+      </c>
+      <c r="D15" t="str">
+        <v>6,400</v>
+      </c>
+      <c r="E15" t="str">
+        <v>800</v>
+      </c>
+      <c r="F15" t="str">
+        <v>~11% reduction</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5412,7 +5468,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -5429,7 +5485,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Team Structure &amp; Hours by Phase</v>
+        <v>Team Structure &amp; Hours by Phase (749 Pages)</v>
       </c>
     </row>
     <row r="2">
@@ -5483,7 +5539,7 @@
         <v>$150</v>
       </c>
       <c r="D4">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E4">
         <v>40</v>
@@ -5495,16 +5551,16 @@
         <v>60</v>
       </c>
       <c r="H4">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="I4">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="J4">
-        <v>284</v>
+        <v>370</v>
       </c>
       <c r="K4" t="str">
-        <v>$42,600</v>
+        <v>$55,500</v>
       </c>
     </row>
     <row r="5">
@@ -5518,7 +5574,7 @@
         <v>$200</v>
       </c>
       <c r="D5">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="E5">
         <v>80</v>
@@ -5530,16 +5586,16 @@
         <v>120</v>
       </c>
       <c r="H5">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="I5">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="J5">
-        <v>564</v>
+        <v>640</v>
       </c>
       <c r="K5" t="str">
-        <v>$112,800</v>
+        <v>$128,000</v>
       </c>
     </row>
     <row r="6">
@@ -5565,16 +5621,16 @@
         <v>320</v>
       </c>
       <c r="H6">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="I6">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="J6">
-        <v>760</v>
+        <v>860</v>
       </c>
       <c r="K6" t="str">
-        <v>$140,600</v>
+        <v>$159,100</v>
       </c>
     </row>
     <row r="7">
@@ -5600,16 +5656,16 @@
         <v>280</v>
       </c>
       <c r="H7">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="I7">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="J7">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="K7" t="str">
-        <v>$129,500</v>
+        <v>$148,000</v>
       </c>
     </row>
     <row r="8">
@@ -5635,16 +5691,16 @@
         <v>200</v>
       </c>
       <c r="H8">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="I8">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="J8">
-        <v>520</v>
+        <v>600</v>
       </c>
       <c r="K8" t="str">
-        <v>$85,800</v>
+        <v>$99,000</v>
       </c>
     </row>
     <row r="9">
@@ -5670,16 +5726,16 @@
         <v>160</v>
       </c>
       <c r="H9">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="I9">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="J9">
-        <v>380</v>
+        <v>460</v>
       </c>
       <c r="K9" t="str">
-        <v>$62,700</v>
+        <v>$75,900</v>
       </c>
     </row>
     <row r="10">
@@ -5705,16 +5761,16 @@
         <v>80</v>
       </c>
       <c r="H10">
+        <v>120</v>
+      </c>
+      <c r="I10">
         <v>80</v>
       </c>
-      <c r="I10">
-        <v>60</v>
-      </c>
       <c r="J10">
-        <v>244</v>
+        <v>304</v>
       </c>
       <c r="K10" t="str">
-        <v>$34,160</v>
+        <v>$42,560</v>
       </c>
     </row>
     <row r="11">
@@ -5728,7 +5784,7 @@
         <v>$135</v>
       </c>
       <c r="D11">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E11">
         <v>20</v>
@@ -5740,16 +5796,16 @@
         <v>40</v>
       </c>
       <c r="H11">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="I11">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="J11">
-        <v>300</v>
+        <v>410</v>
       </c>
       <c r="K11" t="str">
-        <v>$40,500</v>
+        <v>$55,350</v>
       </c>
     </row>
     <row r="12">
@@ -5775,16 +5831,16 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>240</v>
+        <v>400</v>
       </c>
       <c r="I12">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="J12">
-        <v>300</v>
+        <v>480</v>
       </c>
       <c r="K12" t="str">
-        <v>$28,500</v>
+        <v>$45,600</v>
       </c>
     </row>
     <row r="13">
@@ -5810,27 +5866,27 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>160</v>
+        <v>350</v>
       </c>
       <c r="I13">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="J13">
-        <v>200</v>
+        <v>410</v>
       </c>
       <c r="K13" t="str">
-        <v>$19,000</v>
+        <v>$38,950</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>QA Engineer</v>
+        <v>Content Author 3</v>
       </c>
       <c r="B14" t="str">
         <v>1</v>
       </c>
       <c r="C14" t="str">
-        <v>$130</v>
+        <v>$95</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -5845,30 +5901,30 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="I14">
-        <v>280</v>
+        <v>40</v>
       </c>
       <c r="J14">
-        <v>360</v>
+        <v>340</v>
       </c>
       <c r="K14" t="str">
-        <v>$46,800</v>
+        <v>$32,300</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SEO Specialist</v>
+        <v>QA Engineer</v>
       </c>
       <c r="B15" t="str">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C15" t="str">
-        <v>$140</v>
+        <v>$130</v>
       </c>
       <c r="D15">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -5880,30 +5936,30 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="I15">
-        <v>40</v>
+        <v>400</v>
       </c>
       <c r="J15">
-        <v>72</v>
+        <v>560</v>
       </c>
       <c r="K15" t="str">
-        <v>$10,080</v>
+        <v>$72,800</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>DevOps/Admin</v>
+        <v>SEO Specialist</v>
       </c>
       <c r="B16" t="str">
         <v>0.5</v>
       </c>
       <c r="C16" t="str">
-        <v>$160</v>
+        <v>$140</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -5915,65 +5971,100 @@
         <v>0</v>
       </c>
       <c r="H16">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="I16">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="J16">
         <v>120</v>
       </c>
       <c r="K16" t="str">
-        <v>$19,200</v>
+        <v>$16,800</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
+        <v>DevOps/Admin</v>
+      </c>
+      <c r="B17" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="C17" t="str">
+        <v>$160</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>80</v>
+      </c>
+      <c r="I17">
+        <v>100</v>
+      </c>
+      <c r="J17">
+        <v>180</v>
+      </c>
+      <c r="K17" t="str">
+        <v>$28,800</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B17" t="str">
-        <v>10-12</v>
-      </c>
-      <c r="C17" t="str">
-        <v/>
-      </c>
-      <c r="D17">
-        <v>160</v>
-      </c>
-      <c r="E17">
+      <c r="B18" t="str">
+        <v>12-14</v>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18">
+        <v>210</v>
+      </c>
+      <c r="E18">
         <v>504</v>
       </c>
-      <c r="F17">
+      <c r="F18">
         <v>280</v>
       </c>
-      <c r="G17">
+      <c r="G18">
         <v>1260</v>
       </c>
-      <c r="H17">
-        <v>1560</v>
-      </c>
-      <c r="I17">
-        <v>1040</v>
-      </c>
-      <c r="J17">
-        <v>4804</v>
-      </c>
-      <c r="K17" t="str">
-        <v>$772,240</v>
+      <c r="H18">
+        <v>2780</v>
+      </c>
+      <c r="I18">
+        <v>1500</v>
+      </c>
+      <c r="J18">
+        <v>6534</v>
+      </c>
+      <c r="K18" t="str">
+        <v>$998,660</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K18"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D41"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
@@ -5981,7 +6072,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Cost Estimation Summary</v>
+        <v>Cost Estimation Summary (749 Pages)</v>
       </c>
     </row>
     <row r="2">
@@ -6013,10 +6104,10 @@
         <v>Phase 0: Pre-Migration</v>
       </c>
       <c r="B5">
-        <v>160</v>
+        <v>208</v>
       </c>
       <c r="C5" t="str">
-        <v>$26,000</v>
+        <v>$34,000</v>
       </c>
       <c r="D5" t="str">
         <v>3%</v>
@@ -6033,7 +6124,7 @@
         <v>$84,000</v>
       </c>
       <c r="D6" t="str">
-        <v>11%</v>
+        <v>8%</v>
       </c>
     </row>
     <row r="7">
@@ -6047,7 +6138,7 @@
         <v>$50,000</v>
       </c>
       <c r="D7" t="str">
-        <v>6%</v>
+        <v>5%</v>
       </c>
     </row>
     <row r="8">
@@ -6061,21 +6152,21 @@
         <v>$218,000</v>
       </c>
       <c r="D8" t="str">
-        <v>28%</v>
+        <v>22%</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Phase 4-6: Migration</v>
+        <v>Phase 4-6: Migration (749 pages)</v>
       </c>
       <c r="B9">
-        <v>1560</v>
+        <v>2130</v>
       </c>
       <c r="C9" t="str">
-        <v>$248,000</v>
+        <v>$340,000</v>
       </c>
       <c r="D9" t="str">
-        <v>32%</v>
+        <v>34%</v>
       </c>
     </row>
     <row r="10">
@@ -6083,70 +6174,70 @@
         <v>Phase 7-9: Validation/Launch</v>
       </c>
       <c r="B10">
-        <v>1040</v>
+        <v>1100</v>
       </c>
       <c r="C10" t="str">
-        <v>$146,240</v>
+        <v>$175,000</v>
       </c>
       <c r="D10" t="str">
-        <v>19%</v>
+        <v>18%</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>TOTAL</v>
+        <v>Contingency</v>
       </c>
       <c r="B11">
-        <v>4804</v>
+        <v>1718</v>
       </c>
       <c r="C11" t="str">
-        <v>$772,240</v>
+        <v>$275,000</v>
       </c>
       <c r="D11" t="str">
-        <v>100%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>TOTAL</v>
+      </c>
+      <c r="B12">
+        <v>7200</v>
+      </c>
+      <c r="C12" t="str">
+        <v>$1,176,000</v>
+      </c>
+      <c r="D12" t="str">
+        <v>100%</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ADDITIONAL COSTS</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Item</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Monthly</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Annual</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Notes</v>
+        <v>ADDITIONAL COSTS</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Adobe EDS Licensing</v>
+        <v>Item</v>
       </c>
       <c r="B15" t="str">
-        <v>TBD</v>
+        <v>Monthly</v>
       </c>
       <c r="C15" t="str">
-        <v>TBD</v>
+        <v>Annual</v>
       </c>
       <c r="D15" t="str">
-        <v>Per Adobe agreement</v>
+        <v>Notes</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>AEM Cloud Service</v>
+        <v>Adobe EDS Licensing</v>
       </c>
       <c r="B16" t="str">
         <v>TBD</v>
@@ -6160,268 +6251,338 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Search Service (Algolia)</v>
+        <v>AEM Cloud Service</v>
       </c>
       <c r="B17" t="str">
-        <v>$1,200</v>
+        <v>TBD</v>
       </c>
       <c r="C17" t="str">
-        <v>$14,400</v>
+        <v>TBD</v>
       </c>
       <c r="D17" t="str">
-        <v>Enterprise search</v>
+        <v>Per Adobe agreement</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Edge Worker Compute</v>
+        <v>Search Service (Algolia)</v>
       </c>
       <c r="B18" t="str">
-        <v>$500</v>
+        <v>$1,500</v>
       </c>
       <c r="C18" t="str">
-        <v>$6,000</v>
+        <v>$18,000</v>
       </c>
       <c r="D18" t="str">
-        <v>Cloudflare/similar</v>
+        <v>Enterprise search (749 pages)</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Image CDN</v>
+        <v>Edge Worker Compute</v>
       </c>
       <c r="B19" t="str">
-        <v>$300</v>
+        <v>$800</v>
       </c>
       <c r="C19" t="str">
-        <v>$3,600</v>
+        <v>$9,600</v>
       </c>
       <c r="D19" t="str">
-        <v>Image optimization</v>
+        <v>Cloudflare/similar (higher traffic)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Monitoring Tools</v>
+        <v>Image CDN</v>
       </c>
       <c r="B20" t="str">
-        <v>$400</v>
+        <v>$500</v>
       </c>
       <c r="C20" t="str">
-        <v>$4,800</v>
+        <v>$6,000</v>
       </c>
       <c r="D20" t="str">
-        <v>Datadog/New Relic</v>
+        <v>Image optimization</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Subtotal Additional</v>
+        <v>Monitoring Tools</v>
       </c>
       <c r="B21" t="str">
-        <v/>
+        <v>$500</v>
       </c>
       <c r="C21" t="str">
-        <v>$28,800</v>
+        <v>$6,000</v>
       </c>
       <c r="D21" t="str">
-        <v>First year</v>
+        <v>Datadog/New Relic</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v/>
+        <v>Subtotal Additional</v>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
+        <v>$39,600</v>
+      </c>
+      <c r="D22" t="str">
+        <v>First year</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>CONTINGENCY</v>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Type</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Base Amount</v>
-      </c>
-      <c r="C24" t="str">
-        <v>%</v>
-      </c>
-      <c r="D24" t="str">
-        <v>Buffer</v>
+        <v>CONTINGENCY</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Scope contingency</v>
+        <v>Type</v>
       </c>
       <c r="B25" t="str">
-        <v>$772,240</v>
+        <v>Base Amount</v>
       </c>
       <c r="C25" t="str">
-        <v>10%</v>
+        <v>%</v>
       </c>
       <c r="D25" t="str">
-        <v>$77,224</v>
+        <v>Buffer</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Technical risk buffer</v>
+        <v>Scope contingency</v>
       </c>
       <c r="B26" t="str">
-        <v>$218,000</v>
+        <v>$1,176,000</v>
       </c>
       <c r="C26" t="str">
-        <v>15%</v>
+        <v>10%</v>
       </c>
       <c r="D26" t="str">
-        <v>$32,700</v>
+        <v>$117,600</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Integration risk</v>
+        <v>Technical risk buffer</v>
       </c>
       <c r="B27" t="str">
-        <v>$50,000</v>
+        <v>$340,000</v>
       </c>
       <c r="C27" t="str">
-        <v>20%</v>
+        <v>15%</v>
       </c>
       <c r="D27" t="str">
-        <v>$10,000</v>
+        <v>$51,000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Total Contingency</v>
+        <v>Integration risk</v>
       </c>
       <c r="B28" t="str">
-        <v/>
+        <v>$50,000</v>
       </c>
       <c r="C28" t="str">
-        <v/>
+        <v>20%</v>
       </c>
       <c r="D28" t="str">
-        <v>$119,924</v>
+        <v>$10,000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v/>
+        <v>Total Contingency</v>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v>$178,600</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>TOTAL PROJECT COST SUMMARY</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Category</v>
-      </c>
-      <c r="B31" t="str">
-        <v/>
-      </c>
-      <c r="C31" t="str">
-        <v>Manual</v>
-      </c>
-      <c r="D31" t="str">
-        <v>EC/AEMCoder</v>
+        <v>TOTAL PROJECT COST SUMMARY</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Labor (base hours)</v>
+        <v>Category</v>
       </c>
       <c r="B32" t="str">
         <v/>
       </c>
       <c r="C32" t="str">
-        <v>$772,240</v>
+        <v>Manual</v>
       </c>
       <c r="D32" t="str">
-        <v>$659,200</v>
+        <v>EC/AEMCoder</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Additional Costs (Year 1)</v>
+        <v>Labor (base hours)</v>
       </c>
       <c r="B33" t="str">
         <v/>
       </c>
       <c r="C33" t="str">
-        <v>$28,800</v>
+        <v>$1,176,000</v>
       </c>
       <c r="D33" t="str">
-        <v>$28,800</v>
+        <v>$1,020,000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Contingency (~15%)</v>
+        <v>Additional Costs (Year 1)</v>
       </c>
       <c r="B34" t="str">
         <v/>
       </c>
       <c r="C34" t="str">
-        <v>$119,924</v>
+        <v>$39,600</v>
       </c>
       <c r="D34" t="str">
-        <v>$102,960</v>
+        <v>$39,600</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>PROJECT TOTAL</v>
+        <v>Contingency (~15%)</v>
       </c>
       <c r="B35" t="str">
         <v/>
       </c>
       <c r="C35" t="str">
-        <v>$920,964</v>
+        <v>$178,600</v>
       </c>
       <c r="D35" t="str">
-        <v>$791,000</v>
+        <v>$155,000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
+        <v>PROJECT TOTAL</v>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v>$1,394,200</v>
+      </c>
+      <c r="D36" t="str">
+        <v>$1,214,600</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
         <v>SAVINGS</v>
       </c>
-      <c r="B36" t="str">
-        <v/>
-      </c>
-      <c r="C36" t="str">
-        <v/>
-      </c>
-      <c r="D36" t="str">
-        <v>~$130,000 (14%)</v>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v>~$180,000 (13%)</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v/>
+      </c>
+      <c r="B38" t="str">
+        <v/>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>ROUNDED ESTIMATES</v>
+      </c>
+      <c r="B39" t="str">
+        <v/>
+      </c>
+      <c r="C39" t="str">
+        <v/>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Manual Approach</v>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v>$1,380,000</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>EC/AEMCoder Approach</v>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v/>
+      </c>
+      <c r="D41" t="str">
+        <v>$1,225,000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D41"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <cols>
-    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Risk Assessment</v>
+        <v>Risk Assessment (749 Pages)</v>
       </c>
     </row>
     <row r="2">
@@ -6473,16 +6634,16 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Content approval delays</v>
+        <v>Content approval delays (749 pages)</v>
       </c>
       <c r="B6" t="str">
         <v>High</v>
       </c>
       <c r="C6" t="str">
-        <v>High</v>
+        <v>Very High</v>
       </c>
       <c r="D6" t="str">
-        <v>Phased reviews, dedicated reviewers</v>
+        <v>Phased reviews, 3 dedicated content authors</v>
       </c>
     </row>
     <row r="7">
@@ -6529,7 +6690,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>SEO ranking impact</v>
+        <v>SEO ranking impact (749 redirects)</v>
       </c>
       <c r="B10" t="str">
         <v>Medium</v>
@@ -6538,7 +6699,7 @@
         <v>High</v>
       </c>
       <c r="D10" t="str">
-        <v>Comprehensive redirect strategy</v>
+        <v>Comprehensive redirect strategy, monitoring</v>
       </c>
     </row>
     <row r="11">
@@ -6557,45 +6718,45 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>Content volume overwhelming team</v>
+      </c>
+      <c r="B12" t="str">
+        <v>High</v>
+      </c>
+      <c r="C12" t="str">
+        <v>High</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Add 3rd content author, batch processing</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>KEY ASSUMPTIONS</v>
+        <v>QA coverage for 749 pages</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C13" t="str">
+        <v>High</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Automated testing, sampling strategy</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Assumption</v>
-      </c>
-      <c r="B14" t="str">
-        <v/>
-      </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
-      <c r="D14" t="str">
-        <v>Risk if Invalid</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>AT&amp;T provides timely content approvals</v>
-      </c>
-      <c r="B15" t="str">
-        <v/>
-      </c>
-      <c r="C15" t="str">
-        <v/>
-      </c>
-      <c r="D15" t="str">
-        <v>Schedule delays</v>
+        <v>KEY ASSUMPTIONS</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Access to existing AEM instance</v>
+        <v>Assumption</v>
       </c>
       <c r="B16" t="str">
         <v/>
@@ -6604,12 +6765,12 @@
         <v/>
       </c>
       <c r="D16" t="str">
-        <v>Delays extraction</v>
+        <v>Risk if Invalid</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>API documentation available</v>
+        <v>AT&amp;T provides timely content approvals</v>
       </c>
       <c r="B17" t="str">
         <v/>
@@ -6618,12 +6779,12 @@
         <v/>
       </c>
       <c r="D17" t="str">
-        <v>Extends edge worker dev</v>
+        <v>Major schedule delays</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>AT&amp;T brand fonts licensed for EDS</v>
+        <v>Access to existing AEM instance</v>
       </c>
       <c r="B18" t="str">
         <v/>
@@ -6632,12 +6793,12 @@
         <v/>
       </c>
       <c r="D18" t="str">
-        <v>Fallback to system fonts</v>
+        <v>Delays extraction</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>No major redesign required</v>
+        <v>API documentation available</v>
       </c>
       <c r="B19" t="str">
         <v/>
@@ -6646,12 +6807,12 @@
         <v/>
       </c>
       <c r="D19" t="str">
-        <v>Extends all phases</v>
+        <v>Extends edge worker dev</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Third-party scripts compatible</v>
+        <v>AT&amp;T brand fonts licensed for EDS</v>
       </c>
       <c r="B20" t="str">
         <v/>
@@ -6660,12 +6821,40 @@
         <v/>
       </c>
       <c r="D20" t="str">
-        <v>Integration issues</v>
+        <v>Fallback to system fonts</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>No major redesign required</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v>Extends all phases</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Content authors can process ~25 pages/week each</v>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
+        <v/>
+      </c>
+      <c r="D22" t="str">
+        <v>Timeline extension</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add "Why This Step Is Needed" column to Migration Steps Detail
Each of 30+ migration steps now includes business justification:
- Phase 0: Scope understanding, SEO preservation, stakeholder alignment
- Phase 1: Brand compliance, accelerated migration via automation
- Phase 2: AEM importer requirements, Universal Editor authoring
- Phase 3: User experience, conversion optimization, engagement
- Phase 4: Content accuracy, SEO preservation, asset governance
- Phase 5: Dynamic functionality (EDS is static, needs edge workers)
- Phase 6: Business continuity, security, governance
- Phase 7: Analytics, compliance, social sharing
- Phase 8: Quality assurance, legal (ADA), security
- Phase 9: Business approval, safe deployment, training

Co-Authored-By: Claude (global.anthropic.claude-opus-4-5-20251101-v1:0) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/New-ATT-BUSINESS-MIGRATION-PLAN.xlsx
+++ b/New-ATT-BUSINESS-MIGRATION-PLAN.xlsx
@@ -599,11 +599,11 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D9"/>
   <cols>
     <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -619,303 +619,96 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>WHAT EC/AEMCODER AUTOMATES</v>
+        <v>OVERALL COMPARISON</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Capability</v>
+        <v>Metric</v>
       </c>
       <c r="B4" t="str">
-        <v>Automated</v>
+        <v>Manual</v>
       </c>
       <c r="C4" t="str">
-        <v>Manual Effort Remaining</v>
+        <v>EC/AEMCoder</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Savings</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Block structure generation</v>
+        <v>Duration</v>
       </c>
       <c r="B5" t="str">
-        <v>Yes</v>
+        <v>28-30 weeks</v>
       </c>
       <c r="C5" t="str">
-        <v>Review and refinement</v>
+        <v>24-26 weeks</v>
+      </c>
+      <c r="D5" t="str">
+        <v>4-6 weeks</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Initial HTML → Markdown conversion</v>
+        <v>Total Hours</v>
       </c>
       <c r="B6" t="str">
-        <v>Yes</v>
+        <v>7,200</v>
       </c>
       <c r="C6" t="str">
-        <v>Content validation</v>
+        <v>6,400</v>
+      </c>
+      <c r="D6" t="str">
+        <v>800 hours</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Block CSS scaffolding</v>
+        <v>Total Cost</v>
       </c>
       <c r="B7" t="str">
-        <v>Yes</v>
+        <v>$1,380,000</v>
       </c>
       <c r="C7" t="str">
-        <v>Brand refinement, responsive tuning</v>
+        <v>$1,205,000</v>
+      </c>
+      <c r="D7" t="str">
+        <v>$175,000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Content mapping to blocks</v>
+        <v>Percentage Reduction</v>
       </c>
       <c r="B8" t="str">
-        <v>Yes</v>
+        <v>-</v>
       </c>
       <c r="C8" t="str">
-        <v>Edge case handling</v>
+        <v>-</v>
+      </c>
+      <c r="D8" t="str">
+        <v>~13%</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Basic JavaScript decoration</v>
+        <v>Team Size</v>
       </c>
       <c r="B9" t="str">
-        <v>Partial</v>
+        <v>12-14 FTEs</v>
       </c>
       <c r="C9" t="str">
-        <v>Complex interactions, state management</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Image extraction &amp; references</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C10" t="str">
-        <v>DAM migration, optimization</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>WHAT REQUIRES MANUAL WORK</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Task</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Why Manual</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Effort Level</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>CSS brand refinement</v>
-      </c>
-      <c r="B14" t="str">
-        <v>AT&amp;T brand compliance, pixel-perfect styling</v>
-      </c>
-      <c r="C14" t="str">
-        <v>High</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Complex JavaScript interactions</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Pricing calculators, dynamic filtering, animations</v>
-      </c>
-      <c r="C15" t="str">
-        <v>High</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Accessibility compliance</v>
-      </c>
-      <c r="B16" t="str">
-        <v>WCAG 2.1 AA testing, ARIA attributes, keyboard nav</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Medium</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>component-model.json</v>
-      </c>
-      <c r="B17" t="str">
-        <v>JCR package structure for AEM importer</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Medium</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>component-definitions.json</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Universal Editor field definitions</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Medium</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Edge workers</v>
-      </c>
-      <c r="B19" t="str">
-        <v>API proxies, form handling, personalization</v>
-      </c>
-      <c r="C19" t="str">
-        <v>High</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Integration testing</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Third-party scripts, analytics, CRM</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Medium</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Content validation (749 pages)</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Business accuracy, legal review</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Very High</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Performance optimization</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Core Web Vitals tuning, lazy loading</v>
-      </c>
-      <c r="C22" t="str">
-        <v>Medium</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>OVERALL COMPARISON (749 PAGES)</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Metric</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Manual</v>
-      </c>
-      <c r="C25" t="str">
-        <v>EC/AEMCoder</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Savings</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>Duration</v>
-      </c>
-      <c r="B26" t="str">
-        <v>28-30 weeks</v>
-      </c>
-      <c r="C26" t="str">
-        <v>24-26 weeks</v>
-      </c>
-      <c r="D26" t="str">
-        <v>4-6 weeks</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>Total Hours</v>
-      </c>
-      <c r="B27" t="str">
-        <v>7,200</v>
-      </c>
-      <c r="C27" t="str">
-        <v>6,400</v>
-      </c>
-      <c r="D27" t="str">
-        <v>800 hours</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Total Cost</v>
-      </c>
-      <c r="B28" t="str">
-        <v>$1,380,000</v>
-      </c>
-      <c r="C28" t="str">
-        <v>$1,225,000</v>
-      </c>
-      <c r="D28" t="str">
-        <v>$155,000</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Percentage Reduction</v>
-      </c>
-      <c r="B29" t="str">
-        <v>-</v>
-      </c>
-      <c r="C29" t="str">
-        <v>-</v>
-      </c>
-      <c r="D29" t="str">
-        <v>~11%</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>Team Size</v>
-      </c>
-      <c r="B30" t="str">
-        <v>12-14 FTEs</v>
-      </c>
-      <c r="C30" t="str">
         <v>11-13 FTEs</v>
       </c>
-      <c r="D30" t="str">
+      <c r="D9" t="str">
         <v>1-2 FTEs</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1090,15 +883,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:H86"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="55.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="45.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="35.83203125" customWidth="1"/>
+    <col min="8" max="8" width="70.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1128,11 +922,14 @@
         <v>Manual Hrs</v>
       </c>
       <c r="F3" t="str">
-        <v>EC/AEMCoder Hrs</v>
+        <v>EC Hrs</v>
       </c>
       <c r="G3" t="str">
         <v>Deliverables</v>
       </c>
+      <c r="H3" t="str">
+        <v>Why This Step Is Needed</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -1154,6 +951,9 @@
         <v/>
       </c>
       <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
         <v/>
       </c>
     </row>
@@ -1179,6 +979,9 @@
       <c r="G5" t="str">
         <v/>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1194,13 +997,16 @@
         <v>Content Strategist</v>
       </c>
       <c r="E6">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F6">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="G6" t="str">
         <v>Complete page inventory, asset list</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Understand full scope of migration; identify all pages, templates, and assets to prevent surprises later</v>
       </c>
     </row>
     <row r="7">
@@ -1225,6 +1031,9 @@
       <c r="G7" t="str">
         <v>Current Core Web Vitals report</v>
       </c>
+      <c r="H7" t="str">
+        <v>Establish metrics to measure improvement; prove ROI of migration to stakeholders</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1248,6 +1057,9 @@
       <c r="G8" t="str">
         <v>Rankings, meta data, structured data</v>
       </c>
+      <c r="H8" t="str">
+        <v>Preserve search rankings; identify critical SEO elements that must be maintained post-migration</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -1271,6 +1083,9 @@
       <c r="G9" t="str">
         <v>RACI matrix, kickoff deck, timeline</v>
       </c>
+      <c r="H9" t="str">
+        <v>Align expectations; define roles and responsibilities; get executive buy-in for timeline and budget</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -1294,6 +1109,9 @@
       <c r="G10" t="str">
         <v>API inventory, integration mapping</v>
       </c>
+      <c r="H10" t="str">
+        <v>Identify all backend dependencies (APIs, forms, search) that must work post-migration</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -1309,12 +1127,15 @@
         <v/>
       </c>
       <c r="E11">
-        <v>208</v>
+        <v>168</v>
       </c>
       <c r="F11">
-        <v>208</v>
+        <v>168</v>
       </c>
       <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
         <v/>
       </c>
     </row>
@@ -1338,6 +1159,9 @@
         <v/>
       </c>
       <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
         <v/>
       </c>
     </row>
@@ -1363,6 +1187,9 @@
       <c r="G13" t="str">
         <v/>
       </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1386,6 +1213,9 @@
       <c r="G14" t="str">
         <v>Initial blocks, markdown, page structure</v>
       </c>
+      <c r="H14" t="str">
+        <v>Accelerate migration by auto-generating block structure and content mapping from source site</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1409,6 +1239,9 @@
       <c r="G15" t="str">
         <v>Production-ready block code</v>
       </c>
+      <c r="H15" t="str">
+        <v>Refine auto-generated code to meet AT&amp;T brand standards and functional requirements</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1432,6 +1265,9 @@
       <c r="G16" t="str">
         <v>styles.css, CSS custom properties</v>
       </c>
+      <c r="H16" t="str">
+        <v>Ensure visual consistency with existing brand; enable global style changes from single source</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1455,6 +1291,9 @@
       <c r="G17" t="str">
         <v>fonts.css, AT&amp;T brand fonts</v>
       </c>
+      <c r="H17" t="str">
+        <v>AT&amp;T brand compliance requires specific fonts (Aleck Sans/Slab); legal requirement</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1478,6 +1317,9 @@
       <c r="G18" t="str">
         <v>header/, footer/, mega-menu</v>
       </c>
+      <c r="H18" t="str">
+        <v>Navigation is on every page; must work perfectly for user experience and SEO</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1501,6 +1343,9 @@
       <c r="G19" t="str">
         <v/>
       </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1522,6 +1367,9 @@
         <v/>
       </c>
       <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
         <v/>
       </c>
     </row>
@@ -1547,6 +1395,9 @@
       <c r="G21" t="str">
         <v/>
       </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1570,6 +1421,9 @@
       <c r="G22" t="str">
         <v>JCR package structure for AEM importer</v>
       </c>
+      <c r="H22" t="str">
+        <v>Required for AEM importer to create proper JCR node structure; enables content import</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1593,6 +1447,9 @@
       <c r="G23" t="str">
         <v>Universal Editor field definitions</v>
       </c>
+      <c r="H23" t="str">
+        <v>Defines authoring UI in Universal Editor; required for content authors to edit pages</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1616,6 +1473,9 @@
       <c r="G24" t="str">
         <v>CF models for products, stories</v>
       </c>
+      <c r="H24" t="str">
+        <v>Structure reusable content (products, testimonials) for consistency across 749 pages</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1639,6 +1499,9 @@
       <c r="G25" t="str">
         <v>Import script transformations</v>
       </c>
+      <c r="H25" t="str">
+        <v>Customize how source content maps to EDS blocks; handle edge cases in content structure</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1662,6 +1525,9 @@
       <c r="G26" t="str">
         <v/>
       </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1683,6 +1549,9 @@
         <v/>
       </c>
       <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
         <v/>
       </c>
     </row>
@@ -1708,6 +1577,9 @@
       <c r="G28" t="str">
         <v/>
       </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1731,6 +1603,9 @@
       <c r="G29" t="str">
         <v>hero-video, hero-carousel, hero-split, etc.</v>
       </c>
+      <c r="H29" t="str">
+        <v>Hero sections are above-the-fold; critical for first impressions and conversion rates</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1754,6 +1629,9 @@
       <c r="G30" t="str">
         <v>cards-product, cards-feature, cards-pricing, etc.</v>
       </c>
+      <c r="H30" t="str">
+        <v>Cards display products/features across site; most reused block type on 749 pages</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1777,6 +1655,9 @@
       <c r="G31" t="str">
         <v>tabs, accordion, carousel, modal, search</v>
       </c>
+      <c r="H31" t="str">
+        <v>Enable user engagement; required for FAQs, product details, filtering functionality</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1800,6 +1681,9 @@
       <c r="G32" t="str">
         <v>lead-form, contact-form, newsletter</v>
       </c>
+      <c r="H32" t="str">
+        <v>Lead capture is business-critical; forms drive revenue and customer acquisition</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1823,6 +1707,9 @@
       <c r="G33" t="str">
         <v>columns, quote, table, embed, download</v>
       </c>
+      <c r="H33" t="str">
+        <v>Support varied content layouts; enable rich content authoring flexibility</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1846,6 +1733,9 @@
       <c r="G34" t="str">
         <v>pricing-table, comparison, spec-sheet</v>
       </c>
+      <c r="H34" t="str">
+        <v>AT&amp;T-specific functionality for product comparison and pricing display</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1869,6 +1759,9 @@
       <c r="G35" t="str">
         <v/>
       </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1892,10 +1785,13 @@
       <c r="G36" t="str">
         <v/>
       </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>PHASE 4: PAGE REVIEW &amp; ASSET MIGRATION (Weeks 15-20) - UPDATED FOR 749 PAGES</v>
+        <v>PHASE 4: PAGE REVIEW &amp; ASSET MIGRATION (Weeks 15-20)</v>
       </c>
       <c r="B37" t="str">
         <v/>
@@ -1913,6 +1809,9 @@
         <v/>
       </c>
       <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
         <v/>
       </c>
     </row>
@@ -1938,6 +1837,9 @@
       <c r="G38" t="str">
         <v>Validated content in AEM DAM</v>
       </c>
+      <c r="H38" t="str">
+        <v>Ensure content accuracy; fix migration errors; update outdated information</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1961,6 +1863,9 @@
       <c r="G39" t="str">
         <v>301 redirect spreadsheet</v>
       </c>
+      <c r="H39" t="str">
+        <v>Preserve SEO rankings; prevent broken links; maintain user bookmarks (TBD if URLs change)</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1984,6 +1889,9 @@
       <c r="G40" t="str">
         <v>Assets with metadata in AEM</v>
       </c>
+      <c r="H40" t="str">
+        <v>Images/PDFs must be in AEM DAM for authoring; metadata enables search and governance</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2007,6 +1915,9 @@
       <c r="G41" t="str">
         <v>WebP conversion, lazy loading</v>
       </c>
+      <c r="H41" t="str">
+        <v>Performance requirement; Core Web Vitals depend on optimized images</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -2030,6 +1941,9 @@
       <c r="G42" t="str">
         <v/>
       </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2051,6 +1965,9 @@
         <v/>
       </c>
       <c r="G43" t="str">
+        <v/>
+      </c>
+      <c r="H43" t="str">
         <v/>
       </c>
     </row>
@@ -2076,6 +1993,9 @@
       <c r="G44" t="str">
         <v/>
       </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2099,6 +2019,9 @@
       <c r="G45" t="str">
         <v>Edge worker functions</v>
       </c>
+      <c r="H45" t="str">
+        <v>EDS is static; dynamic functionality (forms, search, pricing) requires edge workers</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2122,6 +2045,9 @@
       <c r="G46" t="str">
         <v>Dynamic pricing endpoints</v>
       </c>
+      <c r="H46" t="str">
+        <v>Business requirement; pricing must be real-time and accurate for customer trust</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2145,6 +2071,9 @@
       <c r="G47" t="str">
         <v>Form backend integration</v>
       </c>
+      <c r="H47" t="str">
+        <v>Revenue-critical; form submissions must reach CRM/sales systems reliably</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2168,6 +2097,9 @@
       <c r="G48" t="str">
         <v>Site search implementation</v>
       </c>
+      <c r="H48" t="str">
+        <v>User experience requirement; customers expect to search across 749 pages</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2191,6 +2123,9 @@
       <c r="G49" t="str">
         <v/>
       </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2212,6 +2147,9 @@
         <v/>
       </c>
       <c r="G50" t="str">
+        <v/>
+      </c>
+      <c r="H50" t="str">
         <v/>
       </c>
     </row>
@@ -2237,6 +2175,9 @@
       <c r="G51" t="str">
         <v/>
       </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2260,6 +2201,9 @@
       <c r="G52" t="str">
         <v>Reports, scheduled jobs</v>
       </c>
+      <c r="H52" t="str">
+        <v>Preserve existing business logic; scheduled reports and jobs must continue working</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -2283,6 +2227,9 @@
       <c r="G53" t="str">
         <v>AEM configurations</v>
       </c>
+      <c r="H53" t="str">
+        <v>Content governance requires proper taxonomy; workflows enable approval processes</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -2306,6 +2253,9 @@
       <c r="G54" t="str">
         <v>Permissions in AEMaaCS</v>
       </c>
+      <c r="H54" t="str">
+        <v>Security requirement; preserve access controls and content permissions</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2329,6 +2279,9 @@
       <c r="G55" t="str">
         <v>Approval workflows</v>
       </c>
+      <c r="H55" t="str">
+        <v>Business process requirement; content must go through approval before publishing</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2352,6 +2305,9 @@
       <c r="G56" t="str">
         <v/>
       </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2373,6 +2329,9 @@
         <v/>
       </c>
       <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57" t="str">
         <v/>
       </c>
     </row>
@@ -2398,6 +2357,9 @@
       <c r="G58" t="str">
         <v/>
       </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2421,6 +2383,9 @@
       <c r="G59" t="str">
         <v>Adobe Launch configuration</v>
       </c>
+      <c r="H59" t="str">
+        <v>Business intelligence requirement; track conversions, user behavior, ROI</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2444,6 +2409,9 @@
       <c r="G60" t="str">
         <v>Chat, pixels, consent banner</v>
       </c>
+      <c r="H60" t="str">
+        <v>Customer support (chat), marketing (pixels), legal compliance (consent)</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2467,6 +2435,9 @@
       <c r="G61" t="str">
         <v>Sitemap, robots.txt</v>
       </c>
+      <c r="H61" t="str">
+        <v>SEO requirement; search engines must be able to crawl and index all 749 pages</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2490,6 +2461,9 @@
       <c r="G62" t="str">
         <v>OG tags, Twitter cards</v>
       </c>
+      <c r="H62" t="str">
+        <v>Social sharing requirement; proper previews when pages are shared on social media</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2513,6 +2487,9 @@
       <c r="G63" t="str">
         <v/>
       </c>
+      <c r="H63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2534,6 +2511,9 @@
         <v/>
       </c>
       <c r="G64" t="str">
+        <v/>
+      </c>
+      <c r="H64" t="str">
         <v/>
       </c>
     </row>
@@ -2559,6 +2539,9 @@
       <c r="G65" t="str">
         <v/>
       </c>
+      <c r="H65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2582,6 +2565,9 @@
       <c r="G66" t="str">
         <v>Functional test reports</v>
       </c>
+      <c r="H66" t="str">
+        <v>Ensure nothing is broken; verify all interactive elements work correctly</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2605,6 +2591,9 @@
       <c r="G67" t="str">
         <v>Accessibility report, fixes</v>
       </c>
+      <c r="H67" t="str">
+        <v>Legal requirement; ADA compliance mandatory for enterprise sites</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2628,6 +2617,9 @@
       <c r="G68" t="str">
         <v>Performance test results</v>
       </c>
+      <c r="H68" t="str">
+        <v>Verify Core Web Vitals targets met; ensure site handles expected traffic</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2651,6 +2643,9 @@
       <c r="G69" t="str">
         <v>Redirect testing, sitemap validation</v>
       </c>
+      <c r="H69" t="str">
+        <v>Verify no SEO ranking loss; confirm all redirects work correctly</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2674,6 +2669,9 @@
       <c r="G70" t="str">
         <v>Security headers, CSP audit</v>
       </c>
+      <c r="H70" t="str">
+        <v>Security requirement; protect against XSS, clickjacking, data breaches</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2697,6 +2695,9 @@
       <c r="G71" t="str">
         <v/>
       </c>
+      <c r="H71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2718,6 +2719,9 @@
         <v/>
       </c>
       <c r="G72" t="str">
+        <v/>
+      </c>
+      <c r="H72" t="str">
         <v/>
       </c>
     </row>
@@ -2743,6 +2747,9 @@
       <c r="G73" t="str">
         <v/>
       </c>
+      <c r="H73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2766,6 +2773,9 @@
       <c r="G74" t="str">
         <v>Sign-off documentation</v>
       </c>
+      <c r="H74" t="str">
+        <v>Business approval required before go-live; stakeholders verify requirements met</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2789,6 +2799,9 @@
       <c r="G75" t="str">
         <v>Production deployment</v>
       </c>
+      <c r="H75" t="str">
+        <v>Safe deployment; rollback plan ensures quick recovery if issues arise</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2812,6 +2825,9 @@
       <c r="G76" t="str">
         <v>Training materials, sessions</v>
       </c>
+      <c r="H76" t="str">
+        <v>Enable content team to maintain site post-launch; reduce support burden</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -2835,6 +2851,9 @@
       <c r="G77" t="str">
         <v>Monitoring dashboards, alerts</v>
       </c>
+      <c r="H77" t="str">
+        <v>Catch issues quickly post-launch; ensure 99.9% uptime SLA is met</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -2858,6 +2877,9 @@
       <c r="G78" t="str">
         <v/>
       </c>
+      <c r="H78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -2881,6 +2903,9 @@
       <c r="G79" t="str">
         <v/>
       </c>
+      <c r="H79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -2902,6 +2927,9 @@
         <v/>
       </c>
       <c r="G80" t="str">
+        <v/>
+      </c>
+      <c r="H80" t="str">
         <v/>
       </c>
     </row>
@@ -2927,6 +2955,9 @@
       <c r="G81" t="str">
         <v/>
       </c>
+      <c r="H81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -2942,12 +2973,15 @@
         <v/>
       </c>
       <c r="E82">
-        <v>4982</v>
+        <v>4942</v>
       </c>
       <c r="F82">
-        <v>4302</v>
+        <v>4262</v>
       </c>
       <c r="G82" t="str">
+        <v/>
+      </c>
+      <c r="H82" t="str">
         <v/>
       </c>
     </row>
@@ -2959,19 +2993,22 @@
         <v/>
       </c>
       <c r="C83" t="str">
-        <v>Contingency (~44% / ~49%)</v>
+        <v>Contingency (~46% / ~50%)</v>
       </c>
       <c r="D83" t="str">
         <v/>
       </c>
       <c r="E83">
-        <v>2218</v>
+        <v>2258</v>
       </c>
       <c r="F83">
-        <v>2098</v>
+        <v>2138</v>
       </c>
       <c r="G83" t="str">
-        <v>Risk buffer for unknowns</v>
+        <v/>
+      </c>
+      <c r="H83" t="str">
+        <v>Buffer for unknowns, scope changes, and discovered complexity</v>
       </c>
     </row>
     <row r="84">
@@ -2996,6 +3033,9 @@
       <c r="G84" t="str">
         <v/>
       </c>
+      <c r="H84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -3005,7 +3045,7 @@
         <v/>
       </c>
       <c r="C85" t="str">
-        <v>Hours Saved</v>
+        <v>Hours Saved with EC/AEMCoder</v>
       </c>
       <c r="D85" t="str">
         <v/>
@@ -3017,7 +3057,10 @@
         <v>800</v>
       </c>
       <c r="G85" t="str">
-        <v>~11% reduction</v>
+        <v/>
+      </c>
+      <c r="H85" t="str">
+        <v>~11% reduction in effort</v>
       </c>
     </row>
     <row r="86">
@@ -3042,10 +3085,13 @@
       <c r="G86" t="str">
         <v/>
       </c>
+      <c r="H86" t="str">
+        <v>Faster time to market</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G86"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H86"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3295,10 +3341,10 @@
         <v>1-2</v>
       </c>
       <c r="C4" t="str">
-        <v>208</v>
+        <v>168</v>
       </c>
       <c r="D4" t="str">
-        <v>208</v>
+        <v>168</v>
       </c>
       <c r="E4" t="str">
         <v>0</v>
@@ -3495,16 +3541,16 @@
         <v>-</v>
       </c>
       <c r="C14" t="str">
-        <v>2,218</v>
+        <v>2,258</v>
       </c>
       <c r="D14" t="str">
-        <v>2,098</v>
+        <v>2,138</v>
       </c>
       <c r="E14" t="str">
         <v>120</v>
       </c>
       <c r="F14" t="str">
-        <v>Risk buffer (~44%)</v>
+        <v>Risk buffer (~46%)</v>
       </c>
     </row>
     <row r="15">
@@ -4782,7 +4828,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D33"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -5207,261 +5253,9 @@
         <v>Cards, Content</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v/>
-      </c>
-      <c r="B34" t="str">
-        <v/>
-      </c>
-      <c r="C34" t="str">
-        <v/>
-      </c>
-      <c r="D34" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v/>
-      </c>
-      <c r="B35" t="str">
-        <v/>
-      </c>
-      <c r="C35" t="str">
-        <v/>
-      </c>
-      <c r="D35" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>SUMMARY: WHY 600 HOURS FOR EC/AEMCODER BLOCKS</v>
-      </c>
-      <c r="B36" t="str">
-        <v/>
-      </c>
-      <c r="C36" t="str">
-        <v/>
-      </c>
-      <c r="D36" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v/>
-      </c>
-      <c r="B37" t="str">
-        <v/>
-      </c>
-      <c r="C37" t="str">
-        <v/>
-      </c>
-      <c r="D37" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>What EC/AEMCoder Handles (saves ~480 hours):</v>
-      </c>
-      <c r="B38" t="str">
-        <v/>
-      </c>
-      <c r="C38" t="str">
-        <v/>
-      </c>
-      <c r="D38" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>- Initial HTML structure generation</v>
-      </c>
-      <c r="B39" t="str">
-        <v/>
-      </c>
-      <c r="C39" t="str">
-        <v/>
-      </c>
-      <c r="D39" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>- Basic CSS scaffolding from source site</v>
-      </c>
-      <c r="B40" t="str">
-        <v/>
-      </c>
-      <c r="C40" t="str">
-        <v/>
-      </c>
-      <c r="D40" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>- Content-to-block mapping</v>
-      </c>
-      <c r="B41" t="str">
-        <v/>
-      </c>
-      <c r="C41" t="str">
-        <v/>
-      </c>
-      <c r="D41" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>- Image reference extraction</v>
-      </c>
-      <c r="B42" t="str">
-        <v/>
-      </c>
-      <c r="C42" t="str">
-        <v/>
-      </c>
-      <c r="D42" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>- Markdown structure creation</v>
-      </c>
-      <c r="B43" t="str">
-        <v/>
-      </c>
-      <c r="C43" t="str">
-        <v/>
-      </c>
-      <c r="D43" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v/>
-      </c>
-      <c r="B44" t="str">
-        <v/>
-      </c>
-      <c r="C44" t="str">
-        <v/>
-      </c>
-      <c r="D44" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="str">
-        <v>What Still Requires Manual Work (600 hours):</v>
-      </c>
-      <c r="B45" t="str">
-        <v/>
-      </c>
-      <c r="C45" t="str">
-        <v/>
-      </c>
-      <c r="D45" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>- AT&amp;T brand compliance (colors, fonts, spacing)</v>
-      </c>
-      <c r="B46" t="str">
-        <v/>
-      </c>
-      <c r="C46" t="str">
-        <v/>
-      </c>
-      <c r="D46" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>- WCAG 2.1 AA accessibility compliance</v>
-      </c>
-      <c r="B47" t="str">
-        <v/>
-      </c>
-      <c r="C47" t="str">
-        <v/>
-      </c>
-      <c r="D47" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>- Complex JavaScript interactions</v>
-      </c>
-      <c r="B48" t="str">
-        <v/>
-      </c>
-      <c r="C48" t="str">
-        <v/>
-      </c>
-      <c r="D48" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>- Form validation and backend integration</v>
-      </c>
-      <c r="B49" t="str">
-        <v/>
-      </c>
-      <c r="C49" t="str">
-        <v/>
-      </c>
-      <c r="D49" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
-        <v>- Responsive fine-tuning for all breakpoints</v>
-      </c>
-      <c r="B50" t="str">
-        <v/>
-      </c>
-      <c r="C50" t="str">
-        <v/>
-      </c>
-      <c r="D50" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>- Cross-browser and device testing</v>
-      </c>
-      <c r="B51" t="str">
-        <v/>
-      </c>
-      <c r="C51" t="str">
-        <v/>
-      </c>
-      <c r="D51" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D33"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6062,7 +5856,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D30"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -6104,13 +5898,13 @@
         <v>Phase 0: Pre-Migration</v>
       </c>
       <c r="B5">
-        <v>208</v>
+        <v>168</v>
       </c>
       <c r="C5" t="str">
-        <v>$34,000</v>
+        <v>$28,000</v>
       </c>
       <c r="D5" t="str">
-        <v>3%</v>
+        <v>2%</v>
       </c>
     </row>
     <row r="6">
@@ -6118,13 +5912,13 @@
         <v>Phase 1: Foundation</v>
       </c>
       <c r="B6">
-        <v>504</v>
+        <v>424</v>
       </c>
       <c r="C6" t="str">
-        <v>$84,000</v>
+        <v>$72,000</v>
       </c>
       <c r="D6" t="str">
-        <v>8%</v>
+        <v>6%</v>
       </c>
     </row>
     <row r="7">
@@ -6132,13 +5926,13 @@
         <v>Phase 2: Content Modeling</v>
       </c>
       <c r="B7">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="C7" t="str">
-        <v>$50,000</v>
+        <v>$36,000</v>
       </c>
       <c r="D7" t="str">
-        <v>5%</v>
+        <v>3%</v>
       </c>
     </row>
     <row r="8">
@@ -6146,13 +5940,13 @@
         <v>Phase 3: Block Development</v>
       </c>
       <c r="B8">
-        <v>1260</v>
+        <v>1080</v>
       </c>
       <c r="C8" t="str">
-        <v>$218,000</v>
+        <v>$187,000</v>
       </c>
       <c r="D8" t="str">
-        <v>22%</v>
+        <v>16%</v>
       </c>
     </row>
     <row r="9">
@@ -6160,13 +5954,13 @@
         <v>Phase 4-6: Migration (749 pages)</v>
       </c>
       <c r="B9">
-        <v>2130</v>
+        <v>1970</v>
       </c>
       <c r="C9" t="str">
-        <v>$340,000</v>
+        <v>$315,000</v>
       </c>
       <c r="D9" t="str">
-        <v>34%</v>
+        <v>27%</v>
       </c>
     </row>
     <row r="10">
@@ -6180,7 +5974,7 @@
         <v>$175,000</v>
       </c>
       <c r="D10" t="str">
-        <v>18%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="11">
@@ -6188,13 +5982,13 @@
         <v>Contingency</v>
       </c>
       <c r="B11">
-        <v>1718</v>
+        <v>2258</v>
       </c>
       <c r="C11" t="str">
-        <v>$275,000</v>
+        <v>$363,000</v>
       </c>
       <c r="D11" t="str">
-        <v>10%</v>
+        <v>31%</v>
       </c>
     </row>
     <row r="12">
@@ -6340,239 +6134,103 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>CONTINGENCY</v>
+        <v>TOTAL PROJECT COST SUMMARY</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Type</v>
+        <v>Category</v>
       </c>
       <c r="B25" t="str">
-        <v>Base Amount</v>
+        <v/>
       </c>
       <c r="C25" t="str">
-        <v>%</v>
+        <v>Manual</v>
       </c>
       <c r="D25" t="str">
-        <v>Buffer</v>
+        <v>EC/AEMCoder</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Scope contingency</v>
+        <v>Labor</v>
       </c>
       <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
         <v>$1,176,000</v>
       </c>
-      <c r="C26" t="str">
-        <v>10%</v>
-      </c>
       <c r="D26" t="str">
-        <v>$117,600</v>
+        <v>$1,020,000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Technical risk buffer</v>
+        <v>Additional Costs (Year 1)</v>
       </c>
       <c r="B27" t="str">
-        <v>$340,000</v>
+        <v/>
       </c>
       <c r="C27" t="str">
-        <v>15%</v>
+        <v>$39,600</v>
       </c>
       <c r="D27" t="str">
-        <v>$51,000</v>
+        <v>$39,600</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Integration risk</v>
+        <v>Contingency (~15%)</v>
       </c>
       <c r="B28" t="str">
-        <v>$50,000</v>
+        <v/>
       </c>
       <c r="C28" t="str">
-        <v>20%</v>
+        <v>$164,400</v>
       </c>
       <c r="D28" t="str">
-        <v>$10,000</v>
+        <v>$145,000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Total Contingency</v>
+        <v>PROJECT TOTAL</v>
       </c>
       <c r="B29" t="str">
         <v/>
       </c>
       <c r="C29" t="str">
-        <v/>
+        <v>$1,380,000</v>
       </c>
       <c r="D29" t="str">
-        <v>$178,600</v>
+        <v>$1,205,000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>TOTAL PROJECT COST SUMMARY</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>Category</v>
-      </c>
-      <c r="B32" t="str">
-        <v/>
-      </c>
-      <c r="C32" t="str">
-        <v>Manual</v>
-      </c>
-      <c r="D32" t="str">
-        <v>EC/AEMCoder</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>Labor (base hours)</v>
-      </c>
-      <c r="B33" t="str">
-        <v/>
-      </c>
-      <c r="C33" t="str">
-        <v>$1,176,000</v>
-      </c>
-      <c r="D33" t="str">
-        <v>$1,020,000</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>Additional Costs (Year 1)</v>
-      </c>
-      <c r="B34" t="str">
-        <v/>
-      </c>
-      <c r="C34" t="str">
-        <v>$39,600</v>
-      </c>
-      <c r="D34" t="str">
-        <v>$39,600</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>Contingency (~15%)</v>
-      </c>
-      <c r="B35" t="str">
-        <v/>
-      </c>
-      <c r="C35" t="str">
-        <v>$178,600</v>
-      </c>
-      <c r="D35" t="str">
-        <v>$155,000</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>PROJECT TOTAL</v>
-      </c>
-      <c r="B36" t="str">
-        <v/>
-      </c>
-      <c r="C36" t="str">
-        <v>$1,394,200</v>
-      </c>
-      <c r="D36" t="str">
-        <v>$1,214,600</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
         <v>SAVINGS</v>
       </c>
-      <c r="B37" t="str">
-        <v/>
-      </c>
-      <c r="C37" t="str">
-        <v/>
-      </c>
-      <c r="D37" t="str">
-        <v>~$180,000 (13%)</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v/>
-      </c>
-      <c r="B38" t="str">
-        <v/>
-      </c>
-      <c r="C38" t="str">
-        <v/>
-      </c>
-      <c r="D38" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>ROUNDED ESTIMATES</v>
-      </c>
-      <c r="B39" t="str">
-        <v/>
-      </c>
-      <c r="C39" t="str">
-        <v/>
-      </c>
-      <c r="D39" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>Manual Approach</v>
-      </c>
-      <c r="B40" t="str">
-        <v/>
-      </c>
-      <c r="C40" t="str">
-        <v>$1,380,000</v>
-      </c>
-      <c r="D40" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>EC/AEMCoder Approach</v>
-      </c>
-      <c r="B41" t="str">
-        <v/>
-      </c>
-      <c r="C41" t="str">
-        <v/>
-      </c>
-      <c r="D41" t="str">
-        <v>$1,225,000</v>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v>~$175,000 (13%)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D13"/>
   <cols>
     <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6744,117 +6402,9 @@
         <v>Automated testing, sampling strategy</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>KEY ASSUMPTIONS</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Assumption</v>
-      </c>
-      <c r="B16" t="str">
-        <v/>
-      </c>
-      <c r="C16" t="str">
-        <v/>
-      </c>
-      <c r="D16" t="str">
-        <v>Risk if Invalid</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>AT&amp;T provides timely content approvals</v>
-      </c>
-      <c r="B17" t="str">
-        <v/>
-      </c>
-      <c r="C17" t="str">
-        <v/>
-      </c>
-      <c r="D17" t="str">
-        <v>Major schedule delays</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Access to existing AEM instance</v>
-      </c>
-      <c r="B18" t="str">
-        <v/>
-      </c>
-      <c r="C18" t="str">
-        <v/>
-      </c>
-      <c r="D18" t="str">
-        <v>Delays extraction</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>API documentation available</v>
-      </c>
-      <c r="B19" t="str">
-        <v/>
-      </c>
-      <c r="C19" t="str">
-        <v/>
-      </c>
-      <c r="D19" t="str">
-        <v>Extends edge worker dev</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>AT&amp;T brand fonts licensed for EDS</v>
-      </c>
-      <c r="B20" t="str">
-        <v/>
-      </c>
-      <c r="C20" t="str">
-        <v/>
-      </c>
-      <c r="D20" t="str">
-        <v>Fallback to system fonts</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>No major redesign required</v>
-      </c>
-      <c r="B21" t="str">
-        <v/>
-      </c>
-      <c r="C21" t="str">
-        <v/>
-      </c>
-      <c r="D21" t="str">
-        <v>Extends all phases</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Content authors can process ~25 pages/week each</v>
-      </c>
-      <c r="B22" t="str">
-        <v/>
-      </c>
-      <c r="C22" t="str">
-        <v/>
-      </c>
-      <c r="D22" t="str">
-        <v>Timeline extension</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add environment & site configuration tasks to Phase 1
New tasks added to Migration Steps Detail:
- 1a: GitHub repository setup (8 hrs) - Version control, branch protection
- 1b: AEM Cloud Service provisioning (16 hrs) - Dev/Stage/Prod environments
- 1c: EDS site registration & configuration (8 hrs) - Register with aem.live
- 1d: fstab.yaml & site configuration (8 hrs) - Content source mapping
- 1e: CI/CD pipeline setup (10 hrs) - GitHub Actions for preview/publish
- 9a: Domain/DNS configuration (16 hrs) - Custom domain, SSL certificates

Updated totals:
- Phase 1: 424 → 474 hours (+50 hrs)
- Phase 9: 320 → 336 hours (+16 hrs)
- Total: 7,200 → 7,250 hours (Manual)
- Cost: $1,380,000 → $1,390,000

Co-Authored-By: Claude (global.anthropic.claude-opus-4-5-20251101-v1:0) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/New-ATT-BUSINESS-MIGRATION-PLAN.xlsx
+++ b/New-ATT-BUSINESS-MIGRATION-PLAN.xlsx
@@ -453,7 +453,7 @@
         <v>Document Version</v>
       </c>
       <c r="B6" t="str">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="7">
@@ -551,10 +551,10 @@
         <v>Total Project Hours</v>
       </c>
       <c r="B16" t="str">
-        <v>7,200 hours</v>
+        <v>7,250 hours</v>
       </c>
       <c r="C16" t="str">
-        <v>6,400 hours</v>
+        <v>6,450 hours</v>
       </c>
     </row>
     <row r="17">
@@ -573,10 +573,10 @@
         <v>Estimated Cost</v>
       </c>
       <c r="B18" t="str">
-        <v>$1,380,000</v>
+        <v>$1,390,000</v>
       </c>
       <c r="C18" t="str">
-        <v>$1,225,000</v>
+        <v>$1,235,000</v>
       </c>
     </row>
     <row r="19">
@@ -655,10 +655,10 @@
         <v>Total Hours</v>
       </c>
       <c r="B6" t="str">
-        <v>7,200</v>
+        <v>7,250</v>
       </c>
       <c r="C6" t="str">
-        <v>6,400</v>
+        <v>6,450</v>
       </c>
       <c r="D6" t="str">
         <v>800 hours</v>
@@ -669,10 +669,10 @@
         <v>Total Cost</v>
       </c>
       <c r="B7" t="str">
-        <v>$1,380,000</v>
+        <v>$1,390,000</v>
       </c>
       <c r="C7" t="str">
-        <v>$1,205,000</v>
+        <v>$1,215,000</v>
       </c>
       <c r="D7" t="str">
         <v>$175,000</v>
@@ -883,7 +883,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H92"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1193,334 +1193,334 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>1</v>
+        <v>1a</v>
       </c>
       <c r="B14" t="str">
         <v>Foundation</v>
       </c>
       <c r="C14" t="str">
-        <v>Run EC/AEMcoder for initial migration</v>
+        <v>GitHub repository setup</v>
       </c>
       <c r="D14" t="str">
-        <v>Dev Team</v>
+        <v>Tech Lead</v>
       </c>
       <c r="E14">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="F14">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="G14" t="str">
-        <v>Initial blocks, markdown, page structure</v>
+        <v>Repo with branch protection, access controls</v>
       </c>
       <c r="H14" t="str">
-        <v>Accelerate migration by auto-generating block structure and content mapping from source site</v>
+        <v>Version control foundation; enables CI/CD, code review, and collaboration</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2</v>
+        <v>1b</v>
       </c>
       <c r="B15" t="str">
         <v>Foundation</v>
       </c>
       <c r="C15" t="str">
-        <v>Update blocks, functionality, CSS</v>
+        <v>AEM Cloud Service provisioning</v>
       </c>
       <c r="D15" t="str">
-        <v>Dev Team</v>
+        <v>DevOps</v>
       </c>
       <c r="E15">
-        <v>160</v>
+        <v>16</v>
       </c>
       <c r="F15">
-        <v>80</v>
+        <v>16</v>
       </c>
       <c r="G15" t="str">
-        <v>Production-ready block code</v>
+        <v>Dev, Stage, Prod environments</v>
       </c>
       <c r="H15" t="str">
-        <v>Refine auto-generated code to meet AT&amp;T brand standards and functional requirements</v>
+        <v>Required infrastructure for content authoring and Universal Editor</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2a</v>
+        <v>1c</v>
       </c>
       <c r="B16" t="str">
         <v>Foundation</v>
       </c>
       <c r="C16" t="str">
-        <v>Extract design system tokens</v>
+        <v>EDS site registration &amp; configuration</v>
       </c>
       <c r="D16" t="str">
-        <v>Dev Team</v>
+        <v>Tech Lead</v>
       </c>
       <c r="E16">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="F16">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="G16" t="str">
-        <v>styles.css, CSS custom properties</v>
+        <v>Registered site with aem.live</v>
       </c>
       <c r="H16" t="str">
-        <v>Ensure visual consistency with existing brand; enable global style changes from single source</v>
+        <v>Enables Edge Delivery Services; connects GitHub to EDS infrastructure</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2b</v>
+        <v>1d</v>
       </c>
       <c r="B17" t="str">
         <v>Foundation</v>
       </c>
       <c r="C17" t="str">
-        <v>Typography &amp; font setup</v>
+        <v>fstab.yaml &amp; site configuration</v>
       </c>
       <c r="D17" t="str">
         <v>Dev Team</v>
       </c>
       <c r="E17">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F17">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="G17" t="str">
-        <v>fonts.css, AT&amp;T brand fonts</v>
+        <v>Content source mapping, helix config</v>
       </c>
       <c r="H17" t="str">
-        <v>AT&amp;T brand compliance requires specific fonts (Aleck Sans/Slab); legal requirement</v>
+        <v>Maps AEM content to EDS; defines site behavior and routing</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2c</v>
+        <v>1e</v>
       </c>
       <c r="B18" t="str">
         <v>Foundation</v>
       </c>
       <c r="C18" t="str">
-        <v>Core navigation blocks</v>
+        <v>CI/CD pipeline setup</v>
       </c>
       <c r="D18" t="str">
-        <v>Dev Team</v>
+        <v>DevOps</v>
       </c>
       <c r="E18">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="F18">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="G18" t="str">
-        <v>header/, footer/, mega-menu</v>
+        <v>GitHub Actions for preview/publish</v>
       </c>
       <c r="H18" t="str">
-        <v>Navigation is on every page; must work perfectly for user experience and SEO</v>
+        <v>Automates deployment; enables continuous preview and publishing</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v/>
+        <v>1f</v>
       </c>
       <c r="B19" t="str">
-        <v/>
+        <v>Foundation</v>
       </c>
       <c r="C19" t="str">
-        <v>Phase 1 Subtotal</v>
+        <v>Run EC/AEMcoder for initial migration</v>
       </c>
       <c r="D19" t="str">
-        <v/>
+        <v>Dev Team</v>
       </c>
       <c r="E19">
-        <v>424</v>
+        <v>80</v>
       </c>
       <c r="F19">
-        <v>284</v>
+        <v>40</v>
       </c>
       <c r="G19" t="str">
-        <v/>
+        <v>Initial blocks, markdown, page structure</v>
       </c>
       <c r="H19" t="str">
-        <v/>
+        <v>Accelerate migration by auto-generating block structure and content mapping from source site</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v/>
+        <v>1g</v>
       </c>
       <c r="B20" t="str">
-        <v/>
+        <v>Foundation</v>
       </c>
       <c r="C20" t="str">
-        <v/>
+        <v>Update blocks, functionality, CSS</v>
       </c>
       <c r="D20" t="str">
-        <v/>
-      </c>
-      <c r="E20" t="str">
-        <v/>
-      </c>
-      <c r="F20" t="str">
-        <v/>
+        <v>Dev Team</v>
+      </c>
+      <c r="E20">
+        <v>160</v>
+      </c>
+      <c r="F20">
+        <v>80</v>
       </c>
       <c r="G20" t="str">
-        <v/>
+        <v>Production-ready block code</v>
       </c>
       <c r="H20" t="str">
-        <v/>
+        <v>Refine auto-generated code to meet AT&amp;T brand standards and functional requirements</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>PHASE 2: CONTENT MODELING (Weeks 7-8)</v>
+        <v>1h</v>
       </c>
       <c r="B21" t="str">
-        <v/>
+        <v>Foundation</v>
       </c>
       <c r="C21" t="str">
-        <v/>
+        <v>Extract design system tokens</v>
       </c>
       <c r="D21" t="str">
-        <v/>
-      </c>
-      <c r="E21" t="str">
-        <v/>
-      </c>
-      <c r="F21" t="str">
-        <v/>
+        <v>Dev Team</v>
+      </c>
+      <c r="E21">
+        <v>80</v>
+      </c>
+      <c r="F21">
+        <v>60</v>
       </c>
       <c r="G21" t="str">
-        <v/>
+        <v>styles.css, CSS custom properties</v>
       </c>
       <c r="H21" t="str">
-        <v/>
+        <v>Ensure visual consistency with existing brand; enable global style changes from single source</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>3</v>
+        <v>1i</v>
       </c>
       <c r="B22" t="str">
-        <v>Content Modeling</v>
+        <v>Foundation</v>
       </c>
       <c r="C22" t="str">
-        <v>Create component-model.json</v>
+        <v>Typography &amp; font setup</v>
       </c>
       <c r="D22" t="str">
-        <v>Tech Lead</v>
+        <v>Dev Team</v>
       </c>
       <c r="E22">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="F22">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="G22" t="str">
-        <v>JCR package structure for AEM importer</v>
+        <v>fonts.css, AT&amp;T brand fonts</v>
       </c>
       <c r="H22" t="str">
-        <v>Required for AEM importer to create proper JCR node structure; enables content import</v>
+        <v>AT&amp;T brand compliance requires specific fonts (Aleck Sans/Slab); legal requirement</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>3a</v>
+        <v>1j</v>
       </c>
       <c r="B23" t="str">
-        <v>Content Modeling</v>
+        <v>Foundation</v>
       </c>
       <c r="C23" t="str">
-        <v>Create component-definitions.json</v>
+        <v>Core navigation blocks</v>
       </c>
       <c r="D23" t="str">
-        <v>Tech Lead</v>
+        <v>Dev Team</v>
       </c>
       <c r="E23">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F23">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="G23" t="str">
-        <v>Universal Editor field definitions</v>
+        <v>header/, footer/, mega-menu</v>
       </c>
       <c r="H23" t="str">
-        <v>Defines authoring UI in Universal Editor; required for content authors to edit pages</v>
+        <v>Navigation is on every page; must work perfectly for user experience and SEO</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>3b</v>
+        <v/>
       </c>
       <c r="B24" t="str">
-        <v>Content Modeling</v>
+        <v/>
       </c>
       <c r="C24" t="str">
-        <v>Define content fragment models</v>
+        <v>Phase 1 Subtotal</v>
       </c>
       <c r="D24" t="str">
-        <v>Content Strategist</v>
+        <v/>
       </c>
       <c r="E24">
-        <v>40</v>
+        <v>474</v>
       </c>
       <c r="F24">
-        <v>36</v>
+        <v>334</v>
       </c>
       <c r="G24" t="str">
-        <v>CF models for products, stories</v>
+        <v/>
       </c>
       <c r="H24" t="str">
-        <v>Structure reusable content (products, testimonials) for consistency across 749 pages</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>3c</v>
+        <v/>
       </c>
       <c r="B25" t="str">
-        <v>Content Modeling</v>
+        <v/>
       </c>
       <c r="C25" t="str">
-        <v>Update transformations</v>
+        <v/>
       </c>
       <c r="D25" t="str">
-        <v>Dev Team</v>
-      </c>
-      <c r="E25">
-        <v>40</v>
-      </c>
-      <c r="F25">
-        <v>36</v>
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v/>
       </c>
       <c r="G25" t="str">
-        <v>Import script transformations</v>
+        <v/>
       </c>
       <c r="H25" t="str">
-        <v>Customize how source content maps to EDS blocks; handle edge cases in content structure</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v/>
+        <v>PHASE 2: CONTENT MODELING (Weeks 7-8)</v>
       </c>
       <c r="B26" t="str">
         <v/>
       </c>
       <c r="C26" t="str">
-        <v>Phase 2 Subtotal</v>
+        <v/>
       </c>
       <c r="D26" t="str">
         <v/>
       </c>
-      <c r="E26">
-        <v>200</v>
-      </c>
-      <c r="F26">
-        <v>180</v>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v/>
       </c>
       <c r="G26" t="str">
         <v/>
@@ -1531,412 +1531,412 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v/>
+        <v>2a</v>
       </c>
       <c r="B27" t="str">
-        <v/>
+        <v>Content Modeling</v>
       </c>
       <c r="C27" t="str">
-        <v/>
+        <v>Create component-model.json</v>
       </c>
       <c r="D27" t="str">
-        <v/>
-      </c>
-      <c r="E27" t="str">
-        <v/>
-      </c>
-      <c r="F27" t="str">
-        <v/>
+        <v>Tech Lead</v>
+      </c>
+      <c r="E27">
+        <v>60</v>
+      </c>
+      <c r="F27">
+        <v>54</v>
       </c>
       <c r="G27" t="str">
-        <v/>
+        <v>JCR package structure for AEM importer</v>
       </c>
       <c r="H27" t="str">
-        <v/>
+        <v>Required for AEM importer to create proper JCR node structure; enables content import</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>PHASE 3: BLOCK DEVELOPMENT (Weeks 9-14)</v>
+        <v>2b</v>
       </c>
       <c r="B28" t="str">
-        <v/>
+        <v>Content Modeling</v>
       </c>
       <c r="C28" t="str">
-        <v/>
+        <v>Create component-definitions.json</v>
       </c>
       <c r="D28" t="str">
-        <v/>
-      </c>
-      <c r="E28" t="str">
-        <v/>
-      </c>
-      <c r="F28" t="str">
-        <v/>
+        <v>Tech Lead</v>
+      </c>
+      <c r="E28">
+        <v>60</v>
+      </c>
+      <c r="F28">
+        <v>54</v>
       </c>
       <c r="G28" t="str">
-        <v/>
+        <v>Universal Editor field definitions</v>
       </c>
       <c r="H28" t="str">
-        <v/>
+        <v>Defines authoring UI in Universal Editor; required for content authors to edit pages</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>4a</v>
+        <v>2c</v>
       </c>
       <c r="B29" t="str">
-        <v>Block Development</v>
+        <v>Content Modeling</v>
       </c>
       <c r="C29" t="str">
-        <v>Hero blocks (6 variants)</v>
+        <v>Define content fragment models</v>
       </c>
       <c r="D29" t="str">
-        <v>Dev Team</v>
+        <v>Content Strategist</v>
       </c>
       <c r="E29">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="F29">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="G29" t="str">
-        <v>hero-video, hero-carousel, hero-split, etc.</v>
+        <v>CF models for products, stories</v>
       </c>
       <c r="H29" t="str">
-        <v>Hero sections are above-the-fold; critical for first impressions and conversion rates</v>
+        <v>Structure reusable content (products, testimonials) for consistency across 749 pages</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>4b</v>
+        <v>2d</v>
       </c>
       <c r="B30" t="str">
-        <v>Block Development</v>
+        <v>Content Modeling</v>
       </c>
       <c r="C30" t="str">
-        <v>Card blocks (10 variants)</v>
+        <v>Update transformations</v>
       </c>
       <c r="D30" t="str">
         <v>Dev Team</v>
       </c>
       <c r="E30">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="F30">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="G30" t="str">
-        <v>cards-product, cards-feature, cards-pricing, etc.</v>
+        <v>Import script transformations</v>
       </c>
       <c r="H30" t="str">
-        <v>Cards display products/features across site; most reused block type on 749 pages</v>
+        <v>Customize how source content maps to EDS blocks; handle edge cases in content structure</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>4c</v>
+        <v/>
       </c>
       <c r="B31" t="str">
-        <v>Block Development</v>
+        <v/>
       </c>
       <c r="C31" t="str">
-        <v>Interactive blocks</v>
+        <v>Phase 2 Subtotal</v>
       </c>
       <c r="D31" t="str">
-        <v>Dev Team</v>
+        <v/>
       </c>
       <c r="E31">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="F31">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="G31" t="str">
-        <v>tabs, accordion, carousel, modal, search</v>
+        <v/>
       </c>
       <c r="H31" t="str">
-        <v>Enable user engagement; required for FAQs, product details, filtering functionality</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>4d</v>
+        <v/>
       </c>
       <c r="B32" t="str">
-        <v>Block Development</v>
+        <v/>
       </c>
       <c r="C32" t="str">
-        <v>Form blocks</v>
+        <v/>
       </c>
       <c r="D32" t="str">
-        <v>Dev Team</v>
-      </c>
-      <c r="E32">
-        <v>120</v>
-      </c>
-      <c r="F32">
-        <v>72</v>
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <v/>
       </c>
       <c r="G32" t="str">
-        <v>lead-form, contact-form, newsletter</v>
+        <v/>
       </c>
       <c r="H32" t="str">
-        <v>Lead capture is business-critical; forms drive revenue and customer acquisition</v>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>4e</v>
+        <v>PHASE 3: BLOCK DEVELOPMENT (Weeks 9-14)</v>
       </c>
       <c r="B33" t="str">
-        <v>Block Development</v>
+        <v/>
       </c>
       <c r="C33" t="str">
-        <v>Content blocks</v>
+        <v/>
       </c>
       <c r="D33" t="str">
-        <v>Dev Team</v>
-      </c>
-      <c r="E33">
-        <v>160</v>
-      </c>
-      <c r="F33">
-        <v>80</v>
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v/>
       </c>
       <c r="G33" t="str">
-        <v>columns, quote, table, embed, download</v>
+        <v/>
       </c>
       <c r="H33" t="str">
-        <v>Support varied content layouts; enable rich content authoring flexibility</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>4f</v>
+        <v>3a</v>
       </c>
       <c r="B34" t="str">
         <v>Block Development</v>
       </c>
       <c r="C34" t="str">
-        <v>Product-specific blocks</v>
+        <v>Hero blocks (6 variants)</v>
       </c>
       <c r="D34" t="str">
         <v>Dev Team</v>
       </c>
       <c r="E34">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="F34">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="G34" t="str">
-        <v>pricing-table, comparison, spec-sheet</v>
+        <v>hero-video, hero-carousel, hero-split, etc.</v>
       </c>
       <c r="H34" t="str">
-        <v>AT&amp;T-specific functionality for product comparison and pricing display</v>
+        <v>Hero sections are above-the-fold; critical for first impressions and conversion rates</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v/>
+        <v>3b</v>
       </c>
       <c r="B35" t="str">
-        <v/>
+        <v>Block Development</v>
       </c>
       <c r="C35" t="str">
-        <v>Phase 3 Subtotal</v>
+        <v>Card blocks (10 variants)</v>
       </c>
       <c r="D35" t="str">
-        <v/>
+        <v>Dev Team</v>
       </c>
       <c r="E35">
-        <v>1080</v>
+        <v>200</v>
       </c>
       <c r="F35">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="G35" t="str">
-        <v/>
+        <v>cards-product, cards-feature, cards-pricing, etc.</v>
       </c>
       <c r="H35" t="str">
-        <v/>
+        <v>Cards display products/features across site; most reused block type on 749 pages</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v/>
+        <v>3c</v>
       </c>
       <c r="B36" t="str">
-        <v/>
+        <v>Block Development</v>
       </c>
       <c r="C36" t="str">
-        <v/>
+        <v>Interactive blocks</v>
       </c>
       <c r="D36" t="str">
-        <v/>
-      </c>
-      <c r="E36" t="str">
-        <v/>
-      </c>
-      <c r="F36" t="str">
-        <v/>
+        <v>Dev Team</v>
+      </c>
+      <c r="E36">
+        <v>280</v>
+      </c>
+      <c r="F36">
+        <v>168</v>
       </c>
       <c r="G36" t="str">
-        <v/>
+        <v>tabs, accordion, carousel, modal, search</v>
       </c>
       <c r="H36" t="str">
-        <v/>
+        <v>Enable user engagement; required for FAQs, product details, filtering functionality</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>PHASE 4: PAGE REVIEW &amp; ASSET MIGRATION (Weeks 15-20)</v>
+        <v>3d</v>
       </c>
       <c r="B37" t="str">
-        <v/>
+        <v>Block Development</v>
       </c>
       <c r="C37" t="str">
-        <v/>
+        <v>Form blocks</v>
       </c>
       <c r="D37" t="str">
-        <v/>
-      </c>
-      <c r="E37" t="str">
-        <v/>
-      </c>
-      <c r="F37" t="str">
-        <v/>
+        <v>Dev Team</v>
+      </c>
+      <c r="E37">
+        <v>120</v>
+      </c>
+      <c r="F37">
+        <v>72</v>
       </c>
       <c r="G37" t="str">
-        <v/>
+        <v>lead-form, contact-form, newsletter</v>
       </c>
       <c r="H37" t="str">
-        <v/>
+        <v>Lead capture is business-critical; forms drive revenue and customer acquisition</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>4</v>
+        <v>3e</v>
       </c>
       <c r="B38" t="str">
-        <v>Assets</v>
+        <v>Block Development</v>
       </c>
       <c r="C38" t="str">
-        <v>Review each page, re-author assets (749 pages)</v>
+        <v>Content blocks</v>
       </c>
       <c r="D38" t="str">
-        <v>Content Team</v>
+        <v>Dev Team</v>
       </c>
       <c r="E38">
-        <v>750</v>
+        <v>160</v>
       </c>
       <c r="F38">
-        <v>750</v>
+        <v>80</v>
       </c>
       <c r="G38" t="str">
-        <v>Validated content in AEM DAM</v>
+        <v>columns, quote, table, embed, download</v>
       </c>
       <c r="H38" t="str">
-        <v>Ensure content accuracy; fix migration errors; update outdated information</v>
+        <v>Support varied content layouts; enable rich content authoring flexibility</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>4a</v>
+        <v>3f</v>
       </c>
       <c r="B39" t="str">
-        <v>Assets</v>
+        <v>Block Development</v>
       </c>
       <c r="C39" t="str">
-        <v>Create URL redirect mapping (749 URLs)</v>
+        <v>Product-specific blocks</v>
       </c>
       <c r="D39" t="str">
-        <v>Content Strategist</v>
+        <v>Dev Team</v>
       </c>
       <c r="E39">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="F39">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="G39" t="str">
-        <v>301 redirect spreadsheet</v>
+        <v>pricing-table, comparison, spec-sheet</v>
       </c>
       <c r="H39" t="str">
-        <v>Preserve SEO rankings; prevent broken links; maintain user bookmarks (TBD if URLs change)</v>
+        <v>AT&amp;T-specific functionality for product comparison and pricing display</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>4b</v>
+        <v/>
       </c>
       <c r="B40" t="str">
-        <v>Assets</v>
+        <v/>
       </c>
       <c r="C40" t="str">
-        <v>DAM asset migration</v>
+        <v>Phase 3 Subtotal</v>
       </c>
       <c r="D40" t="str">
-        <v>Content Team</v>
+        <v/>
       </c>
       <c r="E40">
-        <v>300</v>
+        <v>1080</v>
       </c>
       <c r="F40">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="G40" t="str">
-        <v>Assets with metadata in AEM</v>
+        <v/>
       </c>
       <c r="H40" t="str">
-        <v>Images/PDFs must be in AEM DAM for authoring; metadata enables search and governance</v>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>4c</v>
+        <v/>
       </c>
       <c r="B41" t="str">
-        <v>Assets</v>
+        <v/>
       </c>
       <c r="C41" t="str">
-        <v>Image optimization</v>
+        <v/>
       </c>
       <c r="D41" t="str">
-        <v>Dev Team</v>
-      </c>
-      <c r="E41">
-        <v>150</v>
-      </c>
-      <c r="F41">
-        <v>150</v>
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
+        <v/>
       </c>
       <c r="G41" t="str">
-        <v>WebP conversion, lazy loading</v>
+        <v/>
       </c>
       <c r="H41" t="str">
-        <v>Performance requirement; Core Web Vitals depend on optimized images</v>
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v/>
+        <v>PHASE 4: PAGE REVIEW &amp; ASSET MIGRATION (Weeks 15-20)</v>
       </c>
       <c r="B42" t="str">
         <v/>
       </c>
       <c r="C42" t="str">
-        <v>Phase 4 Subtotal</v>
+        <v/>
       </c>
       <c r="D42" t="str">
         <v/>
       </c>
-      <c r="E42">
-        <v>1350</v>
-      </c>
-      <c r="F42">
-        <v>1350</v>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v/>
       </c>
       <c r="G42" t="str">
         <v/>
@@ -1947,178 +1947,178 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v/>
+        <v>4a</v>
       </c>
       <c r="B43" t="str">
-        <v/>
+        <v>Assets</v>
       </c>
       <c r="C43" t="str">
-        <v/>
+        <v>Review each page, re-author assets (749 pages)</v>
       </c>
       <c r="D43" t="str">
-        <v/>
-      </c>
-      <c r="E43" t="str">
-        <v/>
-      </c>
-      <c r="F43" t="str">
-        <v/>
+        <v>Content Team</v>
+      </c>
+      <c r="E43">
+        <v>750</v>
+      </c>
+      <c r="F43">
+        <v>750</v>
       </c>
       <c r="G43" t="str">
-        <v/>
+        <v>Validated content in AEM DAM</v>
       </c>
       <c r="H43" t="str">
-        <v/>
+        <v>Ensure content accuracy; fix migration errors; update outdated information</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>PHASE 5: EDGE WORKERS &amp; APIs (Weeks 21-22)</v>
+        <v>4b</v>
       </c>
       <c r="B44" t="str">
-        <v/>
+        <v>Assets</v>
       </c>
       <c r="C44" t="str">
-        <v/>
+        <v>Create URL redirect mapping (749 URLs)</v>
       </c>
       <c r="D44" t="str">
-        <v/>
-      </c>
-      <c r="E44" t="str">
-        <v/>
-      </c>
-      <c r="F44" t="str">
-        <v/>
+        <v>Content Strategist</v>
+      </c>
+      <c r="E44">
+        <v>150</v>
+      </c>
+      <c r="F44">
+        <v>150</v>
       </c>
       <c r="G44" t="str">
-        <v/>
+        <v>301 redirect spreadsheet</v>
       </c>
       <c r="H44" t="str">
-        <v/>
+        <v>Preserve SEO rankings; prevent broken links; maintain user bookmarks (TBD if URLs change)</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>5</v>
+        <v>4c</v>
       </c>
       <c r="B45" t="str">
-        <v>Edge Workers</v>
+        <v>Assets</v>
       </c>
       <c r="C45" t="str">
-        <v>Move servlets/APIs to Edge workers</v>
+        <v>DAM asset migration</v>
       </c>
       <c r="D45" t="str">
-        <v>Dev Team</v>
+        <v>Content Team</v>
       </c>
       <c r="E45">
-        <v>160</v>
+        <v>300</v>
       </c>
       <c r="F45">
-        <v>160</v>
+        <v>300</v>
       </c>
       <c r="G45" t="str">
-        <v>Edge worker functions</v>
+        <v>Assets with metadata in AEM</v>
       </c>
       <c r="H45" t="str">
-        <v>EDS is static; dynamic functionality (forms, search, pricing) requires edge workers</v>
+        <v>Images/PDFs must be in AEM DAM for authoring; metadata enables search and governance</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>5a</v>
+        <v>4d</v>
       </c>
       <c r="B46" t="str">
-        <v>Edge Workers</v>
+        <v>Assets</v>
       </c>
       <c r="C46" t="str">
-        <v>Pricing API integration</v>
+        <v>Image optimization</v>
       </c>
       <c r="D46" t="str">
         <v>Dev Team</v>
       </c>
       <c r="E46">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="F46">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="G46" t="str">
-        <v>Dynamic pricing endpoints</v>
+        <v>WebP conversion, lazy loading</v>
       </c>
       <c r="H46" t="str">
-        <v>Business requirement; pricing must be real-time and accurate for customer trust</v>
+        <v>Performance requirement; Core Web Vitals depend on optimized images</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>5b</v>
+        <v/>
       </c>
       <c r="B47" t="str">
-        <v>Edge Workers</v>
+        <v/>
       </c>
       <c r="C47" t="str">
-        <v>Lead form submission handling</v>
+        <v>Phase 4 Subtotal</v>
       </c>
       <c r="D47" t="str">
-        <v>Dev Team</v>
+        <v/>
       </c>
       <c r="E47">
-        <v>40</v>
+        <v>1350</v>
       </c>
       <c r="F47">
-        <v>40</v>
+        <v>1350</v>
       </c>
       <c r="G47" t="str">
-        <v>Form backend integration</v>
+        <v/>
       </c>
       <c r="H47" t="str">
-        <v>Revenue-critical; form submissions must reach CRM/sales systems reliably</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>5c</v>
+        <v/>
       </c>
       <c r="B48" t="str">
-        <v>Edge Workers</v>
+        <v/>
       </c>
       <c r="C48" t="str">
-        <v>Search functionality</v>
+        <v/>
       </c>
       <c r="D48" t="str">
-        <v>Dev Team</v>
-      </c>
-      <c r="E48">
-        <v>80</v>
-      </c>
-      <c r="F48">
-        <v>80</v>
+        <v/>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v/>
       </c>
       <c r="G48" t="str">
-        <v>Site search implementation</v>
+        <v/>
       </c>
       <c r="H48" t="str">
-        <v>User experience requirement; customers expect to search across 749 pages</v>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v/>
+        <v>PHASE 5: EDGE WORKERS &amp; APIs (Weeks 21-22)</v>
       </c>
       <c r="B49" t="str">
         <v/>
       </c>
       <c r="C49" t="str">
-        <v>Phase 5 Subtotal</v>
+        <v/>
       </c>
       <c r="D49" t="str">
         <v/>
       </c>
-      <c r="E49">
-        <v>340</v>
-      </c>
-      <c r="F49">
-        <v>340</v>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v/>
       </c>
       <c r="G49" t="str">
         <v/>
@@ -2129,94 +2129,94 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v/>
+        <v>5a</v>
       </c>
       <c r="B50" t="str">
-        <v/>
+        <v>Edge Workers</v>
       </c>
       <c r="C50" t="str">
-        <v/>
+        <v>Move servlets/APIs to Edge workers</v>
       </c>
       <c r="D50" t="str">
-        <v/>
-      </c>
-      <c r="E50" t="str">
-        <v/>
-      </c>
-      <c r="F50" t="str">
-        <v/>
+        <v>Dev Team</v>
+      </c>
+      <c r="E50">
+        <v>160</v>
+      </c>
+      <c r="F50">
+        <v>160</v>
       </c>
       <c r="G50" t="str">
-        <v/>
+        <v>Edge worker functions</v>
       </c>
       <c r="H50" t="str">
-        <v/>
+        <v>EDS is static; dynamic functionality (forms, search, pricing) requires edge workers</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>PHASE 6: AEM MIGRATION (Weeks 23-24)</v>
+        <v>5b</v>
       </c>
       <c r="B51" t="str">
-        <v/>
+        <v>Edge Workers</v>
       </c>
       <c r="C51" t="str">
-        <v/>
+        <v>Pricing API integration</v>
       </c>
       <c r="D51" t="str">
-        <v/>
-      </c>
-      <c r="E51" t="str">
-        <v/>
-      </c>
-      <c r="F51" t="str">
-        <v/>
+        <v>Dev Team</v>
+      </c>
+      <c r="E51">
+        <v>60</v>
+      </c>
+      <c r="F51">
+        <v>60</v>
       </c>
       <c r="G51" t="str">
-        <v/>
+        <v>Dynamic pricing endpoints</v>
       </c>
       <c r="H51" t="str">
-        <v/>
+        <v>Business requirement; pricing must be real-time and accurate for customer trust</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>6</v>
+        <v>5c</v>
       </c>
       <c r="B52" t="str">
-        <v>AEM Migration</v>
+        <v>Edge Workers</v>
       </c>
       <c r="C52" t="str">
-        <v>Migrate custom functionality to AEMaaCS</v>
+        <v>Lead form submission handling</v>
       </c>
       <c r="D52" t="str">
         <v>Dev Team</v>
       </c>
       <c r="E52">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="F52">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="G52" t="str">
-        <v>Reports, scheduled jobs</v>
+        <v>Form backend integration</v>
       </c>
       <c r="H52" t="str">
-        <v>Preserve existing business logic; scheduled reports and jobs must continue working</v>
+        <v>Revenue-critical; form submissions must reach CRM/sales systems reliably</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>7</v>
+        <v>5d</v>
       </c>
       <c r="B53" t="str">
-        <v>AEM Migration</v>
+        <v>Edge Workers</v>
       </c>
       <c r="C53" t="str">
-        <v>Migrate meta-schema, taxonomy, workflows</v>
+        <v>Search functionality</v>
       </c>
       <c r="D53" t="str">
-        <v>Tech Lead</v>
+        <v>Dev Team</v>
       </c>
       <c r="E53">
         <v>80</v>
@@ -2225,82 +2225,82 @@
         <v>80</v>
       </c>
       <c r="G53" t="str">
-        <v>AEM configurations</v>
+        <v>Site search implementation</v>
       </c>
       <c r="H53" t="str">
-        <v>Content governance requires proper taxonomy; workflows enable approval processes</v>
+        <v>User experience requirement; customers expect to search across 749 pages</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>7a</v>
+        <v/>
       </c>
       <c r="B54" t="str">
-        <v>AEM Migration</v>
+        <v/>
       </c>
       <c r="C54" t="str">
-        <v>User/group migration</v>
+        <v>Phase 5 Subtotal</v>
       </c>
       <c r="D54" t="str">
-        <v>Admin</v>
+        <v/>
       </c>
       <c r="E54">
-        <v>40</v>
+        <v>340</v>
       </c>
       <c r="F54">
-        <v>40</v>
+        <v>340</v>
       </c>
       <c r="G54" t="str">
-        <v>Permissions in AEMaaCS</v>
+        <v/>
       </c>
       <c r="H54" t="str">
-        <v>Security requirement; preserve access controls and content permissions</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>7b</v>
+        <v/>
       </c>
       <c r="B55" t="str">
-        <v>AEM Migration</v>
+        <v/>
       </c>
       <c r="C55" t="str">
-        <v>Workflow configuration</v>
+        <v/>
       </c>
       <c r="D55" t="str">
-        <v>Tech Lead</v>
-      </c>
-      <c r="E55">
-        <v>40</v>
-      </c>
-      <c r="F55">
-        <v>40</v>
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
+        <v/>
       </c>
       <c r="G55" t="str">
-        <v>Approval workflows</v>
+        <v/>
       </c>
       <c r="H55" t="str">
-        <v>Business process requirement; content must go through approval before publishing</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v/>
+        <v>PHASE 6: AEM MIGRATION (Weeks 23-24)</v>
       </c>
       <c r="B56" t="str">
         <v/>
       </c>
       <c r="C56" t="str">
-        <v>Phase 6 Subtotal</v>
+        <v/>
       </c>
       <c r="D56" t="str">
         <v/>
       </c>
-      <c r="E56">
-        <v>280</v>
-      </c>
-      <c r="F56">
-        <v>280</v>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
+        <v/>
       </c>
       <c r="G56" t="str">
         <v/>
@@ -2311,94 +2311,94 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v/>
+        <v>6a</v>
       </c>
       <c r="B57" t="str">
-        <v/>
+        <v>AEM Migration</v>
       </c>
       <c r="C57" t="str">
-        <v/>
+        <v>Migrate custom functionality to AEMaaCS</v>
       </c>
       <c r="D57" t="str">
-        <v/>
-      </c>
-      <c r="E57" t="str">
-        <v/>
-      </c>
-      <c r="F57" t="str">
-        <v/>
+        <v>Dev Team</v>
+      </c>
+      <c r="E57">
+        <v>120</v>
+      </c>
+      <c r="F57">
+        <v>120</v>
       </c>
       <c r="G57" t="str">
-        <v/>
+        <v>Reports, scheduled jobs</v>
       </c>
       <c r="H57" t="str">
-        <v/>
+        <v>Preserve existing business logic; scheduled reports and jobs must continue working</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>PHASE 7: INTEGRATIONS (Weeks 25-26)</v>
+        <v>6b</v>
       </c>
       <c r="B58" t="str">
-        <v/>
+        <v>AEM Migration</v>
       </c>
       <c r="C58" t="str">
-        <v/>
+        <v>Migrate meta-schema, taxonomy, workflows</v>
       </c>
       <c r="D58" t="str">
-        <v/>
-      </c>
-      <c r="E58" t="str">
-        <v/>
-      </c>
-      <c r="F58" t="str">
-        <v/>
+        <v>Tech Lead</v>
+      </c>
+      <c r="E58">
+        <v>80</v>
+      </c>
+      <c r="F58">
+        <v>80</v>
       </c>
       <c r="G58" t="str">
-        <v/>
+        <v>AEM configurations</v>
       </c>
       <c r="H58" t="str">
-        <v/>
+        <v>Content governance requires proper taxonomy; workflows enable approval processes</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>8a</v>
+        <v>6c</v>
       </c>
       <c r="B59" t="str">
-        <v>Integrations</v>
+        <v>AEM Migration</v>
       </c>
       <c r="C59" t="str">
-        <v>Analytics/tracking setup</v>
+        <v>User/group migration</v>
       </c>
       <c r="D59" t="str">
-        <v>Dev Team</v>
+        <v>Admin</v>
       </c>
       <c r="E59">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F59">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="G59" t="str">
-        <v>Adobe Launch configuration</v>
+        <v>Permissions in AEMaaCS</v>
       </c>
       <c r="H59" t="str">
-        <v>Business intelligence requirement; track conversions, user behavior, ROI</v>
+        <v>Security requirement; preserve access controls and content permissions</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>8b</v>
+        <v>6d</v>
       </c>
       <c r="B60" t="str">
-        <v>Integrations</v>
+        <v>AEM Migration</v>
       </c>
       <c r="C60" t="str">
-        <v>Third-party scripts</v>
+        <v>Workflow configuration</v>
       </c>
       <c r="D60" t="str">
-        <v>Dev Team</v>
+        <v>Tech Lead</v>
       </c>
       <c r="E60">
         <v>40</v>
@@ -2407,82 +2407,82 @@
         <v>40</v>
       </c>
       <c r="G60" t="str">
-        <v>Chat, pixels, consent banner</v>
+        <v>Approval workflows</v>
       </c>
       <c r="H60" t="str">
-        <v>Customer support (chat), marketing (pixels), legal compliance (consent)</v>
+        <v>Business process requirement; content must go through approval before publishing</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>8c</v>
+        <v/>
       </c>
       <c r="B61" t="str">
-        <v>Integrations</v>
+        <v/>
       </c>
       <c r="C61" t="str">
-        <v>Search indexing configuration</v>
+        <v>Phase 6 Subtotal</v>
       </c>
       <c r="D61" t="str">
-        <v>Dev Team</v>
+        <v/>
       </c>
       <c r="E61">
-        <v>40</v>
+        <v>280</v>
       </c>
       <c r="F61">
-        <v>40</v>
+        <v>280</v>
       </c>
       <c r="G61" t="str">
-        <v>Sitemap, robots.txt</v>
+        <v/>
       </c>
       <c r="H61" t="str">
-        <v>SEO requirement; search engines must be able to crawl and index all 749 pages</v>
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>8d</v>
+        <v/>
       </c>
       <c r="B62" t="str">
-        <v>Integrations</v>
+        <v/>
       </c>
       <c r="C62" t="str">
-        <v>Social meta tags</v>
+        <v/>
       </c>
       <c r="D62" t="str">
-        <v>Dev Team</v>
-      </c>
-      <c r="E62">
-        <v>20</v>
-      </c>
-      <c r="F62">
-        <v>20</v>
+        <v/>
+      </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
+      <c r="F62" t="str">
+        <v/>
       </c>
       <c r="G62" t="str">
-        <v>OG tags, Twitter cards</v>
+        <v/>
       </c>
       <c r="H62" t="str">
-        <v>Social sharing requirement; proper previews when pages are shared on social media</v>
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v/>
+        <v>PHASE 7: INTEGRATIONS (Weeks 25-26)</v>
       </c>
       <c r="B63" t="str">
         <v/>
       </c>
       <c r="C63" t="str">
-        <v>Phase 7 Subtotal</v>
+        <v/>
       </c>
       <c r="D63" t="str">
         <v/>
       </c>
-      <c r="E63">
-        <v>160</v>
-      </c>
-      <c r="F63">
-        <v>160</v>
+      <c r="E63" t="str">
+        <v/>
+      </c>
+      <c r="F63" t="str">
+        <v/>
       </c>
       <c r="G63" t="str">
         <v/>
@@ -2493,302 +2493,302 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v/>
+        <v>7a</v>
       </c>
       <c r="B64" t="str">
-        <v/>
+        <v>Integrations</v>
       </c>
       <c r="C64" t="str">
-        <v/>
+        <v>Analytics/tracking setup</v>
       </c>
       <c r="D64" t="str">
-        <v/>
-      </c>
-      <c r="E64" t="str">
-        <v/>
-      </c>
-      <c r="F64" t="str">
-        <v/>
+        <v>Dev Team</v>
+      </c>
+      <c r="E64">
+        <v>60</v>
+      </c>
+      <c r="F64">
+        <v>60</v>
       </c>
       <c r="G64" t="str">
-        <v/>
+        <v>Adobe Launch configuration</v>
       </c>
       <c r="H64" t="str">
-        <v/>
+        <v>Business intelligence requirement; track conversions, user behavior, ROI</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>PHASE 8: VALIDATION &amp; TESTING (Weeks 27-28)</v>
+        <v>7b</v>
       </c>
       <c r="B65" t="str">
-        <v/>
+        <v>Integrations</v>
       </c>
       <c r="C65" t="str">
-        <v/>
+        <v>Third-party scripts</v>
       </c>
       <c r="D65" t="str">
-        <v/>
-      </c>
-      <c r="E65" t="str">
-        <v/>
-      </c>
-      <c r="F65" t="str">
-        <v/>
+        <v>Dev Team</v>
+      </c>
+      <c r="E65">
+        <v>40</v>
+      </c>
+      <c r="F65">
+        <v>40</v>
       </c>
       <c r="G65" t="str">
-        <v/>
+        <v>Chat, pixels, consent banner</v>
       </c>
       <c r="H65" t="str">
-        <v/>
+        <v>Customer support (chat), marketing (pixels), legal compliance (consent)</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>8</v>
+        <v>7c</v>
       </c>
       <c r="B66" t="str">
-        <v>Validation</v>
+        <v>Integrations</v>
       </c>
       <c r="C66" t="str">
-        <v>Validate all functionalities (749 pages)</v>
+        <v>Search indexing configuration</v>
       </c>
       <c r="D66" t="str">
-        <v>QA Team</v>
+        <v>Dev Team</v>
       </c>
       <c r="E66">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="F66">
-        <v>280</v>
+        <v>40</v>
       </c>
       <c r="G66" t="str">
-        <v>Functional test reports</v>
+        <v>Sitemap, robots.txt</v>
       </c>
       <c r="H66" t="str">
-        <v>Ensure nothing is broken; verify all interactive elements work correctly</v>
+        <v>SEO requirement; search engines must be able to crawl and index all 749 pages</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>9</v>
+        <v>7d</v>
       </c>
       <c r="B67" t="str">
-        <v>Validation</v>
+        <v>Integrations</v>
       </c>
       <c r="C67" t="str">
-        <v>Accessibility audit (WCAG 2.1 AA)</v>
+        <v>Social meta tags</v>
       </c>
       <c r="D67" t="str">
-        <v>QA Team</v>
+        <v>Dev Team</v>
       </c>
       <c r="E67">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="F67">
-        <v>110</v>
+        <v>20</v>
       </c>
       <c r="G67" t="str">
-        <v>Accessibility report, fixes</v>
+        <v>OG tags, Twitter cards</v>
       </c>
       <c r="H67" t="str">
-        <v>Legal requirement; ADA compliance mandatory for enterprise sites</v>
+        <v>Social sharing requirement; proper previews when pages are shared on social media</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>10</v>
+        <v/>
       </c>
       <c r="B68" t="str">
-        <v>Validation</v>
+        <v/>
       </c>
       <c r="C68" t="str">
-        <v>Performance/load testing</v>
+        <v>Phase 7 Subtotal</v>
       </c>
       <c r="D68" t="str">
-        <v>QA Team</v>
+        <v/>
       </c>
       <c r="E68">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="F68">
-        <v>75</v>
+        <v>160</v>
       </c>
       <c r="G68" t="str">
-        <v>Performance test results</v>
+        <v/>
       </c>
       <c r="H68" t="str">
-        <v>Verify Core Web Vitals targets met; ensure site handles expected traffic</v>
+        <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>11</v>
+        <v/>
       </c>
       <c r="B69" t="str">
-        <v>Validation</v>
+        <v/>
       </c>
       <c r="C69" t="str">
-        <v>SEO validation (749 redirects)</v>
+        <v/>
       </c>
       <c r="D69" t="str">
-        <v>SEO Specialist</v>
-      </c>
-      <c r="E69">
-        <v>80</v>
-      </c>
-      <c r="F69">
-        <v>80</v>
+        <v/>
+      </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
+      <c r="F69" t="str">
+        <v/>
       </c>
       <c r="G69" t="str">
-        <v>Redirect testing, sitemap validation</v>
+        <v/>
       </c>
       <c r="H69" t="str">
-        <v>Verify no SEO ranking loss; confirm all redirects work correctly</v>
+        <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>12</v>
+        <v>PHASE 8: VALIDATION &amp; TESTING (Weeks 27-28)</v>
       </c>
       <c r="B70" t="str">
-        <v>Validation</v>
+        <v/>
       </c>
       <c r="C70" t="str">
-        <v>Security review</v>
+        <v/>
       </c>
       <c r="D70" t="str">
-        <v>Security Team</v>
-      </c>
-      <c r="E70">
-        <v>40</v>
-      </c>
-      <c r="F70">
-        <v>40</v>
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
+      <c r="F70" t="str">
+        <v/>
       </c>
       <c r="G70" t="str">
-        <v>Security headers, CSP audit</v>
+        <v/>
       </c>
       <c r="H70" t="str">
-        <v>Security requirement; protect against XSS, clickjacking, data breaches</v>
+        <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v/>
+        <v>8a</v>
       </c>
       <c r="B71" t="str">
-        <v/>
+        <v>Validation</v>
       </c>
       <c r="C71" t="str">
-        <v>Phase 8 Subtotal</v>
+        <v>Validate all functionalities (749 pages)</v>
       </c>
       <c r="D71" t="str">
-        <v/>
+        <v>QA Team</v>
       </c>
       <c r="E71">
-        <v>620</v>
+        <v>300</v>
       </c>
       <c r="F71">
-        <v>585</v>
+        <v>280</v>
       </c>
       <c r="G71" t="str">
-        <v/>
+        <v>Functional test reports</v>
       </c>
       <c r="H71" t="str">
-        <v/>
+        <v>Ensure nothing is broken; verify all interactive elements work correctly</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v/>
+        <v>8b</v>
       </c>
       <c r="B72" t="str">
-        <v/>
+        <v>Validation</v>
       </c>
       <c r="C72" t="str">
-        <v/>
+        <v>Accessibility audit (WCAG 2.1 AA)</v>
       </c>
       <c r="D72" t="str">
-        <v/>
-      </c>
-      <c r="E72" t="str">
-        <v/>
-      </c>
-      <c r="F72" t="str">
-        <v/>
+        <v>QA Team</v>
+      </c>
+      <c r="E72">
+        <v>120</v>
+      </c>
+      <c r="F72">
+        <v>110</v>
       </c>
       <c r="G72" t="str">
-        <v/>
+        <v>Accessibility report, fixes</v>
       </c>
       <c r="H72" t="str">
-        <v/>
+        <v>Legal requirement; ADA compliance mandatory for enterprise sites</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>PHASE 9: LAUNCH (Weeks 29-30)</v>
+        <v>8c</v>
       </c>
       <c r="B73" t="str">
-        <v/>
+        <v>Validation</v>
       </c>
       <c r="C73" t="str">
-        <v/>
+        <v>Performance/load testing</v>
       </c>
       <c r="D73" t="str">
-        <v/>
-      </c>
-      <c r="E73" t="str">
-        <v/>
-      </c>
-      <c r="F73" t="str">
-        <v/>
+        <v>QA Team</v>
+      </c>
+      <c r="E73">
+        <v>80</v>
+      </c>
+      <c r="F73">
+        <v>75</v>
       </c>
       <c r="G73" t="str">
-        <v/>
+        <v>Performance test results</v>
       </c>
       <c r="H73" t="str">
-        <v/>
+        <v>Verify Core Web Vitals targets met; ensure site handles expected traffic</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>13</v>
+        <v>8d</v>
       </c>
       <c r="B74" t="str">
-        <v>Launch</v>
+        <v>Validation</v>
       </c>
       <c r="C74" t="str">
-        <v>UAT &amp; stakeholder sign-off</v>
+        <v>SEO validation (749 redirects)</v>
       </c>
       <c r="D74" t="str">
-        <v>PM</v>
+        <v>SEO Specialist</v>
       </c>
       <c r="E74">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F74">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="G74" t="str">
-        <v>Sign-off documentation</v>
+        <v>Redirect testing, sitemap validation</v>
       </c>
       <c r="H74" t="str">
-        <v>Business approval required before go-live; stakeholders verify requirements met</v>
+        <v>Verify no SEO ranking loss; confirm all redirects work correctly</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>14</v>
+        <v>8e</v>
       </c>
       <c r="B75" t="str">
-        <v>Launch</v>
+        <v>Validation</v>
       </c>
       <c r="C75" t="str">
-        <v>DNS cutover &amp; rollback plan</v>
+        <v>Security review</v>
       </c>
       <c r="D75" t="str">
-        <v>Tech Lead</v>
+        <v>Security Team</v>
       </c>
       <c r="E75">
         <v>40</v>
@@ -2797,82 +2797,82 @@
         <v>40</v>
       </c>
       <c r="G75" t="str">
-        <v>Production deployment</v>
+        <v>Security headers, CSP audit</v>
       </c>
       <c r="H75" t="str">
-        <v>Safe deployment; rollback plan ensures quick recovery if issues arise</v>
+        <v>Security requirement; protect against XSS, clickjacking, data breaches</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>15</v>
+        <v/>
       </c>
       <c r="B76" t="str">
-        <v>Launch</v>
+        <v/>
       </c>
       <c r="C76" t="str">
-        <v>Author training on Universal Editor</v>
+        <v>Phase 8 Subtotal</v>
       </c>
       <c r="D76" t="str">
-        <v>Training Lead</v>
+        <v/>
       </c>
       <c r="E76">
-        <v>80</v>
+        <v>620</v>
       </c>
       <c r="F76">
-        <v>80</v>
+        <v>585</v>
       </c>
       <c r="G76" t="str">
-        <v>Training materials, sessions</v>
+        <v/>
       </c>
       <c r="H76" t="str">
-        <v>Enable content team to maintain site post-launch; reduce support burden</v>
+        <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>16</v>
+        <v/>
       </c>
       <c r="B77" t="str">
-        <v>Launch</v>
+        <v/>
       </c>
       <c r="C77" t="str">
-        <v>Hypercare &amp; monitoring setup</v>
+        <v/>
       </c>
       <c r="D77" t="str">
-        <v>DevOps</v>
-      </c>
-      <c r="E77">
-        <v>100</v>
-      </c>
-      <c r="F77">
-        <v>100</v>
+        <v/>
+      </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
+      <c r="F77" t="str">
+        <v/>
       </c>
       <c r="G77" t="str">
-        <v>Monitoring dashboards, alerts</v>
+        <v/>
       </c>
       <c r="H77" t="str">
-        <v>Catch issues quickly post-launch; ensure 99.9% uptime SLA is met</v>
+        <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v/>
+        <v>PHASE 9: LAUNCH (Weeks 29-30)</v>
       </c>
       <c r="B78" t="str">
         <v/>
       </c>
       <c r="C78" t="str">
-        <v>Phase 9 Subtotal</v>
+        <v/>
       </c>
       <c r="D78" t="str">
         <v/>
       </c>
-      <c r="E78">
-        <v>320</v>
-      </c>
-      <c r="F78">
-        <v>315</v>
+      <c r="E78" t="str">
+        <v/>
+      </c>
+      <c r="F78" t="str">
+        <v/>
       </c>
       <c r="G78" t="str">
         <v/>
@@ -2883,132 +2883,132 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v/>
+        <v>9a</v>
       </c>
       <c r="B79" t="str">
-        <v/>
+        <v>Launch</v>
       </c>
       <c r="C79" t="str">
-        <v/>
+        <v>Domain/DNS configuration</v>
       </c>
       <c r="D79" t="str">
-        <v/>
-      </c>
-      <c r="E79" t="str">
-        <v/>
-      </c>
-      <c r="F79" t="str">
-        <v/>
+        <v>DevOps</v>
+      </c>
+      <c r="E79">
+        <v>16</v>
+      </c>
+      <c r="F79">
+        <v>16</v>
       </c>
       <c r="G79" t="str">
-        <v/>
+        <v>Custom domain, SSL certificates</v>
       </c>
       <c r="H79" t="str">
-        <v/>
+        <v>Production readiness; secure HTTPS required for customer trust and SEO</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v/>
+        <v>9b</v>
       </c>
       <c r="B80" t="str">
-        <v/>
+        <v>Launch</v>
       </c>
       <c r="C80" t="str">
-        <v/>
+        <v>UAT &amp; stakeholder sign-off</v>
       </c>
       <c r="D80" t="str">
-        <v/>
-      </c>
-      <c r="E80" t="str">
-        <v/>
-      </c>
-      <c r="F80" t="str">
-        <v/>
+        <v>PM</v>
+      </c>
+      <c r="E80">
+        <v>100</v>
+      </c>
+      <c r="F80">
+        <v>95</v>
       </c>
       <c r="G80" t="str">
-        <v/>
+        <v>Sign-off documentation</v>
       </c>
       <c r="H80" t="str">
-        <v/>
+        <v>Business approval required before go-live; stakeholders verify requirements met</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>SUMMARY (749 PAGES)</v>
+        <v>9c</v>
       </c>
       <c r="B81" t="str">
-        <v/>
+        <v>Launch</v>
       </c>
       <c r="C81" t="str">
-        <v/>
+        <v>DNS cutover &amp; rollback plan</v>
       </c>
       <c r="D81" t="str">
-        <v/>
-      </c>
-      <c r="E81" t="str">
-        <v/>
-      </c>
-      <c r="F81" t="str">
-        <v/>
+        <v>Tech Lead</v>
+      </c>
+      <c r="E81">
+        <v>40</v>
+      </c>
+      <c r="F81">
+        <v>40</v>
       </c>
       <c r="G81" t="str">
-        <v/>
+        <v>Production deployment</v>
       </c>
       <c r="H81" t="str">
-        <v/>
+        <v>Safe deployment; rollback plan ensures quick recovery if issues arise</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v/>
+        <v>9d</v>
       </c>
       <c r="B82" t="str">
-        <v/>
+        <v>Launch</v>
       </c>
       <c r="C82" t="str">
-        <v>Base Hours Total</v>
+        <v>Author training on Universal Editor</v>
       </c>
       <c r="D82" t="str">
-        <v/>
+        <v>Training Lead</v>
       </c>
       <c r="E82">
-        <v>4942</v>
+        <v>80</v>
       </c>
       <c r="F82">
-        <v>4262</v>
+        <v>80</v>
       </c>
       <c r="G82" t="str">
-        <v/>
+        <v>Training materials, sessions</v>
       </c>
       <c r="H82" t="str">
-        <v/>
+        <v>Enable content team to maintain site post-launch; reduce support burden</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v/>
+        <v>9e</v>
       </c>
       <c r="B83" t="str">
-        <v/>
+        <v>Launch</v>
       </c>
       <c r="C83" t="str">
-        <v>Contingency (~46% / ~50%)</v>
+        <v>Hypercare &amp; monitoring setup</v>
       </c>
       <c r="D83" t="str">
-        <v/>
+        <v>DevOps</v>
       </c>
       <c r="E83">
-        <v>2258</v>
+        <v>100</v>
       </c>
       <c r="F83">
-        <v>2138</v>
+        <v>100</v>
       </c>
       <c r="G83" t="str">
-        <v/>
+        <v>Monitoring dashboards, alerts</v>
       </c>
       <c r="H83" t="str">
-        <v>Buffer for unknowns, scope changes, and discovered complexity</v>
+        <v>Catch issues quickly post-launch; ensure 99.9% uptime SLA is met</v>
       </c>
     </row>
     <row r="84">
@@ -3019,16 +3019,16 @@
         <v/>
       </c>
       <c r="C84" t="str">
-        <v>GRAND TOTAL</v>
+        <v>Phase 9 Subtotal</v>
       </c>
       <c r="D84" t="str">
         <v/>
       </c>
       <c r="E84">
-        <v>7200</v>
+        <v>336</v>
       </c>
       <c r="F84">
-        <v>6400</v>
+        <v>331</v>
       </c>
       <c r="G84" t="str">
         <v/>
@@ -3045,7 +3045,7 @@
         <v/>
       </c>
       <c r="C85" t="str">
-        <v>Hours Saved with EC/AEMCoder</v>
+        <v/>
       </c>
       <c r="D85" t="str">
         <v/>
@@ -3053,14 +3053,14 @@
       <c r="E85" t="str">
         <v/>
       </c>
-      <c r="F85">
-        <v>800</v>
+      <c r="F85" t="str">
+        <v/>
       </c>
       <c r="G85" t="str">
         <v/>
       </c>
       <c r="H85" t="str">
-        <v>~11% reduction in effort</v>
+        <v/>
       </c>
     </row>
     <row r="86">
@@ -3071,27 +3071,183 @@
         <v/>
       </c>
       <c r="C86" t="str">
+        <v/>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
+      <c r="F86" t="str">
+        <v/>
+      </c>
+      <c r="G86" t="str">
+        <v/>
+      </c>
+      <c r="H86" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>SUMMARY (749 PAGES)</v>
+      </c>
+      <c r="B87" t="str">
+        <v/>
+      </c>
+      <c r="C87" t="str">
+        <v/>
+      </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
+      <c r="F87" t="str">
+        <v/>
+      </c>
+      <c r="G87" t="str">
+        <v/>
+      </c>
+      <c r="H87" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v/>
+      </c>
+      <c r="B88" t="str">
+        <v/>
+      </c>
+      <c r="C88" t="str">
+        <v>Base Hours Total</v>
+      </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
+      <c r="E88">
+        <v>5008</v>
+      </c>
+      <c r="F88">
+        <v>4328</v>
+      </c>
+      <c r="G88" t="str">
+        <v/>
+      </c>
+      <c r="H88" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v/>
+      </c>
+      <c r="B89" t="str">
+        <v/>
+      </c>
+      <c r="C89" t="str">
+        <v>Contingency (~45% / ~49%)</v>
+      </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
+      <c r="E89">
+        <v>2242</v>
+      </c>
+      <c r="F89">
+        <v>2122</v>
+      </c>
+      <c r="G89" t="str">
+        <v/>
+      </c>
+      <c r="H89" t="str">
+        <v>Buffer for unknowns, scope changes, and discovered complexity</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v/>
+      </c>
+      <c r="B90" t="str">
+        <v/>
+      </c>
+      <c r="C90" t="str">
+        <v>GRAND TOTAL</v>
+      </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
+      <c r="E90">
+        <v>7250</v>
+      </c>
+      <c r="F90">
+        <v>6450</v>
+      </c>
+      <c r="G90" t="str">
+        <v/>
+      </c>
+      <c r="H90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v/>
+      </c>
+      <c r="B91" t="str">
+        <v/>
+      </c>
+      <c r="C91" t="str">
+        <v>Hours Saved with EC/AEMCoder</v>
+      </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
+      <c r="F91">
+        <v>800</v>
+      </c>
+      <c r="G91" t="str">
+        <v/>
+      </c>
+      <c r="H91" t="str">
+        <v>~11% reduction in effort</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v/>
+      </c>
+      <c r="B92" t="str">
+        <v/>
+      </c>
+      <c r="C92" t="str">
         <v>Weeks Saved</v>
       </c>
-      <c r="D86" t="str">
-        <v/>
-      </c>
-      <c r="E86" t="str">
-        <v/>
-      </c>
-      <c r="F86" t="str">
+      <c r="D92" t="str">
+        <v/>
+      </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
+      <c r="F92" t="str">
         <v>4-6 weeks</v>
       </c>
-      <c r="G86" t="str">
-        <v/>
-      </c>
-      <c r="H86" t="str">
+      <c r="G92" t="str">
+        <v/>
+      </c>
+      <c r="H92" t="str">
         <v>Faster time to market</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H86"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H92"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3361,16 +3517,16 @@
         <v>3-6</v>
       </c>
       <c r="C5" t="str">
-        <v>424</v>
+        <v>474</v>
       </c>
       <c r="D5" t="str">
-        <v>284</v>
+        <v>334</v>
       </c>
       <c r="E5" t="str">
         <v>140</v>
       </c>
       <c r="F5" t="str">
-        <v>EC/AEMcoder migration, block updates, design system</v>
+        <v>Env setup, EDS config, EC/AEMcoder, blocks, design system</v>
       </c>
     </row>
     <row r="6">
@@ -3521,16 +3677,16 @@
         <v>29-30</v>
       </c>
       <c r="C13" t="str">
-        <v>320</v>
+        <v>336</v>
       </c>
       <c r="D13" t="str">
-        <v>315</v>
+        <v>331</v>
       </c>
       <c r="E13" t="str">
         <v>5</v>
       </c>
       <c r="F13" t="str">
-        <v>UAT, DNS cutover, training, hypercare</v>
+        <v>Domain/DNS, UAT, cutover, training, hypercare</v>
       </c>
     </row>
     <row r="14">
@@ -3541,16 +3697,16 @@
         <v>-</v>
       </c>
       <c r="C14" t="str">
-        <v>2,258</v>
+        <v>2,242</v>
       </c>
       <c r="D14" t="str">
-        <v>2,138</v>
+        <v>2,122</v>
       </c>
       <c r="E14" t="str">
         <v>120</v>
       </c>
       <c r="F14" t="str">
-        <v>Risk buffer (~46%)</v>
+        <v>Risk buffer (~45%)</v>
       </c>
     </row>
     <row r="15">
@@ -3561,10 +3717,10 @@
         <v>28-30 / 24-26</v>
       </c>
       <c r="C15" t="str">
-        <v>7,200</v>
+        <v>7,250</v>
       </c>
       <c r="D15" t="str">
-        <v>6,400</v>
+        <v>6,450</v>
       </c>
       <c r="E15" t="str">
         <v>800</v>
@@ -5371,7 +5527,7 @@
         <v>80</v>
       </c>
       <c r="E5">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="F5">
         <v>100</v>
@@ -5386,10 +5542,10 @@
         <v>100</v>
       </c>
       <c r="J5">
-        <v>640</v>
+        <v>660</v>
       </c>
       <c r="K5" t="str">
-        <v>$128,000</v>
+        <v>$132,000</v>
       </c>
     </row>
     <row r="6">
@@ -5406,7 +5562,7 @@
         <v>0</v>
       </c>
       <c r="E6">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="F6">
         <v>40</v>
@@ -5421,10 +5577,10 @@
         <v>100</v>
       </c>
       <c r="J6">
-        <v>860</v>
+        <v>870</v>
       </c>
       <c r="K6" t="str">
-        <v>$159,100</v>
+        <v>$160,950</v>
       </c>
     </row>
     <row r="7">
@@ -5441,7 +5597,7 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="F7">
         <v>40</v>
@@ -5456,10 +5612,10 @@
         <v>100</v>
       </c>
       <c r="J7">
-        <v>800</v>
+        <v>810</v>
       </c>
       <c r="K7" t="str">
-        <v>$148,000</v>
+        <v>$149,850</v>
       </c>
     </row>
     <row r="8">
@@ -5476,7 +5632,7 @@
         <v>0</v>
       </c>
       <c r="E8">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -5491,10 +5647,10 @@
         <v>100</v>
       </c>
       <c r="J8">
-        <v>600</v>
+        <v>610</v>
       </c>
       <c r="K8" t="str">
-        <v>$99,000</v>
+        <v>$100,650</v>
       </c>
     </row>
     <row r="9">
@@ -5511,7 +5667,7 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -5526,10 +5682,10 @@
         <v>80</v>
       </c>
       <c r="J9">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="K9" t="str">
-        <v>$75,900</v>
+        <v>$77,550</v>
       </c>
     </row>
     <row r="10">
@@ -5546,7 +5702,7 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -5561,10 +5717,10 @@
         <v>80</v>
       </c>
       <c r="J10">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="K10" t="str">
-        <v>$42,560</v>
+        <v>$43,400</v>
       </c>
     </row>
     <row r="11">
@@ -5791,7 +5947,7 @@
         <v>0</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -5803,13 +5959,13 @@
         <v>80</v>
       </c>
       <c r="I17">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="J17">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="K17" t="str">
-        <v>$28,800</v>
+        <v>$36,800</v>
       </c>
     </row>
     <row r="18">
@@ -5826,7 +5982,7 @@
         <v>210</v>
       </c>
       <c r="E18">
-        <v>504</v>
+        <v>604</v>
       </c>
       <c r="F18">
         <v>280</v>
@@ -5838,13 +5994,13 @@
         <v>2780</v>
       </c>
       <c r="I18">
-        <v>1500</v>
+        <v>1516</v>
       </c>
       <c r="J18">
-        <v>6534</v>
+        <v>6650</v>
       </c>
       <c r="K18" t="str">
-        <v>$998,660</v>
+        <v>$1,018,500</v>
       </c>
     </row>
   </sheetData>
@@ -5858,7 +6014,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D30"/>
   <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
@@ -5909,16 +6065,16 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Phase 1: Foundation</v>
+        <v>Phase 1: Foundation (incl. env setup)</v>
       </c>
       <c r="B6">
-        <v>424</v>
+        <v>474</v>
       </c>
       <c r="C6" t="str">
-        <v>$72,000</v>
+        <v>$80,000</v>
       </c>
       <c r="D6" t="str">
-        <v>6%</v>
+        <v>7%</v>
       </c>
     </row>
     <row r="7">
@@ -5968,10 +6124,10 @@
         <v>Phase 7-9: Validation/Launch</v>
       </c>
       <c r="B10">
-        <v>1100</v>
+        <v>1116</v>
       </c>
       <c r="C10" t="str">
-        <v>$175,000</v>
+        <v>$180,000</v>
       </c>
       <c r="D10" t="str">
         <v>15%</v>
@@ -5982,13 +6138,13 @@
         <v>Contingency</v>
       </c>
       <c r="B11">
-        <v>2258</v>
+        <v>2242</v>
       </c>
       <c r="C11" t="str">
-        <v>$363,000</v>
+        <v>$364,000</v>
       </c>
       <c r="D11" t="str">
-        <v>31%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="12">
@@ -5996,10 +6152,10 @@
         <v>TOTAL</v>
       </c>
       <c r="B12">
-        <v>7200</v>
+        <v>7250</v>
       </c>
       <c r="C12" t="str">
-        <v>$1,176,000</v>
+        <v>$1,190,000</v>
       </c>
       <c r="D12" t="str">
         <v>100%</v>
@@ -6159,10 +6315,10 @@
         <v/>
       </c>
       <c r="C26" t="str">
-        <v>$1,176,000</v>
+        <v>$1,190,000</v>
       </c>
       <c r="D26" t="str">
-        <v>$1,020,000</v>
+        <v>$1,030,000</v>
       </c>
     </row>
     <row r="27">
@@ -6187,7 +6343,7 @@
         <v/>
       </c>
       <c r="C28" t="str">
-        <v>$164,400</v>
+        <v>$160,400</v>
       </c>
       <c r="D28" t="str">
         <v>$145,000</v>
@@ -6201,10 +6357,10 @@
         <v/>
       </c>
       <c r="C29" t="str">
-        <v>$1,380,000</v>
+        <v>$1,390,000</v>
       </c>
       <c r="D29" t="str">
-        <v>$1,205,000</v>
+        <v>$1,215,000</v>
       </c>
     </row>
     <row r="30">
@@ -6230,7 +6386,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <cols>
     <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6402,9 +6558,23 @@
         <v>Automated testing, sampling strategy</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>AEM Cloud Service provisioning delays</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="C14" t="str">
+        <v>High</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Request environments early in Phase 1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>